<commit_message>
BPF: NSP Database lane shows table names only (no Log, read / write detail)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QL8Do8Pd2rXEDNa1ifG2RK
</commit_message>
<xml_diff>
--- a/deliverables/function_list_v2/bpf/Crossdock_BPF_Level2.xlsx
+++ b/deliverables/function_list_v2/bpf/Crossdock_BPF_Level2.xlsx
@@ -761,7 +761,7 @@
       <xdr:col>9</xdr:col>
       <xdr:colOff>57150</xdr:colOff>
       <xdr:row>17</xdr:row>
-      <xdr:rowOff>260349</xdr:rowOff>
+      <xdr:rowOff>260350</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -771,7 +771,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="4391025" y="2646363"/>
-          <a:ext cx="2276475" cy="2605087"/>
+          <a:ext cx="2276475" cy="2617788"/>
         </a:xfrm>
         <a:custGeom>
           <a:avLst/>
@@ -780,12 +780,12 @@
           <a:cxnLst/>
           <a:rect l="0" t="0" r="r" b="b"/>
           <a:pathLst>
-            <a:path w="2276475" h="2605087" fill="none">
+            <a:path w="2276475" h="2617788" fill="none">
               <a:moveTo>
-                <a:pt x="0" y="2605087"/>
+                <a:pt x="0" y="2617788"/>
               </a:moveTo>
               <a:lnTo>
-                <a:pt x="209550" y="2605087"/>
+                <a:pt x="209550" y="2617788"/>
               </a:lnTo>
               <a:lnTo>
                 <a:pt x="209550" y="0"/>
@@ -989,7 +989,7 @@
       <xdr:col>13</xdr:col>
       <xdr:colOff>57150</xdr:colOff>
       <xdr:row>17</xdr:row>
-      <xdr:rowOff>212724</xdr:rowOff>
+      <xdr:rowOff>212725</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -999,7 +999,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="8201025" y="3048000"/>
-          <a:ext cx="2276475" cy="2155825"/>
+          <a:ext cx="2276475" cy="2168525"/>
         </a:xfrm>
         <a:custGeom>
           <a:avLst/>
@@ -1008,7 +1008,7 @@
           <a:cxnLst/>
           <a:rect l="0" t="0" r="r" b="b"/>
           <a:pathLst>
-            <a:path w="2276475" h="2155825" fill="none">
+            <a:path w="2276475" h="2168525" fill="none">
               <a:moveTo>
                 <a:pt x="0" y="0"/>
               </a:moveTo>
@@ -1016,16 +1016,16 @@
                 <a:pt x="161925" y="0"/>
               </a:lnTo>
               <a:lnTo>
-                <a:pt x="161925" y="1824038"/>
+                <a:pt x="161925" y="1836738"/>
               </a:lnTo>
               <a:lnTo>
-                <a:pt x="2066925" y="1824038"/>
+                <a:pt x="2066925" y="1836738"/>
               </a:lnTo>
               <a:lnTo>
-                <a:pt x="2066925" y="2155825"/>
+                <a:pt x="2066925" y="2168525"/>
               </a:lnTo>
               <a:lnTo>
-                <a:pt x="2276475" y="2155825"/>
+                <a:pt x="2276475" y="2168525"/>
               </a:lnTo>
             </a:path>
           </a:pathLst>
@@ -1052,7 +1052,7 @@
       <xdr:col>15</xdr:col>
       <xdr:colOff>57150</xdr:colOff>
       <xdr:row>20</xdr:row>
-      <xdr:rowOff>330199</xdr:rowOff>
+      <xdr:rowOff>330200</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -1062,7 +1062,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="10106025" y="3048000"/>
-          <a:ext cx="2276475" cy="3098800"/>
+          <a:ext cx="2276475" cy="3111500"/>
         </a:xfrm>
         <a:custGeom>
           <a:avLst/>
@@ -1071,7 +1071,7 @@
           <a:cxnLst/>
           <a:rect l="0" t="0" r="r" b="b"/>
           <a:pathLst>
-            <a:path w="2276475" h="3098800" fill="none">
+            <a:path w="2276475" h="3111500" fill="none">
               <a:moveTo>
                 <a:pt x="0" y="0"/>
               </a:moveTo>
@@ -1079,16 +1079,16 @@
                 <a:pt x="185738" y="0"/>
               </a:lnTo>
               <a:lnTo>
-                <a:pt x="185738" y="2673350"/>
+                <a:pt x="185738" y="2686050"/>
               </a:lnTo>
               <a:lnTo>
-                <a:pt x="2090738" y="2673350"/>
+                <a:pt x="2090738" y="2686050"/>
               </a:lnTo>
               <a:lnTo>
-                <a:pt x="2090738" y="3098800"/>
+                <a:pt x="2090738" y="3111500"/>
               </a:lnTo>
               <a:lnTo>
-                <a:pt x="2276475" y="3098800"/>
+                <a:pt x="2276475" y="3111500"/>
               </a:lnTo>
             </a:path>
           </a:pathLst>
@@ -1109,13 +1109,13 @@
       <xdr:col>15</xdr:col>
       <xdr:colOff>1590675</xdr:colOff>
       <xdr:row>20</xdr:row>
-      <xdr:rowOff>330199</xdr:rowOff>
+      <xdr:rowOff>330200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
       <xdr:colOff>57150</xdr:colOff>
       <xdr:row>20</xdr:row>
-      <xdr:rowOff>377824</xdr:rowOff>
+      <xdr:rowOff>377825</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -1124,7 +1124,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13916025" y="6146800"/>
+          <a:off x="13916025" y="6159500"/>
           <a:ext cx="371475" cy="47625"/>
         </a:xfrm>
         <a:custGeom>
@@ -1172,7 +1172,7 @@
       <xdr:col>19</xdr:col>
       <xdr:colOff>57150</xdr:colOff>
       <xdr:row>20</xdr:row>
-      <xdr:rowOff>330199</xdr:rowOff>
+      <xdr:rowOff>330200</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -1182,7 +1182,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="15821025" y="3000375"/>
-          <a:ext cx="371475" cy="3146425"/>
+          <a:ext cx="371475" cy="3159125"/>
         </a:xfrm>
         <a:custGeom>
           <a:avLst/>
@@ -1191,12 +1191,12 @@
           <a:cxnLst/>
           <a:rect l="0" t="0" r="r" b="b"/>
           <a:pathLst>
-            <a:path w="371475" h="3146425" fill="none">
+            <a:path w="371475" h="3159125" fill="none">
               <a:moveTo>
-                <a:pt x="0" y="3146425"/>
+                <a:pt x="0" y="3159125"/>
               </a:moveTo>
               <a:lnTo>
-                <a:pt x="161925" y="3146425"/>
+                <a:pt x="161925" y="3159125"/>
               </a:lnTo>
               <a:lnTo>
                 <a:pt x="161925" y="0"/>
@@ -1286,7 +1286,7 @@
       <xdr:col>21</xdr:col>
       <xdr:colOff>57150</xdr:colOff>
       <xdr:row>23</xdr:row>
-      <xdr:rowOff>517524</xdr:rowOff>
+      <xdr:rowOff>517525</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -1296,7 +1296,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="17726025" y="3048000"/>
-          <a:ext cx="371475" cy="4251325"/>
+          <a:ext cx="371475" cy="4264025"/>
         </a:xfrm>
         <a:custGeom>
           <a:avLst/>
@@ -1305,7 +1305,7 @@
           <a:cxnLst/>
           <a:rect l="0" t="0" r="r" b="b"/>
           <a:pathLst>
-            <a:path w="371475" h="4251325" fill="none">
+            <a:path w="371475" h="4264025" fill="none">
               <a:moveTo>
                 <a:pt x="0" y="0"/>
               </a:moveTo>
@@ -1313,10 +1313,10 @@
                 <a:pt x="209550" y="0"/>
               </a:lnTo>
               <a:lnTo>
-                <a:pt x="209550" y="4251325"/>
+                <a:pt x="209550" y="4264025"/>
               </a:lnTo>
               <a:lnTo>
-                <a:pt x="371475" y="4251325"/>
+                <a:pt x="371475" y="4264025"/>
               </a:lnTo>
             </a:path>
           </a:pathLst>
@@ -1378,7 +1378,6 @@
             <a:srgbClr val="2E75B6"/>
           </a:solidFill>
           <a:prstDash val="dash"/>
-          <a:headEnd type="triangle" w="sm" len="sm"/>
           <a:tailEnd type="triangle" w="sm" len="sm"/>
         </a:ln>
       </xdr:spPr>
@@ -1390,7 +1389,7 @@
       <xdr:col>5</xdr:col>
       <xdr:colOff>1130617</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>984249</xdr:rowOff>
+      <xdr:rowOff>996950</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
@@ -1405,7 +1404,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3930968" y="4667250"/>
+          <a:off x="3930968" y="4679950"/>
           <a:ext cx="9525" cy="352425"/>
         </a:xfrm>
         <a:custGeom>
@@ -1431,7 +1430,6 @@
             <a:srgbClr val="2E75B6"/>
           </a:solidFill>
           <a:prstDash val="dash"/>
-          <a:headEnd type="triangle" w="sm" len="sm"/>
           <a:tailEnd type="triangle" w="sm" len="sm"/>
         </a:ln>
       </xdr:spPr>
@@ -1484,7 +1482,6 @@
             <a:srgbClr val="2E75B6"/>
           </a:solidFill>
           <a:prstDash val="dash"/>
-          <a:headEnd type="triangle" w="sm" len="sm"/>
           <a:tailEnd type="triangle" w="sm" len="sm"/>
         </a:ln>
       </xdr:spPr>
@@ -1537,7 +1534,6 @@
             <a:srgbClr val="2E75B6"/>
           </a:solidFill>
           <a:prstDash val="dash"/>
-          <a:headEnd type="triangle" w="sm" len="sm"/>
           <a:tailEnd type="triangle" w="sm" len="sm"/>
         </a:ln>
       </xdr:spPr>
@@ -1590,7 +1586,6 @@
             <a:srgbClr val="2E75B6"/>
           </a:solidFill>
           <a:prstDash val="dash"/>
-          <a:headEnd type="triangle" w="sm" len="sm"/>
           <a:tailEnd type="triangle" w="sm" len="sm"/>
         </a:ln>
       </xdr:spPr>
@@ -1602,7 +1597,7 @@
       <xdr:col>13</xdr:col>
       <xdr:colOff>1130617</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>984249</xdr:rowOff>
+      <xdr:rowOff>996950</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>13</xdr:col>
@@ -1617,7 +1612,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="11550968" y="4667250"/>
+          <a:off x="11550968" y="4679950"/>
           <a:ext cx="9525" cy="352425"/>
         </a:xfrm>
         <a:custGeom>
@@ -1643,7 +1638,7 @@
             <a:srgbClr val="2E75B6"/>
           </a:solidFill>
           <a:prstDash val="dash"/>
-          <a:headEnd type="triangle" w="sm" len="sm"/>
+          <a:tailEnd type="triangle" w="sm" len="sm"/>
         </a:ln>
       </xdr:spPr>
     </xdr:sp>
@@ -1654,7 +1649,7 @@
       <xdr:col>15</xdr:col>
       <xdr:colOff>1130617</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>984249</xdr:rowOff>
+      <xdr:rowOff>996950</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>15</xdr:col>
@@ -1669,7 +1664,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13455968" y="4667250"/>
+          <a:off x="13455968" y="4679950"/>
           <a:ext cx="9525" cy="1177925"/>
         </a:xfrm>
         <a:custGeom>
@@ -1695,7 +1690,6 @@
             <a:srgbClr val="2E75B6"/>
           </a:solidFill>
           <a:prstDash val="dash"/>
-          <a:headEnd type="triangle" w="sm" len="sm"/>
           <a:tailEnd type="triangle" w="sm" len="sm"/>
         </a:ln>
       </xdr:spPr>
@@ -1707,7 +1701,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>1130617</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>984249</xdr:rowOff>
+      <xdr:rowOff>996950</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
@@ -1722,7 +1716,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="15360968" y="4667250"/>
+          <a:off x="15360968" y="4679950"/>
           <a:ext cx="9525" cy="1177925"/>
         </a:xfrm>
         <a:custGeom>
@@ -1748,7 +1742,7 @@
             <a:srgbClr val="2E75B6"/>
           </a:solidFill>
           <a:prstDash val="dash"/>
-          <a:headEnd type="triangle" w="sm" len="sm"/>
+          <a:tailEnd type="triangle" w="sm" len="sm"/>
         </a:ln>
       </xdr:spPr>
     </xdr:sp>
@@ -1800,7 +1794,6 @@
             <a:srgbClr val="2E75B6"/>
           </a:solidFill>
           <a:prstDash val="dash"/>
-          <a:headEnd type="triangle" w="sm" len="sm"/>
           <a:tailEnd type="triangle" w="sm" len="sm"/>
         </a:ln>
       </xdr:spPr>
@@ -2221,7 +2214,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2857500" y="5019675"/>
+          <a:off x="2857500" y="5032375"/>
           <a:ext cx="1533525" cy="463550"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2291,7 +2284,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm rot="10800000">
-          <a:off x="4286250" y="5019675"/>
+          <a:off x="4286250" y="5032375"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="rtTriangle">
@@ -2327,7 +2320,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2828925" y="4953000"/>
+          <a:off x="2828925" y="4965700"/>
           <a:ext cx="247650" cy="114300"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2384,7 +2377,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4086225" y="4953000"/>
+          <a:off x="4086225" y="4965700"/>
           <a:ext cx="295275" cy="114300"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3324,7 +3317,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="10477500" y="5019675"/>
+          <a:off x="10477500" y="5032375"/>
           <a:ext cx="1533525" cy="463550"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3394,7 +3387,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm rot="10800000">
-          <a:off x="11906250" y="5019675"/>
+          <a:off x="11906250" y="5032375"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="rtTriangle">
@@ -3430,7 +3423,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="10448925" y="4953000"/>
+          <a:off x="10448925" y="4965700"/>
           <a:ext cx="247650" cy="114300"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3487,7 +3480,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="11706225" y="4953000"/>
+          <a:off x="11706225" y="4965700"/>
           <a:ext cx="295275" cy="114300"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3542,7 +3535,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="12382500" y="5845175"/>
+          <a:off x="12382500" y="5857875"/>
           <a:ext cx="1533525" cy="603250"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3612,7 +3605,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm rot="10800000">
-          <a:off x="13811250" y="5845175"/>
+          <a:off x="13811250" y="5857875"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="rtTriangle">
@@ -3648,7 +3641,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="12353925" y="5778500"/>
+          <a:off x="12353925" y="5791200"/>
           <a:ext cx="247650" cy="114300"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3705,7 +3698,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13611225" y="5778500"/>
+          <a:off x="13611225" y="5791200"/>
           <a:ext cx="295275" cy="114300"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3760,7 +3753,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14287500" y="5845175"/>
+          <a:off x="14287500" y="5857875"/>
           <a:ext cx="1533525" cy="603250"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3830,7 +3823,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm rot="10800000">
-          <a:off x="15716250" y="5845175"/>
+          <a:off x="15716250" y="5857875"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="rtTriangle">
@@ -3866,7 +3859,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14258925" y="5778500"/>
+          <a:off x="14258925" y="5791200"/>
           <a:ext cx="247650" cy="114300"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4330,7 +4323,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="18097500" y="6810375"/>
+          <a:off x="18097500" y="6823075"/>
           <a:ext cx="1533525" cy="882650"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4426,7 +4419,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm rot="10800000">
-          <a:off x="19526250" y="6810375"/>
+          <a:off x="19526250" y="6823075"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="rtTriangle">
@@ -4462,7 +4455,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="18068925" y="6743700"/>
+          <a:off x="18068925" y="6756400"/>
           <a:ext cx="247650" cy="114300"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4510,7 +4503,7 @@
       <xdr:col>3</xdr:col>
       <xdr:colOff>1609725</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>984249</xdr:rowOff>
+      <xdr:rowOff>996950</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -4520,7 +4513,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="933450" y="3702050"/>
-          <a:ext cx="1571625" cy="965200"/>
+          <a:ext cx="1571625" cy="977900"/>
         </a:xfrm>
         <a:prstGeom prst="can">
           <a:avLst/>
@@ -4540,42 +4533,16 @@
         </a:bodyPr>
         <a:lstStyle/>
         <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="7B3F00"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>W: TB_M_H0125_DESTINATION (NSP)</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="7B3F00"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>W: Log</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
               <a:solidFill>
                 <a:srgbClr val="1F3864"/>
               </a:solidFill>
               <a:latin typeface="Arial"/>
               <a:cs typeface="Arial"/>
             </a:rPr>
-            <a:t>R: TB_M_H0125_DESTINATION (DB Surrounding)</a:t>
+            <a:t>TB_M_H0125_DESTINATION</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -4593,7 +4560,7 @@
       <xdr:col>5</xdr:col>
       <xdr:colOff>1609725</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>984249</xdr:rowOff>
+      <xdr:rowOff>996950</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -4603,7 +4570,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="2838450" y="3702050"/>
-          <a:ext cx="1571625" cy="965200"/>
+          <a:ext cx="1571625" cy="977900"/>
         </a:xfrm>
         <a:prstGeom prst="can">
           <a:avLst/>
@@ -4623,42 +4590,29 @@
         </a:bodyPr>
         <a:lstStyle/>
         <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="7B3F00"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>W: TB_M_PART_CANDIDATE</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="7B3F00"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>W: TB_H_PART_CANDIDATE</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="7B3F00"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>W: Log</a:t>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
+              <a:solidFill>
+                <a:srgbClr val="1F3864"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:rPr>
+            <a:t>TB_M_PART_CANDIDATE</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
+              <a:solidFill>
+                <a:srgbClr val="1F3864"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:rPr>
+            <a:t>TB_H_PART_CANDIDATE</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -4676,7 +4630,7 @@
       <xdr:col>7</xdr:col>
       <xdr:colOff>1609725</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>984249</xdr:rowOff>
+      <xdr:rowOff>996950</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -4686,7 +4640,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="4743450" y="3702050"/>
-          <a:ext cx="1571625" cy="965200"/>
+          <a:ext cx="1571625" cy="977900"/>
         </a:xfrm>
         <a:prstGeom prst="can">
           <a:avLst/>
@@ -4706,42 +4660,16 @@
         </a:bodyPr>
         <a:lstStyle/>
         <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="7B3F00"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>W: TB_R_ACTUAL_DEMAND_SUMMARY (NSP)</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="7B3F00"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>W: Log</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
               <a:solidFill>
                 <a:srgbClr val="1F3864"/>
               </a:solidFill>
               <a:latin typeface="Arial"/>
               <a:cs typeface="Arial"/>
             </a:rPr>
-            <a:t>R: TB_R_ACTUAL_DEMAND_SUMMARY (DB Surrounding)</a:t>
+            <a:t>TB_R_ACTUAL_DEMAND_SUMMARY</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -4759,7 +4687,7 @@
       <xdr:col>9</xdr:col>
       <xdr:colOff>1609725</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>984249</xdr:rowOff>
+      <xdr:rowOff>996950</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -4769,7 +4697,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="6648450" y="3702050"/>
-          <a:ext cx="1571625" cy="965200"/>
+          <a:ext cx="1571625" cy="977900"/>
         </a:xfrm>
         <a:prstGeom prst="can">
           <a:avLst/>
@@ -4789,68 +4717,55 @@
         </a:bodyPr>
         <a:lstStyle/>
         <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="7B3F00"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>W: TB_R_PART_DAD_RESULT</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="7B3F00"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>W: TB_M_PART_CANDIDATE</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="7B3F00"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>W: TB_H_PART_CANDIDATE</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="7B3F00"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>W: Log</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
               <a:solidFill>
                 <a:srgbClr val="1F3864"/>
               </a:solidFill>
               <a:latin typeface="Arial"/>
               <a:cs typeface="Arial"/>
             </a:rPr>
-            <a:t>R: TB_R_ACTUAL_DEMAND_SUMMARY</a:t>
+            <a:t>TB_R_PART_DAD_RESULT</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
+              <a:solidFill>
+                <a:srgbClr val="1F3864"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:rPr>
+            <a:t>TB_M_PART_CANDIDATE</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
+              <a:solidFill>
+                <a:srgbClr val="1F3864"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:rPr>
+            <a:t>TB_H_PART_CANDIDATE</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
+              <a:solidFill>
+                <a:srgbClr val="1F3864"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:rPr>
+            <a:t>TB_R_ACTUAL_DEMAND_SUMMARY</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -4868,7 +4783,7 @@
       <xdr:col>11</xdr:col>
       <xdr:colOff>1609725</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>984249</xdr:rowOff>
+      <xdr:rowOff>996950</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -4878,7 +4793,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="8553450" y="3702050"/>
-          <a:ext cx="1571625" cy="965200"/>
+          <a:ext cx="1571625" cy="977900"/>
         </a:xfrm>
         <a:prstGeom prst="can">
           <a:avLst/>
@@ -4898,81 +4813,68 @@
         </a:bodyPr>
         <a:lstStyle/>
         <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="7B3F00"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>W: TB_M_PART_CANDIDATE_DEST</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="7B3F00"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>W: TB_H_PART_CANDIDATE</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="7B3F00"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>W: Log</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
               <a:solidFill>
                 <a:srgbClr val="1F3864"/>
               </a:solidFill>
               <a:latin typeface="Arial"/>
               <a:cs typeface="Arial"/>
             </a:rPr>
-            <a:t>R: TB_R_ACTUAL_DEMAND_SUMMARY</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
+            <a:t>TB_M_PART_CANDIDATE_DEST</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
               <a:solidFill>
                 <a:srgbClr val="1F3864"/>
               </a:solidFill>
               <a:latin typeface="Arial"/>
               <a:cs typeface="Arial"/>
             </a:rPr>
-            <a:t>R: TB_M_PART_CANDIDATE</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
+            <a:t>TB_H_PART_CANDIDATE</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
               <a:solidFill>
                 <a:srgbClr val="1F3864"/>
               </a:solidFill>
               <a:latin typeface="Arial"/>
               <a:cs typeface="Arial"/>
             </a:rPr>
-            <a:t>R: TB_M_H0125_DESTINATION</a:t>
+            <a:t>TB_R_ACTUAL_DEMAND_SUMMARY</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
+              <a:solidFill>
+                <a:srgbClr val="1F3864"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:rPr>
+            <a:t>TB_M_PART_CANDIDATE</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
+              <a:solidFill>
+                <a:srgbClr val="1F3864"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:rPr>
+            <a:t>TB_M_H0125_DESTINATION</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -4990,7 +4892,7 @@
       <xdr:col>13</xdr:col>
       <xdr:colOff>1609725</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>984249</xdr:rowOff>
+      <xdr:rowOff>996950</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -5000,7 +4902,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="10458450" y="3702050"/>
-          <a:ext cx="1571625" cy="965200"/>
+          <a:ext cx="1571625" cy="977900"/>
         </a:xfrm>
         <a:prstGeom prst="can">
           <a:avLst/>
@@ -5020,29 +4922,16 @@
         </a:bodyPr>
         <a:lstStyle/>
         <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
               <a:solidFill>
                 <a:srgbClr val="1F3864"/>
               </a:solidFill>
               <a:latin typeface="Arial"/>
               <a:cs typeface="Arial"/>
             </a:rPr>
-            <a:t>R: TB_M_PART_CANDIDATE</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="1F3864"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>R: Log</a:t>
+            <a:t>TB_M_PART_CANDIDATE</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -5060,7 +4949,7 @@
       <xdr:col>15</xdr:col>
       <xdr:colOff>1609725</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>984249</xdr:rowOff>
+      <xdr:rowOff>996950</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -5070,7 +4959,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="12363450" y="3702050"/>
-          <a:ext cx="1571625" cy="965200"/>
+          <a:ext cx="1571625" cy="977900"/>
         </a:xfrm>
         <a:prstGeom prst="can">
           <a:avLst/>
@@ -5090,55 +4979,55 @@
         </a:bodyPr>
         <a:lstStyle/>
         <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="7B3F00"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>W: TB_M_PART_CANDIDATE_DEST</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="7B3F00"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>W: TB_M_PART_CANDIDATE (SYNC_STATUS No Sync)</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="7B3F00"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>W: TB_H_PART_CANDIDATE</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
               <a:solidFill>
                 <a:srgbClr val="1F3864"/>
               </a:solidFill>
               <a:latin typeface="Arial"/>
               <a:cs typeface="Arial"/>
             </a:rPr>
-            <a:t>R: TB_M_H0125_DESTINATION</a:t>
+            <a:t>TB_M_PART_CANDIDATE_DEST</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
+              <a:solidFill>
+                <a:srgbClr val="1F3864"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:rPr>
+            <a:t>TB_M_PART_CANDIDATE</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
+              <a:solidFill>
+                <a:srgbClr val="1F3864"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:rPr>
+            <a:t>TB_H_PART_CANDIDATE</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
+              <a:solidFill>
+                <a:srgbClr val="1F3864"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:rPr>
+            <a:t>TB_M_H0125_DESTINATION</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -5156,7 +5045,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>1609725</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>984249</xdr:rowOff>
+      <xdr:rowOff>996950</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -5166,7 +5055,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="14268450" y="3702050"/>
-          <a:ext cx="1571625" cy="965200"/>
+          <a:ext cx="1571625" cy="977900"/>
         </a:xfrm>
         <a:prstGeom prst="can">
           <a:avLst/>
@@ -5186,16 +5075,16 @@
         </a:bodyPr>
         <a:lstStyle/>
         <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
               <a:solidFill>
                 <a:srgbClr val="1F3864"/>
               </a:solidFill>
               <a:latin typeface="Arial"/>
               <a:cs typeface="Arial"/>
             </a:rPr>
-            <a:t>R: TB_M_PART_CANDIDATE</a:t>
+            <a:t>TB_M_PART_CANDIDATE</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -5213,7 +5102,7 @@
       <xdr:col>19</xdr:col>
       <xdr:colOff>1609725</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>984249</xdr:rowOff>
+      <xdr:rowOff>996950</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -5223,7 +5112,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="16173450" y="3702050"/>
-          <a:ext cx="1571625" cy="965200"/>
+          <a:ext cx="1571625" cy="977900"/>
         </a:xfrm>
         <a:prstGeom prst="can">
           <a:avLst/>
@@ -5243,81 +5132,55 @@
         </a:bodyPr>
         <a:lstStyle/>
         <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="7B3F00"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>W: TB_R_CROSSDOCK_IF_RESULT (dummy)</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="7B3F00"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>W: TB_M_PART_CANDIDATE (SYNC_STATUS)</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="7B3F00"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>W: TB_H_PART_CANDIDATE</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="7B3F00"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>W: Log</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
               <a:solidFill>
                 <a:srgbClr val="1F3864"/>
               </a:solidFill>
               <a:latin typeface="Arial"/>
               <a:cs typeface="Arial"/>
             </a:rPr>
-            <a:t>R: TB_M_PART_CANDIDATE</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
+            <a:t>TB_R_CROSSDOCK_IF_RESULT</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
               <a:solidFill>
                 <a:srgbClr val="1F3864"/>
               </a:solidFill>
               <a:latin typeface="Arial"/>
               <a:cs typeface="Arial"/>
             </a:rPr>
-            <a:t>R: TB_M_PART_CANDIDATE_DEST</a:t>
+            <a:t>TB_M_PART_CANDIDATE</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
+              <a:solidFill>
+                <a:srgbClr val="1F3864"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:rPr>
+            <a:t>TB_H_PART_CANDIDATE</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
+              <a:solidFill>
+                <a:srgbClr val="1F3864"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:rPr>
+            <a:t>TB_M_PART_CANDIDATE_DEST</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -5344,7 +5207,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1399117" y="7994650"/>
+          <a:off x="1399117" y="8007350"/>
           <a:ext cx="666750" cy="247650"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5401,7 +5264,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm rot="10800000">
-          <a:off x="1961092" y="7994650"/>
+          <a:off x="1961092" y="8007350"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="rtTriangle">
@@ -5437,7 +5300,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="676275" y="8378825"/>
+          <a:off x="676275" y="8391525"/>
           <a:ext cx="2112433" cy="152400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5490,7 +5353,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3511550" y="7994650"/>
+          <a:off x="3511550" y="8007350"/>
           <a:ext cx="666750" cy="247650"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5547,7 +5410,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm rot="10800000">
-          <a:off x="4073525" y="7994650"/>
+          <a:off x="4073525" y="8007350"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="rtTriangle">
@@ -5583,7 +5446,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2788708" y="8378825"/>
+          <a:off x="2788708" y="8391525"/>
           <a:ext cx="2112433" cy="152400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5636,7 +5499,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5623983" y="7994650"/>
+          <a:off x="5623983" y="8007350"/>
           <a:ext cx="666750" cy="247650"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5693,7 +5556,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm rot="10800000">
-          <a:off x="6185958" y="7994650"/>
+          <a:off x="6185958" y="8007350"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="rtTriangle">
@@ -5729,7 +5592,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4901142" y="8378825"/>
+          <a:off x="4901142" y="8391525"/>
           <a:ext cx="2112433" cy="152400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5782,7 +5645,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7736417" y="7994650"/>
+          <a:off x="7736417" y="8007350"/>
           <a:ext cx="666750" cy="247650"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5840,7 +5703,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm rot="10800000">
-          <a:off x="8298392" y="7994650"/>
+          <a:off x="8298392" y="8007350"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="rtTriangle">
@@ -5876,7 +5739,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7013575" y="8378825"/>
+          <a:off x="7013575" y="8391525"/>
           <a:ext cx="2112433" cy="152400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5929,7 +5792,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9848850" y="7975600"/>
+          <a:off x="9848850" y="7988300"/>
           <a:ext cx="666750" cy="285750"/>
         </a:xfrm>
         <a:prstGeom prst="can">
@@ -5986,7 +5849,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9126008" y="8378825"/>
+          <a:off x="9126008" y="8391525"/>
           <a:ext cx="2112433" cy="152400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -6039,7 +5902,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="12170833" y="8061325"/>
+          <a:off x="12170833" y="8074025"/>
           <a:ext cx="247650" cy="114300"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -6096,7 +5959,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="11238442" y="8378825"/>
+          <a:off x="11238442" y="8391525"/>
           <a:ext cx="2112433" cy="152400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -6149,7 +6012,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14264217" y="8061325"/>
+          <a:off x="14264217" y="8074025"/>
           <a:ext cx="295275" cy="114300"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -6204,7 +6067,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13350875" y="8378825"/>
+          <a:off x="13350875" y="8391525"/>
           <a:ext cx="2112433" cy="152400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -6257,7 +6120,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="16186150" y="8118475"/>
+          <a:off x="16186150" y="8131175"/>
           <a:ext cx="666750" cy="9525"/>
         </a:xfrm>
         <a:custGeom>
@@ -6308,7 +6171,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="15463308" y="8378825"/>
+          <a:off x="15463308" y="8391525"/>
           <a:ext cx="2112433" cy="152400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -6356,12 +6219,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="100" name="legend Data flow (W / R)"/>
+        <xdr:cNvPr id="100" name="legend Data flow"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="18298583" y="8118475"/>
+          <a:off x="18298583" y="8131175"/>
           <a:ext cx="666750" cy="9525"/>
         </a:xfrm>
         <a:custGeom>
@@ -6408,12 +6271,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="101" name="legend caption Data flow (W / R)"/>
+        <xdr:cNvPr id="101" name="legend caption Data flow"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="17575742" y="8378825"/>
+          <a:off x="17575742" y="8391525"/>
           <a:ext cx="2112433" cy="152400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -6439,7 +6302,7 @@
               <a:latin typeface="Arial"/>
               <a:cs typeface="Arial"/>
             </a:rPr>
-            <a:t>Data flow (W / R)</a:t>
+            <a:t>Data flow</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -6586,7 +6449,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="4391025" y="3048000"/>
-          <a:ext cx="371475" cy="2371725"/>
+          <a:ext cx="371475" cy="2136775"/>
         </a:xfrm>
         <a:custGeom>
           <a:avLst/>
@@ -6595,7 +6458,7 @@
           <a:cxnLst/>
           <a:rect l="0" t="0" r="r" b="b"/>
           <a:pathLst>
-            <a:path w="371475" h="2371725" fill="none">
+            <a:path w="371475" h="2136775" fill="none">
               <a:moveTo>
                 <a:pt x="0" y="0"/>
               </a:moveTo>
@@ -6603,10 +6466,10 @@
                 <a:pt x="209550" y="0"/>
               </a:lnTo>
               <a:lnTo>
-                <a:pt x="209550" y="2371725"/>
+                <a:pt x="209550" y="2136775"/>
               </a:lnTo>
               <a:lnTo>
-                <a:pt x="371475" y="2371725"/>
+                <a:pt x="371475" y="2136775"/>
               </a:lnTo>
             </a:path>
           </a:pathLst>
@@ -6643,7 +6506,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="4391025" y="3048000"/>
-          <a:ext cx="371475" cy="3171825"/>
+          <a:ext cx="371475" cy="2936875"/>
         </a:xfrm>
         <a:custGeom>
           <a:avLst/>
@@ -6652,7 +6515,7 @@
           <a:cxnLst/>
           <a:rect l="0" t="0" r="r" b="b"/>
           <a:pathLst>
-            <a:path w="371475" h="3171825" fill="none">
+            <a:path w="371475" h="2936875" fill="none">
               <a:moveTo>
                 <a:pt x="0" y="0"/>
               </a:moveTo>
@@ -6660,10 +6523,10 @@
                 <a:pt x="161925" y="0"/>
               </a:lnTo>
               <a:lnTo>
-                <a:pt x="161925" y="3171825"/>
+                <a:pt x="161925" y="2936875"/>
               </a:lnTo>
               <a:lnTo>
-                <a:pt x="371475" y="3171825"/>
+                <a:pt x="371475" y="2936875"/>
               </a:lnTo>
             </a:path>
           </a:pathLst>
@@ -6700,7 +6563,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="6296025" y="3048000"/>
-          <a:ext cx="371475" cy="2324100"/>
+          <a:ext cx="371475" cy="2089150"/>
         </a:xfrm>
         <a:custGeom>
           <a:avLst/>
@@ -6709,12 +6572,12 @@
           <a:cxnLst/>
           <a:rect l="0" t="0" r="r" b="b"/>
           <a:pathLst>
-            <a:path w="371475" h="2324100" fill="none">
+            <a:path w="371475" h="2089150" fill="none">
               <a:moveTo>
-                <a:pt x="0" y="2324100"/>
+                <a:pt x="0" y="2089150"/>
               </a:moveTo>
               <a:lnTo>
-                <a:pt x="185738" y="2324100"/>
+                <a:pt x="185738" y="2089150"/>
               </a:lnTo>
               <a:lnTo>
                 <a:pt x="185738" y="0"/>
@@ -6757,7 +6620,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="6296025" y="3095625"/>
-          <a:ext cx="371475" cy="3171825"/>
+          <a:ext cx="371475" cy="2936875"/>
         </a:xfrm>
         <a:custGeom>
           <a:avLst/>
@@ -6766,12 +6629,12 @@
           <a:cxnLst/>
           <a:rect l="0" t="0" r="r" b="b"/>
           <a:pathLst>
-            <a:path w="371475" h="3171825" fill="none">
+            <a:path w="371475" h="2936875" fill="none">
               <a:moveTo>
-                <a:pt x="0" y="3171825"/>
+                <a:pt x="0" y="2936875"/>
               </a:moveTo>
               <a:lnTo>
-                <a:pt x="209550" y="3171825"/>
+                <a:pt x="209550" y="2936875"/>
               </a:lnTo>
               <a:lnTo>
                 <a:pt x="209550" y="0"/>
@@ -6814,7 +6677,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="8201025" y="3048000"/>
-          <a:ext cx="371475" cy="3171825"/>
+          <a:ext cx="371475" cy="2936875"/>
         </a:xfrm>
         <a:custGeom>
           <a:avLst/>
@@ -6823,7 +6686,7 @@
           <a:cxnLst/>
           <a:rect l="0" t="0" r="r" b="b"/>
           <a:pathLst>
-            <a:path w="371475" h="3171825" fill="none">
+            <a:path w="371475" h="2936875" fill="none">
               <a:moveTo>
                 <a:pt x="0" y="0"/>
               </a:moveTo>
@@ -6831,10 +6694,10 @@
                 <a:pt x="161925" y="0"/>
               </a:lnTo>
               <a:lnTo>
-                <a:pt x="161925" y="3171825"/>
+                <a:pt x="161925" y="2936875"/>
               </a:lnTo>
               <a:lnTo>
-                <a:pt x="371475" y="3171825"/>
+                <a:pt x="371475" y="2936875"/>
               </a:lnTo>
             </a:path>
           </a:pathLst>
@@ -6871,7 +6734,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="10106025" y="3048000"/>
-          <a:ext cx="371475" cy="3219450"/>
+          <a:ext cx="371475" cy="2984500"/>
         </a:xfrm>
         <a:custGeom>
           <a:avLst/>
@@ -6880,12 +6743,12 @@
           <a:cxnLst/>
           <a:rect l="0" t="0" r="r" b="b"/>
           <a:pathLst>
-            <a:path w="371475" h="3219450" fill="none">
+            <a:path w="371475" h="2984500" fill="none">
               <a:moveTo>
-                <a:pt x="0" y="3219450"/>
+                <a:pt x="0" y="2984500"/>
               </a:moveTo>
               <a:lnTo>
-                <a:pt x="185738" y="3219450"/>
+                <a:pt x="185738" y="2984500"/>
               </a:lnTo>
               <a:lnTo>
                 <a:pt x="185738" y="0"/>
@@ -6928,7 +6791,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="12011025" y="3048000"/>
-          <a:ext cx="371475" cy="3267075"/>
+          <a:ext cx="371475" cy="3032125"/>
         </a:xfrm>
         <a:custGeom>
           <a:avLst/>
@@ -6937,7 +6800,7 @@
           <a:cxnLst/>
           <a:rect l="0" t="0" r="r" b="b"/>
           <a:pathLst>
-            <a:path w="371475" h="3267075" fill="none">
+            <a:path w="371475" h="3032125" fill="none">
               <a:moveTo>
                 <a:pt x="0" y="0"/>
               </a:moveTo>
@@ -6945,10 +6808,10 @@
                 <a:pt x="209550" y="0"/>
               </a:lnTo>
               <a:lnTo>
-                <a:pt x="209550" y="3267075"/>
+                <a:pt x="209550" y="3032125"/>
               </a:lnTo>
               <a:lnTo>
-                <a:pt x="371475" y="3267075"/>
+                <a:pt x="371475" y="3032125"/>
               </a:lnTo>
             </a:path>
           </a:pathLst>
@@ -6985,7 +6848,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="13916025" y="3000375"/>
-          <a:ext cx="371475" cy="3267075"/>
+          <a:ext cx="371475" cy="3032125"/>
         </a:xfrm>
         <a:custGeom>
           <a:avLst/>
@@ -6994,12 +6857,12 @@
           <a:cxnLst/>
           <a:rect l="0" t="0" r="r" b="b"/>
           <a:pathLst>
-            <a:path w="371475" h="3267075" fill="none">
+            <a:path w="371475" h="3032125" fill="none">
               <a:moveTo>
-                <a:pt x="0" y="3267075"/>
+                <a:pt x="0" y="3032125"/>
               </a:moveTo>
               <a:lnTo>
-                <a:pt x="161925" y="3267075"/>
+                <a:pt x="161925" y="3032125"/>
               </a:lnTo>
               <a:lnTo>
                 <a:pt x="161925" y="0"/>
@@ -7042,7 +6905,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="15821025" y="3048000"/>
-          <a:ext cx="371475" cy="3219450"/>
+          <a:ext cx="371475" cy="2984500"/>
         </a:xfrm>
         <a:custGeom>
           <a:avLst/>
@@ -7051,7 +6914,7 @@
           <a:cxnLst/>
           <a:rect l="0" t="0" r="r" b="b"/>
           <a:pathLst>
-            <a:path w="371475" h="3219450" fill="none">
+            <a:path w="371475" h="2984500" fill="none">
               <a:moveTo>
                 <a:pt x="0" y="0"/>
               </a:moveTo>
@@ -7059,10 +6922,10 @@
                 <a:pt x="185738" y="0"/>
               </a:lnTo>
               <a:lnTo>
-                <a:pt x="185738" y="3219450"/>
+                <a:pt x="185738" y="2984500"/>
               </a:lnTo>
               <a:lnTo>
-                <a:pt x="371475" y="3219450"/>
+                <a:pt x="371475" y="2984500"/>
               </a:lnTo>
             </a:path>
           </a:pathLst>
@@ -7156,7 +7019,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="15821025" y="3048000"/>
-          <a:ext cx="2276475" cy="3171825"/>
+          <a:ext cx="2276475" cy="2936875"/>
         </a:xfrm>
         <a:custGeom>
           <a:avLst/>
@@ -7165,7 +7028,7 @@
           <a:cxnLst/>
           <a:rect l="0" t="0" r="r" b="b"/>
           <a:pathLst>
-            <a:path w="2276475" h="3171825" fill="none">
+            <a:path w="2276475" h="2936875" fill="none">
               <a:moveTo>
                 <a:pt x="0" y="0"/>
               </a:moveTo>
@@ -7173,16 +7036,16 @@
                 <a:pt x="161925" y="0"/>
               </a:lnTo>
               <a:lnTo>
-                <a:pt x="161925" y="2770188"/>
+                <a:pt x="161925" y="2535237"/>
               </a:lnTo>
               <a:lnTo>
-                <a:pt x="2066925" y="2770188"/>
+                <a:pt x="2066925" y="2535237"/>
               </a:lnTo>
               <a:lnTo>
-                <a:pt x="2066925" y="3171825"/>
+                <a:pt x="2066925" y="2936875"/>
               </a:lnTo>
               <a:lnTo>
-                <a:pt x="2276475" y="3171825"/>
+                <a:pt x="2276475" y="2936875"/>
               </a:lnTo>
             </a:path>
           </a:pathLst>
@@ -7296,7 +7159,6 @@
             <a:srgbClr val="2E75B6"/>
           </a:solidFill>
           <a:prstDash val="dash"/>
-          <a:headEnd type="triangle" w="sm" len="sm"/>
           <a:tailEnd type="triangle" w="sm" len="sm"/>
         </a:ln>
       </xdr:spPr>
@@ -7308,7 +7170,7 @@
       <xdr:col>7</xdr:col>
       <xdr:colOff>1130617</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>1104900</xdr:rowOff>
+      <xdr:rowOff>869949</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
@@ -7323,7 +7185,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5835968" y="4787900"/>
+          <a:off x="5835968" y="4552950"/>
           <a:ext cx="9525" cy="352425"/>
         </a:xfrm>
         <a:custGeom>
@@ -7349,7 +7211,6 @@
             <a:srgbClr val="2E75B6"/>
           </a:solidFill>
           <a:prstDash val="dash"/>
-          <a:headEnd type="triangle" w="sm" len="sm"/>
           <a:tailEnd type="triangle" w="sm" len="sm"/>
         </a:ln>
       </xdr:spPr>
@@ -7402,7 +7263,6 @@
             <a:srgbClr val="2E75B6"/>
           </a:solidFill>
           <a:prstDash val="dash"/>
-          <a:headEnd type="triangle" w="sm" len="sm"/>
           <a:tailEnd type="triangle" w="sm" len="sm"/>
         </a:ln>
       </xdr:spPr>
@@ -7414,7 +7274,7 @@
       <xdr:col>11</xdr:col>
       <xdr:colOff>1130617</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>1104900</xdr:rowOff>
+      <xdr:rowOff>869949</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
@@ -7429,7 +7289,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9645968" y="4787900"/>
+          <a:off x="9645968" y="4552950"/>
           <a:ext cx="9525" cy="1177925"/>
         </a:xfrm>
         <a:custGeom>
@@ -7455,7 +7315,7 @@
             <a:srgbClr val="2E75B6"/>
           </a:solidFill>
           <a:prstDash val="dash"/>
-          <a:headEnd type="triangle" w="sm" len="sm"/>
+          <a:tailEnd type="triangle" w="sm" len="sm"/>
         </a:ln>
       </xdr:spPr>
     </xdr:sp>
@@ -7507,7 +7367,6 @@
             <a:srgbClr val="2E75B6"/>
           </a:solidFill>
           <a:prstDash val="dash"/>
-          <a:headEnd type="triangle" w="sm" len="sm"/>
           <a:tailEnd type="triangle" w="sm" len="sm"/>
         </a:ln>
       </xdr:spPr>
@@ -7519,7 +7378,7 @@
       <xdr:col>15</xdr:col>
       <xdr:colOff>1130617</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>1104900</xdr:rowOff>
+      <xdr:rowOff>869949</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>15</xdr:col>
@@ -7534,7 +7393,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13455968" y="4787900"/>
+          <a:off x="13455968" y="4552950"/>
           <a:ext cx="9525" cy="1177925"/>
         </a:xfrm>
         <a:custGeom>
@@ -7560,7 +7419,7 @@
             <a:srgbClr val="2E75B6"/>
           </a:solidFill>
           <a:prstDash val="dash"/>
-          <a:headEnd type="triangle" w="sm" len="sm"/>
+          <a:tailEnd type="triangle" w="sm" len="sm"/>
         </a:ln>
       </xdr:spPr>
     </xdr:sp>
@@ -7612,7 +7471,6 @@
             <a:srgbClr val="2E75B6"/>
           </a:solidFill>
           <a:prstDash val="dash"/>
-          <a:headEnd type="triangle" w="sm" len="sm"/>
           <a:tailEnd type="triangle" w="sm" len="sm"/>
         </a:ln>
       </xdr:spPr>
@@ -7624,7 +7482,7 @@
       <xdr:col>19</xdr:col>
       <xdr:colOff>1130617</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>1104900</xdr:rowOff>
+      <xdr:rowOff>869949</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>19</xdr:col>
@@ -7639,7 +7497,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="17265968" y="4787900"/>
+          <a:off x="17265968" y="4552950"/>
           <a:ext cx="9525" cy="1177925"/>
         </a:xfrm>
         <a:custGeom>
@@ -7665,59 +7523,7 @@
             <a:srgbClr val="2E75B6"/>
           </a:solidFill>
           <a:prstDash val="dash"/>
-          <a:headEnd type="triangle" w="sm" len="sm"/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>21</xdr:col>
-      <xdr:colOff>1130617</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>1104900</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>21</xdr:col>
-      <xdr:colOff>1140142</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>28575</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="24" name="data D13"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="19170968" y="4787900"/>
-          <a:ext cx="9525" cy="1177925"/>
-        </a:xfrm>
-        <a:custGeom>
-          <a:avLst/>
-          <a:gdLst/>
-          <a:ahLst/>
-          <a:cxnLst/>
-          <a:rect l="0" t="0" r="r" b="b"/>
-          <a:pathLst>
-            <a:path w="9525" h="1177925" fill="none">
-              <a:moveTo>
-                <a:pt x="0" y="1177925"/>
-              </a:moveTo>
-              <a:lnTo>
-                <a:pt x="0" y="0"/>
-              </a:lnTo>
-            </a:path>
-          </a:pathLst>
-        </a:custGeom>
-        <a:noFill/>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="2E75B6"/>
-          </a:solidFill>
-          <a:prstDash val="dash"/>
-          <a:headEnd type="triangle" w="sm" len="sm"/>
+          <a:tailEnd type="triangle" w="sm" len="sm"/>
         </a:ln>
       </xdr:spPr>
     </xdr:sp>
@@ -7738,7 +7544,7 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="25" name="step D1"/>
+        <xdr:cNvPr id="24" name="step D1"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -7821,7 +7627,7 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="26" name="step D1 corner"/>
+        <xdr:cNvPr id="25" name="step D1 corner"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -7857,7 +7663,7 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="27" name="no D1"/>
+        <xdr:cNvPr id="26" name="no D1"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -7914,7 +7720,7 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="28" name="step D2"/>
+        <xdr:cNvPr id="27" name="step D2"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -7985,7 +7791,7 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="29" name="step D2 corner"/>
+        <xdr:cNvPr id="28" name="step D2 corner"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -8021,7 +7827,7 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="30" name="no D2"/>
+        <xdr:cNvPr id="29" name="no D2"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -8078,7 +7884,7 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="31" name="step D3"/>
+        <xdr:cNvPr id="30" name="step D3"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -8148,7 +7954,7 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="32" name="step D3 corner"/>
+        <xdr:cNvPr id="31" name="step D3 corner"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -8184,7 +7990,7 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="33" name="no D3"/>
+        <xdr:cNvPr id="32" name="no D3"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -8241,7 +8047,7 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="34" name="ab D3 AB07"/>
+        <xdr:cNvPr id="33" name="ab D3 AB07"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -8296,12 +8102,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="35" name="step D4"/>
+        <xdr:cNvPr id="34" name="step D4"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4762500" y="5140325"/>
+          <a:off x="4762500" y="4905375"/>
           <a:ext cx="1533525" cy="463550"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -8366,12 +8172,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="36" name="step D4 corner"/>
+        <xdr:cNvPr id="35" name="step D4 corner"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm rot="10800000">
-          <a:off x="6191250" y="5140325"/>
+          <a:off x="6191250" y="4905375"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="rtTriangle">
@@ -8402,12 +8208,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="37" name="no D4"/>
+        <xdr:cNvPr id="36" name="no D4"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4733925" y="5073650"/>
+          <a:off x="4733925" y="4838700"/>
           <a:ext cx="247650" cy="114300"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -8459,12 +8265,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="38" name="step D5"/>
+        <xdr:cNvPr id="37" name="step D5"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4762500" y="5965825"/>
+          <a:off x="4762500" y="5730875"/>
           <a:ext cx="1533525" cy="603250"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -8529,12 +8335,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="39" name="step D5 corner"/>
+        <xdr:cNvPr id="38" name="step D5 corner"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm rot="10800000">
-          <a:off x="6191250" y="5965825"/>
+          <a:off x="6191250" y="5730875"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="rtTriangle">
@@ -8565,12 +8371,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="40" name="no D5"/>
+        <xdr:cNvPr id="39" name="no D5"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4733925" y="5899150"/>
+          <a:off x="4733925" y="5664200"/>
           <a:ext cx="247650" cy="114300"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -8622,7 +8428,7 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="41" name="step D6"/>
+        <xdr:cNvPr id="40" name="step D6"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -8692,7 +8498,7 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="42" name="step D6 corner"/>
+        <xdr:cNvPr id="41" name="step D6 corner"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -8728,7 +8534,7 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="43" name="no D6"/>
+        <xdr:cNvPr id="42" name="no D6"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -8785,7 +8591,7 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="44" name="ab D6 AB08"/>
+        <xdr:cNvPr id="43" name="ab D6 AB08"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -8840,12 +8646,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="45" name="step D7"/>
+        <xdr:cNvPr id="44" name="step D7"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="8572500" y="5965825"/>
+          <a:off x="8572500" y="5730875"/>
           <a:ext cx="1533525" cy="603250"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -8910,12 +8716,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="46" name="step D7 corner"/>
+        <xdr:cNvPr id="45" name="step D7 corner"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm rot="10800000">
-          <a:off x="10001250" y="5965825"/>
+          <a:off x="10001250" y="5730875"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="rtTriangle">
@@ -8946,12 +8752,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="47" name="no D7"/>
+        <xdr:cNvPr id="46" name="no D7"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="8543925" y="5899150"/>
+          <a:off x="8543925" y="5664200"/>
           <a:ext cx="247650" cy="114300"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -9003,12 +8809,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="48" name="ab D7 AB09"/>
+        <xdr:cNvPr id="47" name="ab D7 AB09"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9801225" y="5899150"/>
+          <a:off x="9801225" y="5664200"/>
           <a:ext cx="295275" cy="114300"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -9058,12 +8864,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="49" name="ab D7 AB10"/>
+        <xdr:cNvPr id="48" name="ab D7 AB10"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9486900" y="5899150"/>
+          <a:off x="9486900" y="5664200"/>
           <a:ext cx="295275" cy="114300"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -9113,12 +8919,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="50" name="ab D7 AB11"/>
+        <xdr:cNvPr id="49" name="ab D7 AB11"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9172575" y="5899150"/>
+          <a:off x="9172575" y="5664200"/>
           <a:ext cx="295275" cy="114300"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -9168,7 +8974,7 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="51" name="step D8"/>
+        <xdr:cNvPr id="50" name="step D8"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -9238,7 +9044,7 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="52" name="step D8 corner"/>
+        <xdr:cNvPr id="51" name="step D8 corner"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -9274,7 +9080,7 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="53" name="no D8"/>
+        <xdr:cNvPr id="52" name="no D8"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -9331,12 +9137,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="54" name="step D9"/>
+        <xdr:cNvPr id="53" name="step D9"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="12382500" y="5965825"/>
+          <a:off x="12382500" y="5730875"/>
           <a:ext cx="1533525" cy="603250"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -9401,12 +9207,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="55" name="step D9 corner"/>
+        <xdr:cNvPr id="54" name="step D9 corner"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm rot="10800000">
-          <a:off x="13811250" y="5965825"/>
+          <a:off x="13811250" y="5730875"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="rtTriangle">
@@ -9437,12 +9243,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="56" name="no D9"/>
+        <xdr:cNvPr id="55" name="no D9"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="12353925" y="5899150"/>
+          <a:off x="12353925" y="5664200"/>
           <a:ext cx="247650" cy="114300"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -9494,12 +9300,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="57" name="ab D9 AB12"/>
+        <xdr:cNvPr id="56" name="ab D9 AB12"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13611225" y="5899150"/>
+          <a:off x="13611225" y="5664200"/>
           <a:ext cx="295275" cy="114300"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -9549,7 +9355,7 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="58" name="step D10"/>
+        <xdr:cNvPr id="57" name="step D10"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -9619,7 +9425,7 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="59" name="step D10 corner"/>
+        <xdr:cNvPr id="58" name="step D10 corner"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -9655,7 +9461,7 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="60" name="no D10"/>
+        <xdr:cNvPr id="59" name="no D10"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -9712,7 +9518,7 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="61" name="ab D10 AB13"/>
+        <xdr:cNvPr id="60" name="ab D10 AB13"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -9767,12 +9573,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="62" name="step D11"/>
+        <xdr:cNvPr id="61" name="step D11"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="16192500" y="5965825"/>
+          <a:off x="16192500" y="5730875"/>
           <a:ext cx="1533525" cy="603250"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -9837,12 +9643,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="63" name="step D11 corner"/>
+        <xdr:cNvPr id="62" name="step D11 corner"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm rot="10800000">
-          <a:off x="17621250" y="5965825"/>
+          <a:off x="17621250" y="5730875"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="rtTriangle">
@@ -9873,12 +9679,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="64" name="no D11"/>
+        <xdr:cNvPr id="63" name="no D11"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="16163925" y="5899150"/>
+          <a:off x="16163925" y="5664200"/>
           <a:ext cx="247650" cy="114300"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -9930,7 +9736,7 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="65" name="step D12"/>
+        <xdr:cNvPr id="64" name="step D12"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -10014,7 +9820,7 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="66" name="step D12 corner"/>
+        <xdr:cNvPr id="65" name="step D12 corner"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -10050,7 +9856,7 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="67" name="no D12"/>
+        <xdr:cNvPr id="66" name="no D12"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -10107,12 +9913,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="68" name="step D13"/>
+        <xdr:cNvPr id="67" name="step D13"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="18097500" y="5965825"/>
+          <a:off x="18097500" y="5730875"/>
           <a:ext cx="1533525" cy="603250"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -10177,12 +9983,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="69" name="step D13 corner"/>
+        <xdr:cNvPr id="68" name="step D13 corner"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm rot="10800000">
-          <a:off x="19526250" y="5965825"/>
+          <a:off x="19526250" y="5730875"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="rtTriangle">
@@ -10213,12 +10019,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="70" name="no D13"/>
+        <xdr:cNvPr id="69" name="no D13"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="18068925" y="5899150"/>
+          <a:off x="18068925" y="5664200"/>
           <a:ext cx="247650" cy="114300"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -10270,12 +10076,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="71" name="ab D13 AB13"/>
+        <xdr:cNvPr id="70" name="ab D13 AB13"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="19326225" y="5899150"/>
+          <a:off x="19326225" y="5664200"/>
           <a:ext cx="295275" cy="114300"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -10321,17 +10127,17 @@
       <xdr:col>3</xdr:col>
       <xdr:colOff>1609725</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>1104900</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="72" name="db D2"/>
+      <xdr:rowOff>869949</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="71" name="db D2"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
           <a:off x="933450" y="3702050"/>
-          <a:ext cx="1571625" cy="1085850"/>
+          <a:ext cx="1571625" cy="850900"/>
         </a:xfrm>
         <a:prstGeom prst="can">
           <a:avLst/>
@@ -10351,16 +10157,16 @@
         </a:bodyPr>
         <a:lstStyle/>
         <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="7B3F00"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>W: TB_R_PRA_DAILY_ORDER_MANIFEST / PART</a:t>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
+              <a:solidFill>
+                <a:srgbClr val="1F3864"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:rPr>
+            <a:t>TB_R_PRA_DAILY_ORDER_MANIFEST / PART</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -10378,17 +10184,17 @@
       <xdr:col>5</xdr:col>
       <xdr:colOff>1609725</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>1104900</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="73" name="db D3"/>
+      <xdr:rowOff>869949</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="72" name="db D3"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
           <a:off x="2838450" y="3702050"/>
-          <a:ext cx="1571625" cy="1085850"/>
+          <a:ext cx="1571625" cy="850900"/>
         </a:xfrm>
         <a:prstGeom prst="can">
           <a:avLst/>
@@ -10408,42 +10214,16 @@
         </a:bodyPr>
         <a:lstStyle/>
         <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="7B3F00"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>W: TB_R_H0253_ORDER_CONTROL_PRE (NSP)</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="7B3F00"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>W: Log</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
               <a:solidFill>
                 <a:srgbClr val="1F3864"/>
               </a:solidFill>
               <a:latin typeface="Arial"/>
               <a:cs typeface="Arial"/>
             </a:rPr>
-            <a:t>R: TB_R_H0253_ORDER_CONTROL_PRE (DB Surrounding)</a:t>
+            <a:t>TB_R_H0253_ORDER_CONTROL_PRE</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -10461,17 +10241,17 @@
       <xdr:col>7</xdr:col>
       <xdr:colOff>1609725</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>1104900</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="74" name="db D4"/>
+      <xdr:rowOff>869949</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="73" name="db D4"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
           <a:off x="4743450" y="3702050"/>
-          <a:ext cx="1571625" cy="1085850"/>
+          <a:ext cx="1571625" cy="850900"/>
         </a:xfrm>
         <a:prstGeom prst="can">
           <a:avLst/>
@@ -10491,29 +10271,16 @@
         </a:bodyPr>
         <a:lstStyle/>
         <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="7B3F00"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>W: TB_R_H0253_ORDER_CONTROL_PRE (HOLD_FLAG)</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
               <a:solidFill>
                 <a:srgbClr val="1F3864"/>
               </a:solidFill>
               <a:latin typeface="Arial"/>
               <a:cs typeface="Arial"/>
             </a:rPr>
-            <a:t>R: TB_R_H0253_ORDER_CONTROL_PRE</a:t>
+            <a:t>TB_R_H0253_ORDER_CONTROL_PRE</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -10531,17 +10298,17 @@
       <xdr:col>9</xdr:col>
       <xdr:colOff>1609725</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>1104900</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="75" name="db D6"/>
+      <xdr:rowOff>869949</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="74" name="db D6"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
           <a:off x="6648450" y="3702050"/>
-          <a:ext cx="1571625" cy="1085850"/>
+          <a:ext cx="1571625" cy="850900"/>
         </a:xfrm>
         <a:prstGeom prst="can">
           <a:avLst/>
@@ -10561,55 +10328,55 @@
         </a:bodyPr>
         <a:lstStyle/>
         <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="7B3F00"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>W: #TEMP_INSTRUCTION</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
               <a:solidFill>
                 <a:srgbClr val="1F3864"/>
               </a:solidFill>
               <a:latin typeface="Arial"/>
               <a:cs typeface="Arial"/>
             </a:rPr>
-            <a:t>R: TB_R_H0253_ORDER_CONTROL_PRE (status 7, HOLD N, PO_MAPPED N)</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
+            <a:t>#TEMP_INSTRUCTION</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
               <a:solidFill>
                 <a:srgbClr val="1F3864"/>
               </a:solidFill>
               <a:latin typeface="Arial"/>
               <a:cs typeface="Arial"/>
             </a:rPr>
-            <a:t>R: TB_R_PRA_DAILY_ORDER_MANIFEST / PART</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
+            <a:t>TB_R_H0253_ORDER_CONTROL_PRE</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
               <a:solidFill>
                 <a:srgbClr val="1F3864"/>
               </a:solidFill>
               <a:latin typeface="Arial"/>
               <a:cs typeface="Arial"/>
             </a:rPr>
-            <a:t>R: TB_R_PRA_DAILY_ORDER_MAPPED</a:t>
+            <a:t>TB_R_PRA_DAILY_ORDER_MANIFEST / PART</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
+              <a:solidFill>
+                <a:srgbClr val="1F3864"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:rPr>
+            <a:t>TB_R_PRA_DAILY_ORDER_MAPPED</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -10627,17 +10394,17 @@
       <xdr:col>11</xdr:col>
       <xdr:colOff>1609725</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>1104900</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="76" name="db D7"/>
+      <xdr:rowOff>869949</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="75" name="db D7"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
           <a:off x="8553450" y="3702050"/>
-          <a:ext cx="1571625" cy="1085850"/>
+          <a:ext cx="1571625" cy="850900"/>
         </a:xfrm>
         <a:prstGeom prst="can">
           <a:avLst/>
@@ -10657,16 +10424,16 @@
         </a:bodyPr>
         <a:lstStyle/>
         <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
               <a:solidFill>
                 <a:srgbClr val="1F3864"/>
               </a:solidFill>
               <a:latin typeface="Arial"/>
               <a:cs typeface="Arial"/>
             </a:rPr>
-            <a:t>R: #TEMP_INSTRUCTION</a:t>
+            <a:t>#TEMP_INSTRUCTION</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -10684,17 +10451,17 @@
       <xdr:col>13</xdr:col>
       <xdr:colOff>1609725</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>1104900</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="77" name="db D8"/>
+      <xdr:rowOff>869949</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="76" name="db D8"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
           <a:off x="10458450" y="3702050"/>
-          <a:ext cx="1571625" cy="1085850"/>
+          <a:ext cx="1571625" cy="850900"/>
         </a:xfrm>
         <a:prstGeom prst="can">
           <a:avLst/>
@@ -10714,68 +10481,55 @@
         </a:bodyPr>
         <a:lstStyle/>
         <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="7B3F00"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>W: TB_R_INSTRUCTION</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="7B3F00"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>W: TB_R_H0253_ORDER_CONTROL_PRE (PO_MAPPED_FLAG Y)</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="7B3F00"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>W: TB_R_PRA_DAILY_ORDER_MAPPED (MAPPED_QTY)</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
               <a:solidFill>
                 <a:srgbClr val="1F3864"/>
               </a:solidFill>
               <a:latin typeface="Arial"/>
               <a:cs typeface="Arial"/>
             </a:rPr>
-            <a:t>R: #TEMP_INSTRUCTION</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
+            <a:t>TB_R_INSTRUCTION</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
               <a:solidFill>
                 <a:srgbClr val="1F3864"/>
               </a:solidFill>
               <a:latin typeface="Arial"/>
               <a:cs typeface="Arial"/>
             </a:rPr>
-            <a:t>R: TB_R_H0253_ORDER_CONTROL_PRE</a:t>
+            <a:t>TB_R_H0253_ORDER_CONTROL_PRE</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
+              <a:solidFill>
+                <a:srgbClr val="1F3864"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:rPr>
+            <a:t>TB_R_PRA_DAILY_ORDER_MAPPED</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
+              <a:solidFill>
+                <a:srgbClr val="1F3864"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:rPr>
+            <a:t>#TEMP_INSTRUCTION</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -10793,17 +10547,17 @@
       <xdr:col>15</xdr:col>
       <xdr:colOff>1609725</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>1104900</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="78" name="db D9"/>
+      <xdr:rowOff>869949</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="77" name="db D9"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
           <a:off x="12363450" y="3702050"/>
-          <a:ext cx="1571625" cy="1085850"/>
+          <a:ext cx="1571625" cy="850900"/>
         </a:xfrm>
         <a:prstGeom prst="can">
           <a:avLst/>
@@ -10823,16 +10577,16 @@
         </a:bodyPr>
         <a:lstStyle/>
         <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
               <a:solidFill>
                 <a:srgbClr val="1F3864"/>
               </a:solidFill>
               <a:latin typeface="Arial"/>
               <a:cs typeface="Arial"/>
             </a:rPr>
-            <a:t>R: TB_R_INSTRUCTION</a:t>
+            <a:t>TB_R_INSTRUCTION</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -10850,17 +10604,17 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>1609725</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>1104900</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="79" name="db D10"/>
+      <xdr:rowOff>869949</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="78" name="db D10"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
           <a:off x="14268450" y="3702050"/>
-          <a:ext cx="1571625" cy="1085850"/>
+          <a:ext cx="1571625" cy="850900"/>
         </a:xfrm>
         <a:prstGeom prst="can">
           <a:avLst/>
@@ -10880,81 +10634,42 @@
         </a:bodyPr>
         <a:lstStyle/>
         <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="7B3F00"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>W: TB_R_DAILY_ORDER_MANIFEST</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="7B3F00"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>W: TB_R_DAILY_ORDER_PART</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="7B3F00"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>W: TB_R_INSTRUCTION (ASN_NO, CASE_NO)</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="7B3F00"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>W: Log</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
               <a:solidFill>
                 <a:srgbClr val="1F3864"/>
               </a:solidFill>
               <a:latin typeface="Arial"/>
               <a:cs typeface="Arial"/>
             </a:rPr>
-            <a:t>R: TB_R_INSTRUCTION</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
+            <a:t>TB_R_DAILY_ORDER_MANIFEST</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
               <a:solidFill>
                 <a:srgbClr val="1F3864"/>
               </a:solidFill>
               <a:latin typeface="Arial"/>
               <a:cs typeface="Arial"/>
             </a:rPr>
-            <a:t>R: Existing last sequence table</a:t>
+            <a:t>TB_R_DAILY_ORDER_PART</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
+              <a:solidFill>
+                <a:srgbClr val="1F3864"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:rPr>
+            <a:t>TB_R_INSTRUCTION</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -10972,17 +10687,17 @@
       <xdr:col>19</xdr:col>
       <xdr:colOff>1609725</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>1104900</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="80" name="db D11"/>
+      <xdr:rowOff>869949</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="79" name="db D11"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
           <a:off x="16173450" y="3702050"/>
-          <a:ext cx="1571625" cy="1085850"/>
+          <a:ext cx="1571625" cy="850900"/>
         </a:xfrm>
         <a:prstGeom prst="can">
           <a:avLst/>
@@ -11002,86 +10717,29 @@
         </a:bodyPr>
         <a:lstStyle/>
         <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
               <a:solidFill>
                 <a:srgbClr val="1F3864"/>
               </a:solidFill>
               <a:latin typeface="Arial"/>
               <a:cs typeface="Arial"/>
             </a:rPr>
-            <a:t>R: TB_R_DAILY_ORDER_MANIFEST</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
+            <a:t>TB_R_DAILY_ORDER_MANIFEST</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
               <a:solidFill>
                 <a:srgbClr val="1F3864"/>
               </a:solidFill>
               <a:latin typeface="Arial"/>
               <a:cs typeface="Arial"/>
             </a:rPr>
-            <a:t>R: TB_R_DAILY_ORDER_PART</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>21</xdr:col>
-      <xdr:colOff>38100</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>21</xdr:col>
-      <xdr:colOff>1609725</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>1104900</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="81" name="db D13"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="18078450" y="3702050"/>
-          <a:ext cx="1571625" cy="1085850"/>
-        </a:xfrm>
-        <a:prstGeom prst="can">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="D9D9E8"/>
-        </a:solidFill>
-        <a:ln w="9525">
-          <a:solidFill>
-            <a:srgbClr val="595959"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="overflow" horzOverflow="overflow" wrap="square" lIns="28575" tIns="28575" rIns="28575" bIns="28575" anchor="b">
-          <a:noAutofit/>
-        </a:bodyPr>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="1F3864"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>R: Log</a:t>
+            <a:t>TB_R_DAILY_ORDER_PART</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -11103,12 +10761,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="82" name="legend NSP System"/>
+        <xdr:cNvPr id="80" name="legend NSP System"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1399117" y="6870700"/>
+          <a:off x="1399117" y="6635750"/>
           <a:ext cx="666750" cy="247650"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -11160,12 +10818,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="83" name="legend NSP System corner"/>
+        <xdr:cNvPr id="81" name="legend NSP System corner"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm rot="10800000">
-          <a:off x="1961092" y="6870700"/>
+          <a:off x="1961092" y="6635750"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="rtTriangle">
@@ -11196,12 +10854,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="84" name="legend caption NSP System"/>
+        <xdr:cNvPr id="82" name="legend caption NSP System"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="676275" y="7254875"/>
+          <a:off x="676275" y="7019925"/>
           <a:ext cx="2112433" cy="152400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -11249,12 +10907,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="85" name="legend G-TOPAS / AP POLE"/>
+        <xdr:cNvPr id="83" name="legend G-TOPAS / AP POLE"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3511550" y="6870700"/>
+          <a:off x="3511550" y="6635750"/>
           <a:ext cx="666750" cy="247650"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -11306,12 +10964,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="86" name="legend G-TOPAS / AP POLE corner"/>
+        <xdr:cNvPr id="84" name="legend G-TOPAS / AP POLE corner"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm rot="10800000">
-          <a:off x="4073525" y="6870700"/>
+          <a:off x="4073525" y="6635750"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="rtTriangle">
@@ -11342,12 +11000,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="87" name="legend caption G-TOPAS / AP POLE"/>
+        <xdr:cNvPr id="85" name="legend caption G-TOPAS / AP POLE"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2788708" y="7254875"/>
+          <a:off x="2788708" y="7019925"/>
           <a:ext cx="2112433" cy="152400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -11395,12 +11053,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="88" name="legend User (manual / screen)"/>
+        <xdr:cNvPr id="86" name="legend User (manual / screen)"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5623983" y="6870700"/>
+          <a:off x="5623983" y="6635750"/>
           <a:ext cx="666750" cy="247650"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -11452,12 +11110,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="89" name="legend User (manual / screen) corner"/>
+        <xdr:cNvPr id="87" name="legend User (manual / screen) corner"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm rot="10800000">
-          <a:off x="6185958" y="6870700"/>
+          <a:off x="6185958" y="6635750"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="rtTriangle">
@@ -11488,12 +11146,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="90" name="legend caption User (manual / screen)"/>
+        <xdr:cNvPr id="88" name="legend caption User (manual / screen)"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4901142" y="7254875"/>
+          <a:off x="4901142" y="7019925"/>
           <a:ext cx="2112433" cy="152400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -11541,12 +11199,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="91" name="legend Existing / manual"/>
+        <xdr:cNvPr id="89" name="legend Existing / manual"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7736417" y="6870700"/>
+          <a:off x="7736417" y="6635750"/>
           <a:ext cx="666750" cy="247650"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -11599,12 +11257,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="92" name="legend Existing / manual corner"/>
+        <xdr:cNvPr id="90" name="legend Existing / manual corner"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm rot="10800000">
-          <a:off x="8298392" y="6870700"/>
+          <a:off x="8298392" y="6635750"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="rtTriangle">
@@ -11635,12 +11293,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="93" name="legend caption Existing / manual"/>
+        <xdr:cNvPr id="91" name="legend caption Existing / manual"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7013575" y="7254875"/>
+          <a:off x="7013575" y="7019925"/>
           <a:ext cx="2112433" cy="152400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -11688,12 +11346,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="94" name="legend DB Storage (table)"/>
+        <xdr:cNvPr id="92" name="legend DB Storage (table)"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9848850" y="6851650"/>
+          <a:off x="9848850" y="6616700"/>
           <a:ext cx="666750" cy="285750"/>
         </a:xfrm>
         <a:prstGeom prst="can">
@@ -11745,12 +11403,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="95" name="legend caption DB Storage (table)"/>
+        <xdr:cNvPr id="93" name="legend caption DB Storage (table)"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9126008" y="7254875"/>
+          <a:off x="9126008" y="7019925"/>
           <a:ext cx="2112433" cy="152400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -11798,12 +11456,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="96" name="legend Step No"/>
+        <xdr:cNvPr id="94" name="legend Step No"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="12170833" y="6937375"/>
+          <a:off x="12170833" y="6702425"/>
           <a:ext cx="247650" cy="114300"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -11855,12 +11513,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="97" name="legend caption Step No"/>
+        <xdr:cNvPr id="95" name="legend caption Step No"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="11238442" y="7254875"/>
+          <a:off x="11238442" y="7019925"/>
           <a:ext cx="2112433" cy="152400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -11908,12 +11566,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="98" name="legend Abnormality"/>
+        <xdr:cNvPr id="96" name="legend Abnormality"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14264217" y="6937375"/>
+          <a:off x="14264217" y="6702425"/>
           <a:ext cx="295275" cy="114300"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -11963,12 +11621,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="99" name="legend caption Abnormality"/>
+        <xdr:cNvPr id="97" name="legend caption Abnormality"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13350875" y="7254875"/>
+          <a:off x="13350875" y="7019925"/>
           <a:ext cx="2112433" cy="152400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -12016,12 +11674,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="100" name="legend Process flow"/>
+        <xdr:cNvPr id="98" name="legend Process flow"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="16186150" y="6994525"/>
+          <a:off x="16186150" y="6759575"/>
           <a:ext cx="666750" cy="9525"/>
         </a:xfrm>
         <a:custGeom>
@@ -12067,12 +11725,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="101" name="legend caption Process flow"/>
+        <xdr:cNvPr id="99" name="legend caption Process flow"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="15463308" y="7254875"/>
+          <a:off x="15463308" y="7019925"/>
           <a:ext cx="2112433" cy="152400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -12120,12 +11778,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="102" name="legend Data flow (W / R)"/>
+        <xdr:cNvPr id="100" name="legend Data flow"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="18298583" y="6994525"/>
+          <a:off x="18298583" y="6759575"/>
           <a:ext cx="666750" cy="9525"/>
         </a:xfrm>
         <a:custGeom>
@@ -12172,12 +11830,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="103" name="legend caption Data flow (W / R)"/>
+        <xdr:cNvPr id="101" name="legend caption Data flow"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="17575742" y="7254875"/>
+          <a:off x="17575742" y="7019925"/>
           <a:ext cx="2112433" cy="152400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -12203,7 +11861,7 @@
               <a:latin typeface="Arial"/>
               <a:cs typeface="Arial"/>
             </a:rPr>
-            <a:t>Data flow (W / R)</a:t>
+            <a:t>Data flow</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -12464,7 +12122,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="8201025" y="3048000"/>
-          <a:ext cx="4181475" cy="2825750"/>
+          <a:ext cx="4181475" cy="2228850"/>
         </a:xfrm>
         <a:custGeom>
           <a:avLst/>
@@ -12473,7 +12131,7 @@
           <a:cxnLst/>
           <a:rect l="0" t="0" r="r" b="b"/>
           <a:pathLst>
-            <a:path w="4181475" h="2825750" fill="none">
+            <a:path w="4181475" h="2228850" fill="none">
               <a:moveTo>
                 <a:pt x="0" y="0"/>
               </a:moveTo>
@@ -12481,16 +12139,16 @@
                 <a:pt x="185738" y="0"/>
               </a:lnTo>
               <a:lnTo>
-                <a:pt x="185738" y="2330450"/>
+                <a:pt x="185738" y="1733550"/>
               </a:lnTo>
               <a:lnTo>
-                <a:pt x="3995738" y="2330450"/>
+                <a:pt x="3995738" y="1733550"/>
               </a:lnTo>
               <a:lnTo>
-                <a:pt x="3995738" y="2825750"/>
+                <a:pt x="3995738" y="2228850"/>
               </a:lnTo>
               <a:lnTo>
-                <a:pt x="4181475" y="2825750"/>
+                <a:pt x="4181475" y="2228850"/>
               </a:lnTo>
             </a:path>
           </a:pathLst>
@@ -12527,7 +12185,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="10106025" y="3048000"/>
-          <a:ext cx="371475" cy="3908425"/>
+          <a:ext cx="371475" cy="3311525"/>
         </a:xfrm>
         <a:custGeom>
           <a:avLst/>
@@ -12536,7 +12194,7 @@
           <a:cxnLst/>
           <a:rect l="0" t="0" r="r" b="b"/>
           <a:pathLst>
-            <a:path w="371475" h="3908425" fill="none">
+            <a:path w="371475" h="3311525" fill="none">
               <a:moveTo>
                 <a:pt x="0" y="0"/>
               </a:moveTo>
@@ -12544,10 +12202,10 @@
                 <a:pt x="209550" y="0"/>
               </a:lnTo>
               <a:lnTo>
-                <a:pt x="209550" y="3908425"/>
+                <a:pt x="209550" y="3311525"/>
               </a:lnTo>
               <a:lnTo>
-                <a:pt x="371475" y="3908425"/>
+                <a:pt x="371475" y="3311525"/>
               </a:lnTo>
             </a:path>
           </a:pathLst>
@@ -12583,7 +12241,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13916025" y="5826125"/>
+          <a:off x="13916025" y="5229225"/>
           <a:ext cx="371475" cy="47625"/>
         </a:xfrm>
         <a:custGeom>
@@ -12666,7 +12324,6 @@
             <a:srgbClr val="2E75B6"/>
           </a:solidFill>
           <a:prstDash val="dash"/>
-          <a:headEnd type="triangle" w="sm" len="sm"/>
           <a:tailEnd type="triangle" w="sm" len="sm"/>
         </a:ln>
       </xdr:spPr>
@@ -12719,7 +12376,6 @@
             <a:srgbClr val="2E75B6"/>
           </a:solidFill>
           <a:prstDash val="dash"/>
-          <a:headEnd type="triangle" w="sm" len="sm"/>
           <a:tailEnd type="triangle" w="sm" len="sm"/>
         </a:ln>
       </xdr:spPr>
@@ -12772,7 +12428,6 @@
             <a:srgbClr val="2E75B6"/>
           </a:solidFill>
           <a:prstDash val="dash"/>
-          <a:headEnd type="triangle" w="sm" len="sm"/>
           <a:tailEnd type="triangle" w="sm" len="sm"/>
         </a:ln>
       </xdr:spPr>
@@ -12784,7 +12439,7 @@
       <xdr:col>13</xdr:col>
       <xdr:colOff>1130617</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>1466850</xdr:rowOff>
+      <xdr:rowOff>869949</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>13</xdr:col>
@@ -12799,7 +12454,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="11550968" y="5149850"/>
+          <a:off x="11550968" y="4552950"/>
           <a:ext cx="9525" cy="1457325"/>
         </a:xfrm>
         <a:custGeom>
@@ -12825,7 +12480,7 @@
             <a:srgbClr val="2E75B6"/>
           </a:solidFill>
           <a:prstDash val="dash"/>
-          <a:headEnd type="triangle" w="sm" len="sm"/>
+          <a:tailEnd type="triangle" w="sm" len="sm"/>
         </a:ln>
       </xdr:spPr>
     </xdr:sp>
@@ -12836,7 +12491,7 @@
       <xdr:col>15</xdr:col>
       <xdr:colOff>1130617</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>1466850</xdr:rowOff>
+      <xdr:rowOff>869949</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>15</xdr:col>
@@ -12851,7 +12506,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13455968" y="5149850"/>
+          <a:off x="13455968" y="4552950"/>
           <a:ext cx="9525" cy="352425"/>
         </a:xfrm>
         <a:custGeom>
@@ -12877,7 +12532,7 @@
             <a:srgbClr val="2E75B6"/>
           </a:solidFill>
           <a:prstDash val="dash"/>
-          <a:headEnd type="triangle" w="sm" len="sm"/>
+          <a:tailEnd type="triangle" w="sm" len="sm"/>
         </a:ln>
       </xdr:spPr>
     </xdr:sp>
@@ -14019,7 +13674,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="10477500" y="6607175"/>
+          <a:off x="10477500" y="6010275"/>
           <a:ext cx="1533525" cy="603250"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -14089,7 +13744,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm rot="10800000">
-          <a:off x="11906250" y="6607175"/>
+          <a:off x="11906250" y="6010275"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="rtTriangle">
@@ -14125,7 +13780,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="10448925" y="6540500"/>
+          <a:off x="10448925" y="5943600"/>
           <a:ext cx="247650" cy="114300"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -14182,7 +13837,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="11706225" y="6540500"/>
+          <a:off x="11706225" y="5943600"/>
           <a:ext cx="295275" cy="114300"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -14237,7 +13892,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="12382500" y="5502275"/>
+          <a:off x="12382500" y="4905375"/>
           <a:ext cx="1533525" cy="742950"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -14307,7 +13962,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm rot="10800000">
-          <a:off x="13811250" y="5502275"/>
+          <a:off x="13811250" y="4905375"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="rtTriangle">
@@ -14343,7 +13998,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="12353925" y="5435600"/>
+          <a:off x="12353925" y="4838700"/>
           <a:ext cx="247650" cy="114300"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -14400,7 +14055,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13611225" y="5435600"/>
+          <a:off x="13611225" y="4838700"/>
           <a:ext cx="295275" cy="114300"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -14455,7 +14110,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14287500" y="5502275"/>
+          <a:off x="14287500" y="4905375"/>
           <a:ext cx="1533525" cy="742950"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -14526,7 +14181,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm rot="10800000">
-          <a:off x="15716250" y="5502275"/>
+          <a:off x="15716250" y="4905375"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="rtTriangle">
@@ -14562,7 +14217,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14258925" y="5435600"/>
+          <a:off x="14258925" y="4838700"/>
           <a:ext cx="247650" cy="114300"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -14610,7 +14265,7 @@
       <xdr:col>7</xdr:col>
       <xdr:colOff>1609725</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>1466850</xdr:rowOff>
+      <xdr:rowOff>869949</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -14620,7 +14275,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="4743450" y="3702050"/>
-          <a:ext cx="1571625" cy="1447800"/>
+          <a:ext cx="1571625" cy="850900"/>
         </a:xfrm>
         <a:prstGeom prst="can">
           <a:avLst/>
@@ -14640,42 +14295,16 @@
         </a:bodyPr>
         <a:lstStyle/>
         <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="7B3F00"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>W: TB_R_H0253_ORDER_CONTROL_PRE (NSP)</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="7B3F00"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>W: Log</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
               <a:solidFill>
                 <a:srgbClr val="1F3864"/>
               </a:solidFill>
               <a:latin typeface="Arial"/>
               <a:cs typeface="Arial"/>
             </a:rPr>
-            <a:t>R: TB_R_H0253_ORDER_CONTROL_PRE (DB Surrounding)</a:t>
+            <a:t>TB_R_H0253_ORDER_CONTROL_PRE</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -14693,7 +14322,7 @@
       <xdr:col>9</xdr:col>
       <xdr:colOff>1609725</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>1466850</xdr:rowOff>
+      <xdr:rowOff>869949</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -14703,7 +14332,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="6648450" y="3702050"/>
-          <a:ext cx="1571625" cy="1447800"/>
+          <a:ext cx="1571625" cy="850900"/>
         </a:xfrm>
         <a:prstGeom prst="can">
           <a:avLst/>
@@ -14723,94 +14352,55 @@
         </a:bodyPr>
         <a:lstStyle/>
         <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="7B3F00"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>W: TB_R_INSTRUCTION (delete rows without ASN_NO)</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="7B3F00"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>W: TB_R_PRA_DAILY_ORDER_MAPPED (MAPPED_QTY −)</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="7B3F00"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>W: TB_R_H0253_ORDER_CONTROL_PRE (PO_MAPPED_FLAG N, CANCEL_STATUS D)</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="7B3F00"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>W: TB_R_CROSSDOCK_CANCEL_RESULT</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="7B3F00"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>W: Log</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
               <a:solidFill>
                 <a:srgbClr val="1F3864"/>
               </a:solidFill>
               <a:latin typeface="Arial"/>
               <a:cs typeface="Arial"/>
             </a:rPr>
-            <a:t>R: TB_R_H0253_ORDER_CONTROL_PRE (NSP)</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
+            <a:t>TB_R_INSTRUCTION</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
               <a:solidFill>
                 <a:srgbClr val="1F3864"/>
               </a:solidFill>
               <a:latin typeface="Arial"/>
               <a:cs typeface="Arial"/>
             </a:rPr>
-            <a:t>R: TB_R_INSTRUCTION</a:t>
+            <a:t>TB_R_PRA_DAILY_ORDER_MAPPED</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
+              <a:solidFill>
+                <a:srgbClr val="1F3864"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:rPr>
+            <a:t>TB_R_H0253_ORDER_CONTROL_PRE</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
+              <a:solidFill>
+                <a:srgbClr val="1F3864"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:rPr>
+            <a:t>TB_R_CROSSDOCK_CANCEL_RESULT</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -14828,7 +14418,7 @@
       <xdr:col>11</xdr:col>
       <xdr:colOff>1609725</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>1466850</xdr:rowOff>
+      <xdr:rowOff>869949</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -14838,7 +14428,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="8553450" y="3702050"/>
-          <a:ext cx="1571625" cy="1447800"/>
+          <a:ext cx="1571625" cy="850900"/>
         </a:xfrm>
         <a:prstGeom prst="can">
           <a:avLst/>
@@ -14858,42 +14448,16 @@
         </a:bodyPr>
         <a:lstStyle/>
         <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="7B3F00"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>W: TB_R_H0253_ORDER_CONTROL_PRE (NSP)</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="7B3F00"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>W: Log</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
               <a:solidFill>
                 <a:srgbClr val="1F3864"/>
               </a:solidFill>
               <a:latin typeface="Arial"/>
               <a:cs typeface="Arial"/>
             </a:rPr>
-            <a:t>R: TB_R_H0253_ORDER_CONTROL_PRE (DB Surrounding)</a:t>
+            <a:t>TB_R_H0253_ORDER_CONTROL_PRE</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -14911,7 +14475,7 @@
       <xdr:col>13</xdr:col>
       <xdr:colOff>1609725</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>1466850</xdr:rowOff>
+      <xdr:rowOff>869949</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -14921,7 +14485,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="10458450" y="3702050"/>
-          <a:ext cx="1571625" cy="1447800"/>
+          <a:ext cx="1571625" cy="850900"/>
         </a:xfrm>
         <a:prstGeom prst="can">
           <a:avLst/>
@@ -14941,16 +14505,16 @@
         </a:bodyPr>
         <a:lstStyle/>
         <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
               <a:solidFill>
                 <a:srgbClr val="1F3864"/>
               </a:solidFill>
               <a:latin typeface="Arial"/>
               <a:cs typeface="Arial"/>
             </a:rPr>
-            <a:t>R: #TEMP_INSTRUCTION</a:t>
+            <a:t>#TEMP_INSTRUCTION</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -14968,7 +14532,7 @@
       <xdr:col>15</xdr:col>
       <xdr:colOff>1609725</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>1466850</xdr:rowOff>
+      <xdr:rowOff>869949</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -14978,7 +14542,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="12363450" y="3702050"/>
-          <a:ext cx="1571625" cy="1447800"/>
+          <a:ext cx="1571625" cy="850900"/>
         </a:xfrm>
         <a:prstGeom prst="can">
           <a:avLst/>
@@ -14998,29 +14562,16 @@
         </a:bodyPr>
         <a:lstStyle/>
         <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="0" dirty="0">
               <a:solidFill>
                 <a:srgbClr val="1F3864"/>
               </a:solidFill>
               <a:latin typeface="Arial"/>
               <a:cs typeface="Arial"/>
             </a:rPr>
-            <a:t>R: Log</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="600" b="0" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="1F3864"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>R: TB_R_CROSSDOCK_CANCEL_RESULT</a:t>
+            <a:t>TB_R_CROSSDOCK_CANCEL_RESULT</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -15047,7 +14598,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1187450" y="7512050"/>
+          <a:off x="1187450" y="6915150"/>
           <a:ext cx="666750" cy="247650"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -15104,7 +14655,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm rot="10800000">
-          <a:off x="1749425" y="7512050"/>
+          <a:off x="1749425" y="6915150"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="rtTriangle">
@@ -15140,7 +14691,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="676275" y="7896225"/>
+          <a:off x="676275" y="7299325"/>
           <a:ext cx="1689100" cy="152400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -15193,7 +14744,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2876550" y="7512050"/>
+          <a:off x="2876550" y="6915150"/>
           <a:ext cx="666750" cy="247650"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -15250,7 +14801,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm rot="10800000">
-          <a:off x="3438525" y="7512050"/>
+          <a:off x="3438525" y="6915150"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="rtTriangle">
@@ -15286,7 +14837,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2365375" y="7896225"/>
+          <a:off x="2365375" y="7299325"/>
           <a:ext cx="1689100" cy="152400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -15339,7 +14890,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4565650" y="7512050"/>
+          <a:off x="4565650" y="6915150"/>
           <a:ext cx="666750" cy="247650"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -15396,7 +14947,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm rot="10800000">
-          <a:off x="5127625" y="7512050"/>
+          <a:off x="5127625" y="6915150"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="rtTriangle">
@@ -15432,7 +14983,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4054475" y="7896225"/>
+          <a:off x="4054475" y="7299325"/>
           <a:ext cx="1689100" cy="152400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -15485,7 +15036,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6254750" y="7512050"/>
+          <a:off x="6254750" y="6915150"/>
           <a:ext cx="666750" cy="247650"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -15543,7 +15094,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm rot="10800000">
-          <a:off x="6816725" y="7512050"/>
+          <a:off x="6816725" y="6915150"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="rtTriangle">
@@ -15579,7 +15130,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5743575" y="7896225"/>
+          <a:off x="5743575" y="7299325"/>
           <a:ext cx="1689100" cy="152400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -15632,7 +15183,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7943850" y="7493000"/>
+          <a:off x="7943850" y="6896100"/>
           <a:ext cx="666750" cy="285750"/>
         </a:xfrm>
         <a:prstGeom prst="can">
@@ -15689,7 +15240,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7432675" y="7896225"/>
+          <a:off x="7432675" y="7299325"/>
           <a:ext cx="1689100" cy="152400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -15742,7 +15293,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9842500" y="7578725"/>
+          <a:off x="9842500" y="6981825"/>
           <a:ext cx="247650" cy="114300"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -15799,7 +15350,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9121775" y="7896225"/>
+          <a:off x="9121775" y="7299325"/>
           <a:ext cx="1689100" cy="152400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -15852,7 +15403,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="11512550" y="7578725"/>
+          <a:off x="11512550" y="6981825"/>
           <a:ext cx="295275" cy="114300"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -15907,7 +15458,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="10810875" y="7896225"/>
+          <a:off x="10810875" y="7299325"/>
           <a:ext cx="1689100" cy="152400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -15960,7 +15511,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13011150" y="7635875"/>
+          <a:off x="13011150" y="7038975"/>
           <a:ext cx="666750" cy="9525"/>
         </a:xfrm>
         <a:custGeom>
@@ -16011,7 +15562,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="12499975" y="7896225"/>
+          <a:off x="12499975" y="7299325"/>
           <a:ext cx="1689100" cy="152400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -16059,12 +15610,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="70" name="legend Data flow (W / R)"/>
+        <xdr:cNvPr id="70" name="legend Data flow"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14700250" y="7635875"/>
+          <a:off x="14700250" y="7038975"/>
           <a:ext cx="666750" cy="9525"/>
         </a:xfrm>
         <a:custGeom>
@@ -16111,12 +15662,12 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="71" name="legend caption Data flow (W / R)"/>
+        <xdr:cNvPr id="71" name="legend caption Data flow"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14189075" y="7896225"/>
+          <a:off x="14189075" y="7299325"/>
           <a:ext cx="1689100" cy="152400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -16142,7 +15693,7 @@
               <a:latin typeface="Arial"/>
               <a:cs typeface="Arial"/>
             </a:rPr>
-            <a:t>Data flow (W / R)</a:t>
+            <a:t>Data flow</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -17594,7 +17145,7 @@
       <c r="V14" s="47" t="n"/>
       <c r="W14" s="48" t="n"/>
     </row>
-    <row r="15" ht="79" customHeight="1">
+    <row r="15" ht="80" customHeight="1">
       <c r="A15" s="36" t="n"/>
       <c r="B15" s="37" t="n"/>
       <c r="C15" s="37" t="n"/>
@@ -18486,7 +18037,7 @@
       <c r="V14" s="47" t="n"/>
       <c r="W14" s="48" t="n"/>
     </row>
-    <row r="15" ht="88.5" customHeight="1">
+    <row r="15" ht="70" customHeight="1">
       <c r="A15" s="36" t="n"/>
       <c r="B15" s="37" t="n"/>
       <c r="C15" s="37" t="n"/>
@@ -19237,7 +18788,7 @@
       <c r="R14" s="47" t="n"/>
       <c r="S14" s="48" t="n"/>
     </row>
-    <row r="15" ht="117" customHeight="1">
+    <row r="15" ht="70" customHeight="1">
       <c r="A15" s="36" t="n"/>
       <c r="B15" s="37" t="n"/>
       <c r="C15" s="37" t="n"/>

</xml_diff>

<commit_message>
Existing table structures (GTOPAS SPS DB): ASN submit, case label last sequence, part master
UISS XD10 / XD15 use TB_R_DAILY_ORDER_MANIFEST / PART as in the DB structure, TB_R_CASE_LABEL_LAST_SEQ
for the last sequence and TB_M_PART_MASTER for the part name; ERD updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QL8Do8Pd2rXEDNa1ifG2RK
</commit_message>
<xml_diff>
--- a/deliverables/function_list_v2/bpf/Crossdock_BPF_Level2.xlsx
+++ b/deliverables/function_list_v2/bpf/Crossdock_BPF_Level2.xlsx
@@ -22657,7 +22657,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="60" customHeight="1">
+    <row r="26" ht="84" customHeight="1">
       <c r="A26" s="142" t="inlineStr">
         <is>
           <t>D10</t>
@@ -22691,13 +22691,16 @@
       <c r="G26" s="141" t="inlineStr">
         <is>
           <t>TB_R_INSTRUCTION
-Existing last sequence table</t>
+TB_R_PRA_DAILY_ORDER_MANIFEST
+TB_R_PRA_DAILY_ORDER_PART
+TB_M_PART_MASTER (PART_NAME)</t>
         </is>
       </c>
       <c r="H26" s="141" t="inlineStr">
         <is>
           <t>TB_R_DAILY_ORDER_MANIFEST
 TB_R_DAILY_ORDER_PART
+TB_R_CASE_LABEL_LAST_SEQ
 TB_R_INSTRUCTION (ASN_NO, CASE_NO)
 Log</t>
         </is>

</xml_diff>

<commit_message>
XD09 / XD10: receiving scan order, supplier cases and ASN option blocks (21-Oct)
- XD09 pre-maps the open qty of the H0253 lines in the G-System allocation order per
  Part No + Customer Order Date, cuts supplier cases of PCS_CASE pcs and groups them into
  blocks at valid cuts (every destination a multiple of PCS_CASE); block status Ready only
  when all earlier blocks have a PO. New temp table columns, new sample input.
- XD10: ASN Option per unit (first n Ready blocks), Partially Ready status, case sequence
  from XD09, PO_MAPPED_FLAG Y only for complete lines.
- ERD: SIM-2/3/4 recomputed with scan_pack, new SIM-7 (two ASNs); DB Structure and BPF texts.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QL8Do8Pd2rXEDNa1ifG2RK
</commit_message>
<xml_diff>
--- a/deliverables/function_list_v2/bpf/Crossdock_BPF_Level2.xlsx
+++ b/deliverables/function_list_v2/bpf/Crossdock_BPF_Level2.xlsx
@@ -22443,7 +22443,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="84" customHeight="1">
+    <row r="22" ht="96" customHeight="1">
       <c r="A22" s="142" t="inlineStr">
         <is>
           <t>D6</t>
@@ -22471,12 +22471,13 @@
       </c>
       <c r="F22" s="141" t="inlineStr">
         <is>
-          <t>Pre-map order lines to PO (FIFO); Case Qty, PO Readiness, Ready / Not Ready</t>
+          <t>Pre-map in scan order; supplier cases, blocks (ASN options), Ready / Not Ready</t>
         </is>
       </c>
       <c r="G22" s="141" t="inlineStr">
         <is>
-          <t>TB_R_H0253_ORDER_CONTROL_PRE (status 7, HOLD N, PO_MAPPED N)
+          <t>TB_R_H0253_ORDER_CONTROL_PRE (status 7, HOLD N, open qty)
+TB_R_INSTRUCTION
 TB_R_PRA_DAILY_ORDER_MANIFEST
 TB_R_PRA_DAILY_ORDER_PART
 TB_R_PRA_DAILY_ORDER_MAPPED</t>
@@ -22498,7 +22499,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="15" customHeight="1">
+    <row r="23" ht="24" customHeight="1">
       <c r="A23" s="150" t="inlineStr">
         <is>
           <t>D7</t>
@@ -22526,7 +22527,7 @@
       </c>
       <c r="F23" s="141" t="inlineStr">
         <is>
-          <t>Select Ready units, [Create ASN]</t>
+          <t>Tick units, choose ASN option (first n Ready blocks), [Create ASN]</t>
         </is>
       </c>
       <c r="G23" s="141" t="inlineStr">
@@ -22578,7 +22579,7 @@
       </c>
       <c r="F24" s="141" t="inlineStr">
         <is>
-          <t>Lock + re-check; pack cases per destination by pcs/case; real mapping</t>
+          <t>Lock + re-check; insert the chosen blocks (cases of XD09); real mapping</t>
         </is>
       </c>
       <c r="G24" s="141" t="inlineStr">
@@ -23938,7 +23939,7 @@
       </c>
       <c r="D14" s="163" t="inlineStr">
         <is>
-          <t>Choose Delivery Date and Rit, click [Search]: units Ready / Not Ready.</t>
+          <t>Choose Delivery Date and Rit, click [Search]: units Ready / Partially Ready / Not Ready.</t>
         </is>
       </c>
       <c r="E14" s="163" t="inlineStr">
@@ -23954,7 +23955,7 @@
       </c>
       <c r="H14" s="163" t="inlineStr">
         <is>
-          <t>AB08: unit Not Ready, wait for the next PO.</t>
+          <t>AB08: block without PO, send the Ready blocks or wait.</t>
         </is>
       </c>
       <c r="I14" s="163" t="inlineStr">
@@ -23981,7 +23982,7 @@
       </c>
       <c r="D15" s="163" t="inlineStr">
         <is>
-          <t>Tick Ready units of one supplier + plant and click [Create ASN].</t>
+          <t>Tick units of one supplier + plant, choose the ASN option (first n Ready blocks) and click [Create ASN].</t>
         </is>
       </c>
       <c r="E15" s="163" t="inlineStr">
@@ -23992,7 +23993,7 @@
       <c r="F15" s="163" t="inlineStr"/>
       <c r="G15" s="163" t="inlineStr">
         <is>
-          <t>TB_R_INSTRUCTION, PO_MAPPED_FLAG Y, MAPPED_QTY</t>
+          <t>TB_R_INSTRUCTION, PO_MAPPED_FLAG Y (whole line), MAPPED_QTY</t>
         </is>
       </c>
       <c r="H15" s="163" t="inlineStr">
@@ -24024,7 +24025,7 @@
       </c>
       <c r="D16" s="163" t="inlineStr">
         <is>
-          <t>Check the Case List (cases of pcs/case per destination) and click [Submit ASN].</t>
+          <t>Check the Case List (supplier cases of pcs/case in scan order) and click [Submit ASN].</t>
         </is>
       </c>
       <c r="E16" s="163" t="inlineStr">
@@ -24600,7 +24601,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="24" customHeight="1">
+    <row r="12" ht="36" customHeight="1">
       <c r="A12" s="168" t="inlineStr">
         <is>
           <t>AB08</t>
@@ -24623,17 +24624,17 @@
       </c>
       <c r="E12" s="141" t="inlineStr">
         <is>
-          <t>Unit Not Ready: a case of the unit has no PO yet</t>
+          <t>Block without PO: the block and every later block are Not Ready</t>
         </is>
       </c>
       <c r="F12" s="141" t="inlineStr">
         <is>
-          <t>Check box disabled, tooltip MSG2</t>
+          <t>Partially Ready (later block) / check box disabled + MSG2 (first block)</t>
         </is>
       </c>
       <c r="G12" s="141" t="inlineStr">
         <is>
-          <t>Unit is not selectable (the unit stays whole, decided A2).</t>
+          <t>Only the Ready blocks before it can be sent; blocks are never skipped (scan order, decided 21-Oct).</t>
         </is>
       </c>
       <c r="H12" s="141" t="inlineStr">
@@ -24643,7 +24644,7 @@
       </c>
       <c r="I12" s="141" t="inlineStr">
         <is>
-          <t>Wait for the next PO; the unit becomes Ready on a later [Search].</t>
+          <t>Send the Ready blocks or wait for the next PO; the block becomes Ready on a later [Search].</t>
         </is>
       </c>
     </row>
@@ -24717,7 +24718,7 @@
       </c>
       <c r="E14" s="141" t="inlineStr">
         <is>
-          <t>A ticked unit is no longer Ready (PO or order changed)</t>
+          <t>A chosen block is no longer Ready (PO or order changed)</t>
         </is>
       </c>
       <c r="F14" s="141" t="inlineStr">

</xml_diff>

<commit_message>
H0253 replicate: rename CANCEL_STATUS to UPD_STATUS (step 1, name only)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QL8Do8Pd2rXEDNa1ifG2RK
</commit_message>
<xml_diff>
--- a/deliverables/function_list_v2/bpf/Crossdock_BPF_Level2.xlsx
+++ b/deliverables/function_list_v2/bpf/Crossdock_BPF_Level2.xlsx
@@ -15170,7 +15170,7 @@
               <a:latin typeface="Arial"/>
               <a:cs typeface="Arial"/>
             </a:rPr>
-            <a:t>Upsert status 2 rows of crossdock lines + other changed rows of the line; CANCEL_STATUS P</a:t>
+            <a:t>Upsert status 2 rows of crossdock lines + other changed rows of the line; UPD_STATUS P</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -23187,7 +23187,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="48" customHeight="1">
+    <row r="36" ht="36" customHeight="1">
       <c r="A36" s="142" t="inlineStr">
         <is>
           <t>C3</t>
@@ -23215,7 +23215,7 @@
       </c>
       <c r="F36" s="141" t="inlineStr">
         <is>
-          <t>Upsert status 2 rows of crossdock lines + other changed rows of the line; CANCEL_STATUS P</t>
+          <t>Upsert status 2 rows of crossdock lines + other changed rows of the line; UPD_STATUS P</t>
         </is>
       </c>
       <c r="G36" s="141" t="inlineStr">
@@ -23281,7 +23281,7 @@
         <is>
           <t>TB_R_INSTRUCTION (delete rows without ASN_NO)
 TB_R_PRA_DAILY_ORDER_MAPPED (MAPPED_QTY −)
-TB_R_H0253_ORDER_CONTROL_PRE (PO_MAPPED_FLAG N, CANCEL_STATUS D)
+TB_R_H0253_ORDER_CONTROL_PRE (PO_MAPPED_FLAG N, UPD_STATUS D)
 TB_R_CROSSDOCK_CANCEL_RESULT
 Log</t>
         </is>

</xml_diff>

<commit_message>
Documents updated to the latest business logic and reviewed
- BPF: PO rule on D2 (1 PO per Part + order date, PO date + 1), receiving step D14 (partial
  receipt splits the serial), XD08 serial split on D3, D7 / U9 oldest order date first and
  cut, D8 PO_MAPPED_FLAG rule; AB08 extended; new AB17 Short PO, AB18 receiving order (TBC),
  AB19 / AB20 open decisions (open PO qty of cancelled orders, XD11 without candidate).
  Diagram shots F1 / F2 / F4 (F3 did not exist any more).
- UISS XD10 Sample Input A-G = Create ASN 18-Oct of simulasi_asn_rev (ASN0003); H-I kept as
  the example of cases that belong together.
- md XD09 / XD10: Business Logic ASN; README: superseded XD12 notes marked; ERD README and
  example ASN number.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QL8Do8Pd2rXEDNa1ifG2RK
</commit_message>
<xml_diff>
--- a/deliverables/function_list_v2/bpf/Crossdock_BPF_Level2.xlsx
+++ b/deliverables/function_list_v2/bpf/Crossdock_BPF_Level2.xlsx
@@ -21609,7 +21609,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J41"/>
+  <dimension ref="A1:J42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -22399,7 +22399,7 @@
       </c>
       <c r="C18" s="140" t="inlineStr">
         <is>
-          <t>D-1 · during the day</t>
+          <t>D-1 · customer order / D · PO (existing)</t>
         </is>
       </c>
       <c r="D18" s="141" t="inlineStr">
@@ -22438,7 +22438,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="36" customHeight="1">
+    <row r="19" ht="60" customHeight="1">
       <c r="A19" s="142" t="inlineStr">
         <is>
           <t>D2</t>
@@ -22451,7 +22451,7 @@
       </c>
       <c r="C19" s="143" t="inlineStr">
         <is>
-          <t>D-1 · during the day</t>
+          <t>D-1 · customer order / D · PO (existing)</t>
         </is>
       </c>
       <c r="D19" s="141" t="inlineStr">
@@ -22466,7 +22466,7 @@
       </c>
       <c r="F19" s="141" t="inlineStr">
         <is>
-          <t>Release PO Supplier (manifest CROSS_DOCK_FLAG X, parts in Pra Daily Order Part)</t>
+          <t>Release PO Supplier: one PO per Part per Customer Order Date, PO date = order date + 1, qty = total order qty of all destinations (CROSS_DOCK_FLAG X)</t>
         </is>
       </c>
       <c r="G19" s="141" t="inlineStr">
@@ -22487,11 +22487,11 @@
       </c>
       <c r="J19" s="141" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>AB17</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="36" customHeight="1">
+    <row r="20" ht="60" customHeight="1">
       <c r="A20" s="142" t="inlineStr">
         <is>
           <t>D3</t>
@@ -22519,7 +22519,7 @@
       </c>
       <c r="F20" s="141" t="inlineStr">
         <is>
-          <t>Upsert changed rows (delta INTF_UPDATE_DT); UPD_STATUS 6 / 2; release all drafts</t>
+          <t>Upsert changed rows (delta INTF_UPDATE_DT); UPD_STATUS 6 / 2; serial split: each part stays linked to its ASN; release all drafts</t>
         </is>
       </c>
       <c r="G20" s="141" t="inlineStr">
@@ -22530,6 +22530,7 @@
       <c r="H20" s="141" t="inlineStr">
         <is>
           <t>TB_R_H0253_ORDER_CONTROL_PRE (NSP)
+TB_R_INSTRUCTION (SERIAL_NO)
 Log</t>
         </is>
       </c>
@@ -22540,7 +22541,7 @@
       </c>
       <c r="J20" s="141" t="inlineStr">
         <is>
-          <t>AB07</t>
+          <t>AB07, AB18</t>
         </is>
       </c>
     </row>
@@ -22652,7 +22653,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="24" customHeight="1">
+    <row r="23" ht="36" customHeight="1">
       <c r="A23" s="150" t="inlineStr">
         <is>
           <t>D7</t>
@@ -22680,7 +22681,7 @@
       </c>
       <c r="F23" s="141" t="inlineStr">
         <is>
-          <t>Tick units, choose ASN option (first n Ready blocks), [Create ASN]</t>
+          <t>Tick cases: per part the oldest Customer Order Date first; from case 1 up to a cut (CUT_FLAG); [Create ASN]</t>
         </is>
       </c>
       <c r="G23" s="141" t="inlineStr">
@@ -22732,7 +22733,7 @@
       </c>
       <c r="F24" s="141" t="inlineStr">
         <is>
-          <t>Lock + re-check; insert the chosen blocks (cases of XD09); real mapping</t>
+          <t>Lock + re-check; insert the ticked cases (XD09); real mapping; PO_MAPPED_FLAG Y when the whole line is in the ASN</t>
         </is>
       </c>
       <c r="G24" s="141" t="inlineStr">
@@ -22883,7 +22884,7 @@
       </c>
       <c r="C27" s="140" t="inlineStr">
         <is>
-          <t>Day D · after submit</t>
+          <t>Day D · after submit / receiving</t>
         </is>
       </c>
       <c r="D27" s="141" t="inlineStr">
@@ -22935,7 +22936,7 @@
       </c>
       <c r="C28" s="151" t="inlineStr">
         <is>
-          <t>Day D · after submit</t>
+          <t>Day D · after submit / receiving</t>
         </is>
       </c>
       <c r="D28" s="141" t="inlineStr">
@@ -22975,45 +22976,45 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="24" customHeight="1">
-      <c r="A29" s="150" t="inlineStr">
-        <is>
-          <t>D13</t>
-        </is>
-      </c>
-      <c r="B29" s="151" t="inlineStr">
+    <row r="29" ht="36" customHeight="1">
+      <c r="A29" s="139" t="inlineStr">
+        <is>
+          <t>D14</t>
+        </is>
+      </c>
+      <c r="B29" s="140" t="inlineStr">
         <is>
           <t>F2</t>
         </is>
       </c>
-      <c r="C29" s="151" t="inlineStr">
-        <is>
-          <t>Day D · after submit</t>
+      <c r="C29" s="140" t="inlineStr">
+        <is>
+          <t>Day D · after submit / receiving</t>
         </is>
       </c>
       <c r="D29" s="141" t="inlineStr">
         <is>
-          <t>Supplier</t>
+          <t>G-System / DB Surrounding</t>
         </is>
       </c>
       <c r="E29" s="141" t="inlineStr">
         <is>
-          <t>Log Monitoring</t>
+          <t>existing</t>
         </is>
       </c>
       <c r="F29" s="141" t="inlineStr">
         <is>
-          <t>Check the submit result per Submit ID</t>
+          <t>Receive the ASN in scan order → ORDER_STATUS 6; a partial receipt splits the line (new SERIAL_NO); taken by the next XD08 run (D3)</t>
         </is>
       </c>
       <c r="G29" s="141" t="inlineStr">
         <is>
-          <t>Log</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H29" s="141" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>TB_R_H0253_ORDER_CONTROL_PRE (DB Surrounding, INTF_UPDATE_DT)</t>
         </is>
       </c>
       <c r="I29" s="141" t="inlineStr">
@@ -23023,44 +23024,44 @@
       </c>
       <c r="J29" s="141" t="inlineStr">
         <is>
-          <t>AB13</t>
+          <t>AB18</t>
         </is>
       </c>
     </row>
     <row r="30" ht="24" customHeight="1">
-      <c r="A30" s="146" t="inlineStr">
-        <is>
-          <t>H1</t>
-        </is>
-      </c>
-      <c r="B30" s="147" t="inlineStr">
-        <is>
-          <t>F4</t>
-        </is>
-      </c>
-      <c r="C30" s="147" t="inlineStr">
-        <is>
-          <t>Day D · working hours (hold)</t>
+      <c r="A30" s="150" t="inlineStr">
+        <is>
+          <t>D13</t>
+        </is>
+      </c>
+      <c r="B30" s="151" t="inlineStr">
+        <is>
+          <t>F2</t>
+        </is>
+      </c>
+      <c r="C30" s="151" t="inlineStr">
+        <is>
+          <t>Day D · after submit / receiving</t>
         </is>
       </c>
       <c r="D30" s="141" t="inlineStr">
         <is>
-          <t>D/S Team</t>
+          <t>Supplier</t>
         </is>
       </c>
       <c r="E30" s="141" t="inlineStr">
         <is>
-          <t>XD10</t>
+          <t>Log Monitoring</t>
         </is>
       </c>
       <c r="F30" s="141" t="inlineStr">
         <is>
-          <t>Monitor the destination detail of the delivery plan (View as D/S team)</t>
+          <t>Check the submit result per Submit ID</t>
         </is>
       </c>
       <c r="G30" s="141" t="inlineStr">
         <is>
-          <t>TB_R_H0253_ORDER_CONTROL_PRE</t>
+          <t>Log</t>
         </is>
       </c>
       <c r="H30" s="141" t="inlineStr">
@@ -23070,590 +23071,642 @@
       </c>
       <c r="I30" s="141" t="inlineStr">
         <is>
-          <t>H2</t>
+          <t>End</t>
         </is>
       </c>
       <c r="J30" s="141" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>AB13</t>
         </is>
       </c>
     </row>
     <row r="31" ht="24" customHeight="1">
       <c r="A31" s="146" t="inlineStr">
         <is>
+          <t>H1</t>
+        </is>
+      </c>
+      <c r="B31" s="147" t="inlineStr">
+        <is>
+          <t>F4</t>
+        </is>
+      </c>
+      <c r="C31" s="147" t="inlineStr">
+        <is>
+          <t>Day D · working hours (hold)</t>
+        </is>
+      </c>
+      <c r="D31" s="141" t="inlineStr">
+        <is>
+          <t>D/S Team</t>
+        </is>
+      </c>
+      <c r="E31" s="141" t="inlineStr">
+        <is>
+          <t>XD10</t>
+        </is>
+      </c>
+      <c r="F31" s="141" t="inlineStr">
+        <is>
+          <t>Monitor the destination detail of the delivery plan (View as D/S team)</t>
+        </is>
+      </c>
+      <c r="G31" s="141" t="inlineStr">
+        <is>
+          <t>TB_R_H0253_ORDER_CONTROL_PRE</t>
+        </is>
+      </c>
+      <c r="H31" s="141" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I31" s="141" t="inlineStr">
+        <is>
           <t>H2</t>
         </is>
       </c>
-      <c r="B31" s="147" t="inlineStr">
+      <c r="J31" s="141" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="24" customHeight="1">
+      <c r="A32" s="146" t="inlineStr">
+        <is>
+          <t>H2</t>
+        </is>
+      </c>
+      <c r="B32" s="147" t="inlineStr">
         <is>
           <t>F4</t>
         </is>
       </c>
-      <c r="C31" s="147" t="inlineStr">
+      <c r="C32" s="147" t="inlineStr">
         <is>
           <t>Day D · working hours (hold)</t>
         </is>
       </c>
-      <c r="D31" s="141" t="inlineStr">
+      <c r="D32" s="141" t="inlineStr">
         <is>
           <t>D/S Team</t>
         </is>
       </c>
-      <c r="E31" s="141" t="inlineStr">
+      <c r="E32" s="141" t="inlineStr">
         <is>
           <t>XD10</t>
         </is>
       </c>
-      <c r="F31" s="141" t="inlineStr">
+      <c r="F32" s="141" t="inlineStr">
         <is>
           <t>Hold / Release a destination (all its order lines)</t>
         </is>
       </c>
-      <c r="G31" s="141" t="inlineStr">
+      <c r="G32" s="141" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H31" s="141" t="inlineStr">
+      <c r="H32" s="141" t="inlineStr">
         <is>
           <t>TB_R_H0253_ORDER_CONTROL_PRE (HOLD_FLAG Y / N)</t>
         </is>
       </c>
-      <c r="I31" s="141" t="inlineStr">
+      <c r="I32" s="141" t="inlineStr">
         <is>
           <t>H3</t>
         </is>
       </c>
-      <c r="J31" s="141" t="inlineStr">
+      <c r="J32" s="141" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="36" customHeight="1">
-      <c r="A32" s="142" t="inlineStr">
+    <row r="33" ht="36" customHeight="1">
+      <c r="A33" s="142" t="inlineStr">
         <is>
           <t>H3</t>
         </is>
       </c>
-      <c r="B32" s="143" t="inlineStr">
+      <c r="B33" s="143" t="inlineStr">
         <is>
           <t>F4</t>
         </is>
       </c>
-      <c r="C32" s="143" t="inlineStr">
+      <c r="C33" s="143" t="inlineStr">
         <is>
           <t>Day D · working hours (hold)</t>
         </is>
       </c>
-      <c r="D32" s="141" t="inlineStr">
+      <c r="D33" s="141" t="inlineStr">
         <is>
           <t>NSP Batch (System)</t>
         </is>
       </c>
-      <c r="E32" s="141" t="inlineStr">
+      <c r="E33" s="141" t="inlineStr">
         <is>
           <t>XD09</t>
         </is>
       </c>
-      <c r="F32" s="141" t="inlineStr">
+      <c r="F33" s="141" t="inlineStr">
         <is>
           <t>[Search]: lines with HOLD_FLAG Y are not pre-mapped; the unit is computed without the held destination</t>
         </is>
       </c>
-      <c r="G32" s="141" t="inlineStr">
+      <c r="G33" s="141" t="inlineStr">
         <is>
           <t>TB_R_H0253_ORDER_CONTROL_PRE (HOLD N)</t>
         </is>
       </c>
-      <c r="H32" s="141" t="inlineStr">
+      <c r="H33" s="141" t="inlineStr">
         <is>
           <t>#TEMP_INSTRUCTION</t>
         </is>
       </c>
-      <c r="I32" s="141" t="inlineStr">
+      <c r="I33" s="141" t="inlineStr">
         <is>
           <t>H4</t>
         </is>
       </c>
-      <c r="J32" s="141" t="inlineStr">
+      <c r="J33" s="141" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="48" customHeight="1">
-      <c r="A33" s="150" t="inlineStr">
+    <row r="34" ht="48" customHeight="1">
+      <c r="A34" s="150" t="inlineStr">
         <is>
           <t>H4</t>
         </is>
       </c>
-      <c r="B33" s="151" t="inlineStr">
+      <c r="B34" s="151" t="inlineStr">
         <is>
           <t>F4</t>
         </is>
       </c>
-      <c r="C33" s="151" t="inlineStr">
+      <c r="C34" s="151" t="inlineStr">
         <is>
           <t>Day D · working hours (hold)</t>
         </is>
       </c>
-      <c r="D33" s="141" t="inlineStr">
+      <c r="D34" s="141" t="inlineStr">
         <is>
           <t>Supplier</t>
         </is>
       </c>
-      <c r="E33" s="141" t="inlineStr">
+      <c r="E34" s="141" t="inlineStr">
         <is>
           <t>XD10</t>
         </is>
       </c>
-      <c r="F33" s="141" t="inlineStr">
+      <c r="F34" s="141" t="inlineStr">
         <is>
           <t>[Create ASN] re-checks the hold: a line held after the tick → whole create fails, list refreshed</t>
         </is>
       </c>
-      <c r="G33" s="141" t="inlineStr">
+      <c r="G34" s="141" t="inlineStr">
         <is>
           <t>#TEMP_INSTRUCTION
 TB_R_H0253_ORDER_CONTROL_PRE</t>
         </is>
       </c>
-      <c r="H33" s="141" t="inlineStr">
+      <c r="H34" s="141" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I33" s="141" t="inlineStr">
+      <c r="I34" s="141" t="inlineStr">
         <is>
           <t>End</t>
         </is>
       </c>
-      <c r="J33" s="141" t="inlineStr">
+      <c r="J34" s="141" t="inlineStr">
         <is>
           <t>AB09</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="24" customHeight="1">
-      <c r="A34" s="139" t="inlineStr">
-        <is>
-          <t>C1</t>
-        </is>
-      </c>
-      <c r="B34" s="140" t="inlineStr">
-        <is>
-          <t>F4</t>
-        </is>
-      </c>
-      <c r="C34" s="140" t="inlineStr">
-        <is>
-          <t>Any time · G-System (cancel)</t>
-        </is>
-      </c>
-      <c r="D34" s="141" t="inlineStr">
-        <is>
-          <t>G-System / DB Surrounding</t>
-        </is>
-      </c>
-      <c r="E34" s="141" t="inlineStr">
-        <is>
-          <t>SOP</t>
-        </is>
-      </c>
-      <c r="F34" s="141" t="inlineStr">
-        <is>
-          <t>Check the ASN feedback: only qty not yet in an ASN may be cancelled</t>
-        </is>
-      </c>
-      <c r="G34" s="141" t="inlineStr">
-        <is>
-          <t>Existing ASN feedback</t>
-        </is>
-      </c>
-      <c r="H34" s="141" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I34" s="141" t="inlineStr">
-        <is>
-          <t>C2</t>
-        </is>
-      </c>
-      <c r="J34" s="141" t="inlineStr">
-        <is>
-          <t>-</t>
         </is>
       </c>
     </row>
     <row r="35" ht="24" customHeight="1">
       <c r="A35" s="139" t="inlineStr">
         <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="B35" s="140" t="inlineStr">
+        <is>
+          <t>F4</t>
+        </is>
+      </c>
+      <c r="C35" s="140" t="inlineStr">
+        <is>
+          <t>Any time · G-System (cancel)</t>
+        </is>
+      </c>
+      <c r="D35" s="141" t="inlineStr">
+        <is>
+          <t>G-System / DB Surrounding</t>
+        </is>
+      </c>
+      <c r="E35" s="141" t="inlineStr">
+        <is>
+          <t>SOP</t>
+        </is>
+      </c>
+      <c r="F35" s="141" t="inlineStr">
+        <is>
+          <t>Check the ASN feedback: only qty not yet in an ASN may be cancelled</t>
+        </is>
+      </c>
+      <c r="G35" s="141" t="inlineStr">
+        <is>
+          <t>Existing ASN feedback</t>
+        </is>
+      </c>
+      <c r="H35" s="141" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I35" s="141" t="inlineStr">
+        <is>
           <t>C2</t>
         </is>
       </c>
-      <c r="B35" s="140" t="inlineStr">
+      <c r="J35" s="141" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="24" customHeight="1">
+      <c r="A36" s="139" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="B36" s="140" t="inlineStr">
         <is>
           <t>F4</t>
         </is>
       </c>
-      <c r="C35" s="140" t="inlineStr">
+      <c r="C36" s="140" t="inlineStr">
         <is>
           <t>Any time · G-System (cancel)</t>
         </is>
       </c>
-      <c r="D35" s="141" t="inlineStr">
+      <c r="D36" s="141" t="inlineStr">
         <is>
           <t>G-System / DB Surrounding</t>
         </is>
       </c>
-      <c r="E35" s="141" t="inlineStr">
+      <c r="E36" s="141" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F35" s="141" t="inlineStr">
+      <c r="F36" s="141" t="inlineStr">
         <is>
           <t>Cancel (with or without HOLD_FLAG): ORDER_STATUS 2; partial cancel = new SERIAL_NO</t>
         </is>
       </c>
-      <c r="G35" s="141" t="inlineStr">
+      <c r="G36" s="141" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H35" s="141" t="inlineStr">
+      <c r="H36" s="141" t="inlineStr">
         <is>
           <t>TB_R_H0253_ORDER_CONTROL_PRE (DB Surrounding, INTF_UPDATE_DT)</t>
         </is>
       </c>
-      <c r="I35" s="141" t="inlineStr">
+      <c r="I36" s="141" t="inlineStr">
         <is>
           <t>C3</t>
         </is>
       </c>
-      <c r="J35" s="141" t="inlineStr">
+      <c r="J36" s="141" t="inlineStr">
         <is>
           <t>AB16</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="48" customHeight="1">
-      <c r="A36" s="142" t="inlineStr">
+    <row r="37" ht="48" customHeight="1">
+      <c r="A37" s="142" t="inlineStr">
         <is>
           <t>C3</t>
         </is>
       </c>
-      <c r="B36" s="143" t="inlineStr">
+      <c r="B37" s="143" t="inlineStr">
         <is>
           <t>F4</t>
         </is>
       </c>
-      <c r="C36" s="143" t="inlineStr">
+      <c r="C37" s="143" t="inlineStr">
         <is>
           <t>27:30 · XD08 (one H0253 batch)</t>
         </is>
       </c>
-      <c r="D36" s="141" t="inlineStr">
+      <c r="D37" s="141" t="inlineStr">
         <is>
           <t>NSP Batch (System)</t>
         </is>
       </c>
-      <c r="E36" s="141" t="inlineStr">
+      <c r="E37" s="141" t="inlineStr">
         <is>
           <t>XD08</t>
         </is>
       </c>
-      <c r="F36" s="141" t="inlineStr">
+      <c r="F37" s="141" t="inlineStr">
         <is>
           <t>Upsert the changed rows: UPD_STATUS 2 (cancel) / 6 (received); ORDER_STATUS keeps the first value</t>
         </is>
       </c>
-      <c r="G36" s="141" t="inlineStr">
+      <c r="G37" s="141" t="inlineStr">
         <is>
           <t>TB_R_H0253_ORDER_CONTROL_PRE (DB Surrounding)</t>
         </is>
       </c>
-      <c r="H36" s="141" t="inlineStr">
+      <c r="H37" s="141" t="inlineStr">
         <is>
           <t>TB_R_H0253_ORDER_CONTROL_PRE (NSP, UPD_STATUS)
 Log</t>
         </is>
       </c>
-      <c r="I36" s="141" t="inlineStr">
+      <c r="I37" s="141" t="inlineStr">
         <is>
           <t>C4</t>
         </is>
       </c>
-      <c r="J36" s="141" t="inlineStr">
+      <c r="J37" s="141" t="inlineStr">
         <is>
           <t>AB07</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="60" customHeight="1">
-      <c r="A37" s="142" t="inlineStr">
+    <row r="38" ht="60" customHeight="1">
+      <c r="A38" s="142" t="inlineStr">
         <is>
           <t>C4</t>
         </is>
       </c>
-      <c r="B37" s="143" t="inlineStr">
+      <c r="B38" s="143" t="inlineStr">
         <is>
           <t>F4</t>
         </is>
       </c>
-      <c r="C37" s="143" t="inlineStr">
+      <c r="C38" s="143" t="inlineStr">
         <is>
           <t>27:30 · XD08 (one H0253 batch)</t>
         </is>
       </c>
-      <c r="D37" s="141" t="inlineStr">
+      <c r="D38" s="141" t="inlineStr">
         <is>
           <t>NSP Batch (System)</t>
         </is>
       </c>
-      <c r="E37" s="141" t="inlineStr">
+      <c r="E38" s="141" t="inlineStr">
         <is>
           <t>XD08</t>
         </is>
       </c>
-      <c r="F37" s="141" t="inlineStr">
+      <c r="F38" s="141" t="inlineStr">
         <is>
           <t>Release all drafts (Create ASN not submitted); the cases come back in the delivery plan</t>
         </is>
       </c>
-      <c r="G37" s="141" t="inlineStr">
+      <c r="G38" s="141" t="inlineStr">
         <is>
           <t>TB_R_INSTRUCTION (ASN_NO NULL)</t>
         </is>
       </c>
-      <c r="H37" s="141" t="inlineStr">
+      <c r="H38" s="141" t="inlineStr">
         <is>
           <t>TB_R_INSTRUCTION (delete drafts)
 TB_R_PRA_DAILY_ORDER_MAPPED (MAPPED_QTY −)
 TB_R_H0253_ORDER_CONTROL_PRE (PO_MAPPED_FLAG N)</t>
         </is>
       </c>
-      <c r="I37" s="141" t="inlineStr">
+      <c r="I38" s="141" t="inlineStr">
         <is>
           <t>C5, C6</t>
         </is>
       </c>
-      <c r="J37" s="141" t="inlineStr">
+      <c r="J38" s="141" t="inlineStr">
         <is>
           <t>AB12</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="36" customHeight="1">
-      <c r="A38" s="142" t="inlineStr">
+    <row r="39" ht="36" customHeight="1">
+      <c r="A39" s="142" t="inlineStr">
         <is>
           <t>C5</t>
         </is>
       </c>
-      <c r="B38" s="143" t="inlineStr">
+      <c r="B39" s="143" t="inlineStr">
         <is>
           <t>F4</t>
         </is>
       </c>
-      <c r="C38" s="143" t="inlineStr">
+      <c r="C39" s="143" t="inlineStr">
         <is>
           <t>27:30 · XD08 (one H0253 batch)</t>
         </is>
       </c>
-      <c r="D38" s="141" t="inlineStr">
+      <c r="D39" s="141" t="inlineStr">
         <is>
           <t>NSP Batch (System)</t>
         </is>
       </c>
-      <c r="E38" s="141" t="inlineStr">
+      <c r="E39" s="141" t="inlineStr">
         <is>
           <t>XD08</t>
         </is>
       </c>
-      <c r="F38" s="141" t="inlineStr">
+      <c r="F39" s="141" t="inlineStr">
         <is>
           <t>Cancel of qty in a submitted ASN: LOG5, listed in Change Order Number (ASN not changed)</t>
         </is>
       </c>
-      <c r="G38" s="141" t="inlineStr">
+      <c r="G39" s="141" t="inlineStr">
         <is>
           <t>TB_R_H0253_ORDER_CONTROL_PRE (UPD_STATUS 2)
 TB_R_INSTRUCTION (ASN_NO)</t>
         </is>
       </c>
-      <c r="H38" s="141" t="inlineStr">
+      <c r="H39" s="141" t="inlineStr">
         <is>
           <t>Log</t>
         </is>
       </c>
-      <c r="I38" s="141" t="inlineStr">
+      <c r="I39" s="141" t="inlineStr">
         <is>
           <t>C7</t>
         </is>
       </c>
-      <c r="J38" s="141" t="inlineStr">
+      <c r="J39" s="141" t="inlineStr">
         <is>
           <t>AB16</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="24" customHeight="1">
-      <c r="A39" s="150" t="inlineStr">
+    <row r="40" ht="24" customHeight="1">
+      <c r="A40" s="150" t="inlineStr">
         <is>
           <t>C6</t>
         </is>
       </c>
-      <c r="B39" s="151" t="inlineStr">
+      <c r="B40" s="151" t="inlineStr">
         <is>
           <t>F4</t>
         </is>
       </c>
-      <c r="C39" s="151" t="inlineStr">
+      <c r="C40" s="151" t="inlineStr">
         <is>
           <t>Day D · working hours</t>
         </is>
       </c>
-      <c r="D39" s="141" t="inlineStr">
+      <c r="D40" s="141" t="inlineStr">
         <is>
           <t>Supplier</t>
         </is>
       </c>
-      <c r="E39" s="141" t="inlineStr">
+      <c r="E40" s="141" t="inlineStr">
         <is>
           <t>XD10</t>
         </is>
       </c>
-      <c r="F39" s="141" t="inlineStr">
+      <c r="F40" s="141" t="inlineStr">
         <is>
           <t>[Search] again and tick the cases again; [Submit ASN] of an old draft fails (MSG11)</t>
         </is>
       </c>
-      <c r="G39" s="141" t="inlineStr">
+      <c r="G40" s="141" t="inlineStr">
         <is>
           <t>#TEMP_INSTRUCTION</t>
         </is>
       </c>
-      <c r="H39" s="141" t="inlineStr">
+      <c r="H40" s="141" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I39" s="141" t="inlineStr">
+      <c r="I40" s="141" t="inlineStr">
         <is>
           <t>End</t>
         </is>
       </c>
-      <c r="J39" s="141" t="inlineStr">
+      <c r="J40" s="141" t="inlineStr">
         <is>
           <t>AB12</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="48" customHeight="1">
-      <c r="A40" s="146" t="inlineStr">
+    <row r="41" ht="48" customHeight="1">
+      <c r="A41" s="146" t="inlineStr">
         <is>
           <t>C7</t>
         </is>
       </c>
-      <c r="B40" s="147" t="inlineStr">
+      <c r="B41" s="147" t="inlineStr">
         <is>
           <t>F4</t>
         </is>
       </c>
-      <c r="C40" s="147" t="inlineStr">
+      <c r="C41" s="147" t="inlineStr">
         <is>
           <t>Day D · working hours</t>
         </is>
       </c>
-      <c r="D40" s="141" t="inlineStr">
+      <c r="D41" s="141" t="inlineStr">
         <is>
           <t>D/S Team</t>
         </is>
       </c>
-      <c r="E40" s="141" t="inlineStr">
+      <c r="E41" s="141" t="inlineStr">
         <is>
           <t>XD11</t>
         </is>
       </c>
-      <c r="F40" s="141" t="inlineStr">
+      <c r="F41" s="141" t="inlineStr">
         <is>
           <t>Change Order Number: cancelled qty and candidates (same part, UPD_STATUS 6, PO_MAPPED N, no ASN, oldest first)</t>
         </is>
       </c>
-      <c r="G40" s="141" t="inlineStr">
+      <c r="G41" s="141" t="inlineStr">
         <is>
           <t>TB_R_H0253_ORDER_CONTROL_PRE
 TB_R_INSTRUCTION</t>
         </is>
       </c>
-      <c r="H40" s="141" t="inlineStr">
+      <c r="H41" s="141" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I40" s="141" t="inlineStr">
+      <c r="I41" s="141" t="inlineStr">
         <is>
           <t>C8</t>
         </is>
       </c>
-      <c r="J40" s="141" t="inlineStr">
+      <c r="J41" s="141" t="inlineStr">
         <is>
           <t>AB16</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="60" customHeight="1">
-      <c r="A41" s="146" t="inlineStr">
+    <row r="42" ht="60" customHeight="1">
+      <c r="A42" s="146" t="inlineStr">
         <is>
           <t>C8</t>
         </is>
       </c>
-      <c r="B41" s="147" t="inlineStr">
+      <c r="B42" s="147" t="inlineStr">
         <is>
           <t>F4</t>
         </is>
       </c>
-      <c r="C41" s="147" t="inlineStr">
+      <c r="C42" s="147" t="inlineStr">
         <is>
           <t>Day D · working hours</t>
         </is>
       </c>
-      <c r="D41" s="141" t="inlineStr">
+      <c r="D42" s="141" t="inlineStr">
         <is>
           <t>D/S Team</t>
         </is>
       </c>
-      <c r="E41" s="141" t="inlineStr">
+      <c r="E42" s="141" t="inlineStr">
         <is>
           <t>XD11</t>
         </is>
       </c>
-      <c r="F41" s="141" t="inlineStr">
+      <c r="F42" s="141" t="inlineStr">
         <is>
           <t>Move the qty from the last case (row split when needed) to one or more lines; history</t>
         </is>
       </c>
-      <c r="G41" s="141" t="inlineStr">
+      <c r="G42" s="141" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H41" s="141" t="inlineStr">
+      <c r="H42" s="141" t="inlineStr">
         <is>
           <t>TB_R_INSTRUCTION (order key / split)
 TB_R_H0253_ORDER_CONTROL_PRE (PO_MAPPED_FLAG Y)
 TB_H_CROSSDOCK_ORDER_CHANGE</t>
         </is>
       </c>
-      <c r="I41" s="141" t="inlineStr">
+      <c r="I42" s="141" t="inlineStr">
         <is>
           <t>End</t>
         </is>
       </c>
-      <c r="J41" s="141" t="inlineStr">
+      <c r="J42" s="141" t="inlineStr">
         <is>
           <t>AB15</t>
         </is>
@@ -24091,7 +24144,7 @@
       </c>
       <c r="D14" s="163" t="inlineStr">
         <is>
-          <t>Choose Delivery Date and Rit, click [Search]: units Ready / Partially Ready / Not Ready.</t>
+          <t>Choose Delivery Date and Rit, click [Search]: units Ready / Partially Ready / Not Ready, PO check (Short PO).</t>
         </is>
       </c>
       <c r="E14" s="163" t="inlineStr">
@@ -24107,7 +24160,7 @@
       </c>
       <c r="H14" s="163" t="inlineStr">
         <is>
-          <t>AB08: block without PO, send the Ready blocks or wait.</t>
+          <t>AB08 / AB17: case without PO (short PO), send the Ready cases or wait for the split PO.</t>
         </is>
       </c>
       <c r="I14" s="163" t="inlineStr">
@@ -24134,7 +24187,7 @@
       </c>
       <c r="D15" s="163" t="inlineStr">
         <is>
-          <t>Tick units of one supplier + plant, choose the ASN option (first n Ready blocks) and click [Create ASN].</t>
+          <t>Tick the cases of one supplier + plant (per part the oldest Customer Order Date first, from case 1 up to a cut) and click [Create ASN].</t>
         </is>
       </c>
       <c r="E15" s="163" t="inlineStr">
@@ -24349,7 +24402,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -24766,27 +24819,27 @@
       </c>
       <c r="C12" s="141" t="inlineStr">
         <is>
-          <t>D6</t>
+          <t>D6 / D7</t>
         </is>
       </c>
       <c r="D12" s="141" t="inlineStr">
         <is>
-          <t>XD09</t>
+          <t>XD09 / XD10</t>
         </is>
       </c>
       <c r="E12" s="141" t="inlineStr">
         <is>
-          <t>Block without PO: the block and every later block are Not Ready</t>
+          <t>Case without PO: the case and every later case are Not Ready; later Customer Order Dates of the part wait too</t>
         </is>
       </c>
       <c r="F12" s="141" t="inlineStr">
         <is>
-          <t>Partially Ready (later block) / check box disabled + MSG2 (first block)</t>
+          <t>Partially Ready / check box disabled + MSG2; Wait: dd-Mon first</t>
         </is>
       </c>
       <c r="G12" s="141" t="inlineStr">
         <is>
-          <t>Only the Ready blocks before it can be sent; blocks are never skipped (scan order, decided 21-Oct).</t>
+          <t>Only the Ready cases before it can be sent; cases and order dates are never skipped (scan order, decided 21-Oct / 26-Oct).</t>
         </is>
       </c>
       <c r="H12" s="141" t="inlineStr">
@@ -24796,7 +24849,7 @@
       </c>
       <c r="I12" s="141" t="inlineStr">
         <is>
-          <t>Send the Ready blocks or wait for the next PO; the block becomes Ready on a later [Search].</t>
+          <t>Send the Ready cases or wait for the next PO; the case becomes Ready on a later [Search].</t>
         </is>
       </c>
     </row>
@@ -25126,6 +25179,194 @@
       <c r="I19" s="141" t="inlineStr">
         <is>
           <t>Move the qty to received lines of the same part (UPD_STATUS 6) in Change Order Number; several lines / another destination allowed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="36" customHeight="1">
+      <c r="A20" s="168" t="inlineStr">
+        <is>
+          <t>AB17</t>
+        </is>
+      </c>
+      <c r="B20" s="141" t="inlineStr">
+        <is>
+          <t>F2</t>
+        </is>
+      </c>
+      <c r="C20" s="141" t="inlineStr">
+        <is>
+          <t>D2 / D6</t>
+        </is>
+      </c>
+      <c r="D20" s="141" t="inlineStr">
+        <is>
+          <t>existing PO / XD09</t>
+        </is>
+      </c>
+      <c r="E20" s="141" t="inlineStr">
+        <is>
+          <t>Short PO: PO qty &lt; total customer order qty of the Customer Order Date (all destinations)</t>
+        </is>
+      </c>
+      <c r="F20" s="141" t="inlineStr">
+        <is>
+          <t>Short PO chip and PO check on XD10; last cases Not Ready</t>
+        </is>
+      </c>
+      <c r="G20" s="141" t="inlineStr">
+        <is>
+          <t>The cases without PO wait; the rest comes in a split PO (later PO date); later order dates of the part wait (AB08).</t>
+        </is>
+      </c>
+      <c r="H20" s="141" t="inlineStr">
+        <is>
+          <t>Procurement / Supplier</t>
+        </is>
+      </c>
+      <c r="I20" s="141" t="inlineStr">
+        <is>
+          <t>Procurement issues the split PO; the supplier sends when the cases are Ready.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="48" customHeight="1">
+      <c r="A21" s="168" t="inlineStr">
+        <is>
+          <t>AB18</t>
+        </is>
+      </c>
+      <c r="B21" s="141" t="inlineStr">
+        <is>
+          <t>F2</t>
+        </is>
+      </c>
+      <c r="C21" s="141" t="inlineStr">
+        <is>
+          <t>D14 / D3</t>
+        </is>
+      </c>
+      <c r="D21" s="141" t="inlineStr">
+        <is>
+          <t>XD08</t>
+        </is>
+      </c>
+      <c r="E21" s="141" t="inlineStr">
+        <is>
+          <t>A line in more than one ASN is received partly; H0253 does not carry the received ASN No (TBC G-System: receiving in ASN order?)</t>
+        </is>
+      </c>
+      <c r="F21" s="141" t="inlineStr">
+        <is>
+          <t>New SERIAL_NO in H0253; LOG7</t>
+        </is>
+      </c>
+      <c r="G21" s="141" t="inlineStr">
+        <is>
+          <t>XD08 links the received part to the ASN sent first and the remaining part to the next ASN; qty always correct, the ASN-serial link can be swapped when the receiving order differs.</t>
+        </is>
+      </c>
+      <c r="H21" s="141" t="inlineStr">
+        <is>
+          <t>System admin / G-System</t>
+        </is>
+      </c>
+      <c r="I21" s="141" t="inlineStr">
+        <is>
+          <t>Confirm the receiving order with G-System; if not in ASN order, G-System provides the received ASN No.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="36" customHeight="1">
+      <c r="A22" s="168" t="inlineStr">
+        <is>
+          <t>AB19</t>
+        </is>
+      </c>
+      <c r="B22" s="141" t="inlineStr">
+        <is>
+          <t>F2 / F4</t>
+        </is>
+      </c>
+      <c r="C22" s="141" t="inlineStr">
+        <is>
+          <t>D2 / C2</t>
+        </is>
+      </c>
+      <c r="D22" s="141" t="inlineStr">
+        <is>
+          <t>existing PO</t>
+        </is>
+      </c>
+      <c r="E22" s="141" t="inlineStr">
+        <is>
+          <t>Open decision: PO qty left by cancelled orders (e.g. 12 pcs in simulasi_asn_rev) has no owner</t>
+        </is>
+      </c>
+      <c r="F22" s="141" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G22" s="141" t="inlineStr">
+        <is>
+          <t>Today: the open PO qty is taken by the next customer orders of the part (older PO date first).</t>
+        </is>
+      </c>
+      <c r="H22" s="141" t="inlineStr">
+        <is>
+          <t>Procurement / D/S Team</t>
+        </is>
+      </c>
+      <c r="I22" s="141" t="inlineStr">
+        <is>
+          <t>To decide: keep for the next orders, reduce / cancel the PO, or deliver as stock.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="36" customHeight="1">
+      <c r="A23" s="168" t="inlineStr">
+        <is>
+          <t>AB20</t>
+        </is>
+      </c>
+      <c r="B23" s="141" t="inlineStr">
+        <is>
+          <t>F4</t>
+        </is>
+      </c>
+      <c r="C23" s="141" t="inlineStr">
+        <is>
+          <t>C7</t>
+        </is>
+      </c>
+      <c r="D23" s="141" t="inlineStr">
+        <is>
+          <t>XD11</t>
+        </is>
+      </c>
+      <c r="E23" s="141" t="inlineStr">
+        <is>
+          <t>Open decision: a cancelled qty in an ASN without candidate stays in Change Order Number without time limit</t>
+        </is>
+      </c>
+      <c r="F23" s="141" t="inlineStr">
+        <is>
+          <t>Waiting for a candidate</t>
+        </is>
+      </c>
+      <c r="G23" s="141" t="inlineStr">
+        <is>
+          <t>Nothing is moved until a received line of the same part exists.</t>
+        </is>
+      </c>
+      <c r="H23" s="141" t="inlineStr">
+        <is>
+          <t>D/S Team</t>
+        </is>
+      </c>
+      <c r="I23" s="141" t="inlineStr">
+        <is>
+          <t>To decide: time limit and escalation when no candidate comes (pcs already in the warehouse).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Order of the H0253 replicate instead of the receiving scan explanation
The documents and the prototype no longer explain the receiving scan: they state the
order of the H0253 replicate (ORDER BY Allocation Priority = Customer Order Date, Customer
Code, Customer Order No, Order Date, Order Time, Destination, Detailed Item No, Serial No).
UISS XD09 4.1 'H0253 Order', XD10, BPF, ERD simulations, simulasi_asn_rev notes, web texts.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QL8Do8Pd2rXEDNa1ifG2RK
</commit_message>
<xml_diff>
--- a/deliverables/function_list_v2/bpf/Crossdock_BPF_Level2.xlsx
+++ b/deliverables/function_list_v2/bpf/Crossdock_BPF_Level2.xlsx
@@ -22625,7 +22625,7 @@
       </c>
       <c r="F22" s="141" t="inlineStr">
         <is>
-          <t>Pre-map in scan order; supplier cases, blocks (ASN options), Ready / Not Ready</t>
+          <t>Pre-map in H0253 order; supplier cases, blocks (ASN options), Ready / Not Ready</t>
         </is>
       </c>
       <c r="G22" s="141" t="inlineStr">
@@ -23004,7 +23004,7 @@
       </c>
       <c r="F29" s="141" t="inlineStr">
         <is>
-          <t>Receive the ASN in scan order → ORDER_STATUS 6; a partial receipt splits the line (new SERIAL_NO); taken by the next XD08 run (D3)</t>
+          <t>Receive the ASN → ORDER_STATUS 6; a partial receipt splits the line (new SERIAL_NO); taken by the next XD08 run (D3)</t>
         </is>
       </c>
       <c r="G29" s="141" t="inlineStr">
@@ -24230,7 +24230,7 @@
       </c>
       <c r="D16" s="163" t="inlineStr">
         <is>
-          <t>Check the Case List (supplier cases of pcs/case in scan order) and click [Submit ASN].</t>
+          <t>Check the Case List (supplier cases of pcs/case in H0253 order) and click [Submit ASN].</t>
         </is>
       </c>
       <c r="E16" s="163" t="inlineStr">
@@ -24839,7 +24839,7 @@
       </c>
       <c r="G12" s="141" t="inlineStr">
         <is>
-          <t>Only the Ready cases before it can be sent; cases and order dates are never skipped (scan order, decided 21-Oct / 26-Oct).</t>
+          <t>Only the Ready cases before it can be sent; cases and order dates are never skipped (H0253 order, decided 21-Oct / 26-Oct).</t>
         </is>
       </c>
       <c r="H12" s="141" t="inlineStr">

</xml_diff>

<commit_message>
BPF F2 diagram (hand-edited sheet) patched to the latest business logic
Texts of D2 (1 PO per Part + order date, PO date D+1), D3 (UPD_STATUS, serial split, draft
release), D6 (H0253 order, CUT_FLAG, Short PO), D7 (oldest order date first, up to a cut),
D8 (PO_MAPPED_FLAG rule); new step D14 receiving; badges AB17 / AB18; band labels (XD08 one
batch, receiving); patch_f2_manual.py keeps the manual layout.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QL8Do8Pd2rXEDNa1ifG2RK
</commit_message>
<xml_diff>
--- a/deliverables/function_list_v2/bpf/Crossdock_BPF_Level2.xlsx
+++ b/deliverables/function_list_v2/bpf/Crossdock_BPF_Level2.xlsx
@@ -8475,7 +8475,7 @@
               <a:latin typeface="Arial"/>
               <a:cs typeface="Arial"/>
             </a:rPr>
-            <a:t>Release PO Supplier (CROSSDOCK_FLAG X)</a:t>
+            <a:t>Release PO: 1 PO per Part + order date, PO date = D+1, qty = total order</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -8638,7 +8638,7 @@
               <a:latin typeface="Arial"/>
               <a:cs typeface="Arial"/>
             </a:rPr>
-            <a:t>Upsert status 7 rows + status 6 of existing keys (delta INTF_UPDATE_DT)</a:t>
+            <a:t>Upsert changed rows; UPD_STATUS 6 / 2; serial split; release drafts</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -9019,7 +9019,7 @@
               <a:latin typeface="Arial"/>
               <a:cs typeface="Arial"/>
             </a:rPr>
-            <a:t>Pre-map order lines to PO (FIFO); Case Qty, PO Readiness, Ready / Not Ready</a:t>
+            <a:t>Pre-map in H0253 order; supplier cases, CUT_FLAG; Ready / Not Ready; PO check (Short PO)</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -9237,7 +9237,7 @@
               <a:latin typeface="Arial"/>
               <a:cs typeface="Arial"/>
             </a:rPr>
-            <a:t>Select Ready units </a:t>
+            <a:t>Tick cases: oldest Customer Order Date first, from case 1 up to a cut </a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -9578,7 +9578,7 @@
               <a:latin typeface="Arial"/>
               <a:cs typeface="Arial"/>
             </a:rPr>
-            <a:t>Lock + re-check; pack cases per destination by pcs/case; real mapping</a:t>
+            <a:t>Lock + re-check; insert the ticked cases; real mapping; PO_MAPPED_FLAG Y when the whole line is in the ASN</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -12942,6 +12942,335 @@
         </a:fontRef>
       </xdr:style>
     </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>57150</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>1590675</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>911225</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="162" name="step D14"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="18097500" y="1501775"/>
+          <a:ext cx="1533525" cy="882650"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="E4DFEC"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:prstDash val="dash"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="overflow" horzOverflow="overflow" wrap="square" lIns="28575" tIns="28575" rIns="28575" bIns="28575" anchor="ctr">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="750" b="1" dirty="0">
+              <a:solidFill>
+                <a:srgbClr val="C00000"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:rPr>
+            <a:t>existing</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="750" b="0" dirty="0">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:rPr>
+            <a:t>Receive the ASN → ORDER_STATUS 6; a partial receipt splits the line (new SERIAL_NO); taken by the next XD08 run (D3)</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>1485900</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>1590675</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="163" name="corner D14"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm rot="10800000">
+          <a:off x="19526250" y="1501775"/>
+          <a:ext cx="104775" cy="104775"/>
+        </a:xfrm>
+        <a:prstGeom prst="rtTriangle">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="000000"/>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>28575</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>276225</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="164" name="no D14"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="18068925" y="1435100"/>
+          <a:ext cx="247650" cy="114300"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="000000"/>
+        </a:solidFill>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="C00000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="overflow" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="1" dirty="0">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:rPr>
+            <a:t>D14</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>1285875</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>1581150</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="165" name="ab D14 AB18"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19326225" y="1435100"/>
+          <a:ext cx="295275" cy="114300"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="C00000"/>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="overflow" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="600" b="1" dirty="0">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:rPr>
+            <a:t>AB18</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1285875</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1581150</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="166" name="ab D2 AB17"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2181225" y="2679700"/>
+          <a:ext cx="295275" cy="114300"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="C00000"/>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="overflow" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="600" b="1" dirty="0">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:rPr>
+            <a:t>AB17</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>965835</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>1261110</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="167" name="ab D3 AB18"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3766225" y="2679700"/>
+          <a:ext cx="295275" cy="114300"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="C00000"/>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="overflow" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="600" b="1" dirty="0">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:rPr>
+            <a:t>AB18</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -20064,7 +20393,7 @@
       <c r="P3" s="46" t="n"/>
       <c r="Q3" s="82" t="inlineStr">
         <is>
-          <t>19-Oct-26</t>
+          <t>27-Oct-26</t>
         </is>
       </c>
       <c r="R3" s="46" t="n"/>
@@ -20146,13 +20475,13 @@
       <c r="B7" s="46" t="n"/>
       <c r="C7" s="88" t="inlineStr">
         <is>
-          <t>D-1 · during the day</t>
+          <t>D-1 · customer order / D · PO (existing)</t>
         </is>
       </c>
       <c r="D7" s="46" t="n"/>
       <c r="E7" s="88" t="inlineStr">
         <is>
-          <t>27:30 (D 03:30) · job chain XD12 → XD11 → XD08</t>
+          <t>27:30 (D 03:30) · XD08 (one H0253 batch)</t>
         </is>
       </c>
       <c r="F7" s="46" t="n"/>
@@ -20174,7 +20503,7 @@
       <c r="R7" s="46" t="n"/>
       <c r="S7" s="89" t="inlineStr">
         <is>
-          <t>Day D · after submit</t>
+          <t>Day D · after submit / receiving</t>
         </is>
       </c>
       <c r="T7" s="45" t="n"/>

</xml_diff>

<commit_message>
BPF F2: header, title and legend as wide as the diagram (to column AG)
- Rows 1-3, 5 and legend rows 24-25 widened from Y to AG; row 6 centred (F1 and F2)
- tidy/fix_header.py (keeps the shapes of the flow sheets)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QL8Do8Pd2rXEDNa1ifG2RK
</commit_message>
<xml_diff>
--- a/deliverables/function_list_v2/bpf/Crossdock_BPF_Level2.xlsx
+++ b/deliverables/function_list_v2/bpf/Crossdock_BPF_Level2.xlsx
@@ -129,7 +129,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="135">
+  <borders count="156">
     <border>
       <left/>
       <right/>
@@ -1539,11 +1539,238 @@
         <color rgb="FF808080"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="57"/>
   </cellStyleXfs>
-  <cellXfs count="236">
+  <cellXfs count="263">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1983,6 +2210,67 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="131" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="143" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="144" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="145" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="146" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="147" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="148" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="149" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="135" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="135" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="137" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="140" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="138" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="135" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="142" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="104" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="141" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="107" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="101" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="136" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="139" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="101" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="75" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="76" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="131" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="131" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="131" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -21502,7 +21790,7 @@
       <c r="X5" s="153" t="n"/>
     </row>
     <row r="6" ht="15" customHeight="1">
-      <c r="A6" s="89" t="inlineStr">
+      <c r="A6" s="236" t="inlineStr">
         <is>
           <t>NSP Crossdock (XD01 – XD15)</t>
         </is>
@@ -22355,7 +22643,15 @@
       <c r="V1" s="91" t="n"/>
       <c r="W1" s="91" t="n"/>
       <c r="X1" s="91" t="n"/>
-      <c r="Y1" s="94" t="n"/>
+      <c r="Y1" s="91" t="n"/>
+      <c r="Z1" s="91" t="n"/>
+      <c r="AA1" s="91" t="n"/>
+      <c r="AB1" s="91" t="n"/>
+      <c r="AC1" s="91" t="n"/>
+      <c r="AD1" s="91" t="n"/>
+      <c r="AE1" s="91" t="n"/>
+      <c r="AF1" s="91" t="n"/>
+      <c r="AG1" s="94" t="n"/>
     </row>
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="74" t="inlineStr">
@@ -22414,7 +22710,15 @@
         </is>
       </c>
       <c r="X2" s="91" t="n"/>
-      <c r="Y2" s="94" t="n"/>
+      <c r="Y2" s="91" t="n"/>
+      <c r="Z2" s="91" t="n"/>
+      <c r="AA2" s="91" t="n"/>
+      <c r="AB2" s="91" t="n"/>
+      <c r="AC2" s="91" t="n"/>
+      <c r="AD2" s="91" t="n"/>
+      <c r="AE2" s="91" t="n"/>
+      <c r="AF2" s="91" t="n"/>
+      <c r="AG2" s="94" t="n"/>
     </row>
     <row r="3" ht="14" customHeight="1">
       <c r="A3" s="74" t="inlineStr">
@@ -22473,7 +22777,15 @@
         </is>
       </c>
       <c r="X3" s="91" t="n"/>
-      <c r="Y3" s="94" t="n"/>
+      <c r="Y3" s="91" t="n"/>
+      <c r="Z3" s="91" t="n"/>
+      <c r="AA3" s="91" t="n"/>
+      <c r="AB3" s="91" t="n"/>
+      <c r="AC3" s="91" t="n"/>
+      <c r="AD3" s="91" t="n"/>
+      <c r="AE3" s="91" t="n"/>
+      <c r="AF3" s="91" t="n"/>
+      <c r="AG3" s="94" t="n"/>
     </row>
     <row r="4" ht="6" customHeight="1"/>
     <row r="5" ht="20" customHeight="1" thickBot="1">
@@ -22505,15 +22817,15 @@
       <c r="V5" s="147" t="n"/>
       <c r="W5" s="147" t="n"/>
       <c r="X5" s="147" t="n"/>
-      <c r="Y5" s="148" t="n"/>
-      <c r="Z5" s="26" t="n"/>
-      <c r="AA5" s="26" t="n"/>
-      <c r="AB5" s="26" t="n"/>
-      <c r="AC5" s="26" t="n"/>
-      <c r="AD5" s="26" t="n"/>
-      <c r="AE5" s="26" t="n"/>
-      <c r="AF5" s="26" t="n"/>
-      <c r="AG5" s="26" t="n"/>
+      <c r="Y5" s="147" t="n"/>
+      <c r="Z5" s="147" t="n"/>
+      <c r="AA5" s="147" t="n"/>
+      <c r="AB5" s="147" t="n"/>
+      <c r="AC5" s="147" t="n"/>
+      <c r="AD5" s="147" t="n"/>
+      <c r="AE5" s="147" t="n"/>
+      <c r="AF5" s="147" t="n"/>
+      <c r="AG5" s="148" t="n"/>
     </row>
     <row r="6" ht="15" customHeight="1" thickBot="1">
       <c r="A6" s="158" t="inlineStr">
@@ -23204,7 +23516,15 @@
       <c r="V24" s="15" t="n"/>
       <c r="W24" s="15" t="n"/>
       <c r="X24" s="15" t="n"/>
-      <c r="Y24" s="13" t="n"/>
+      <c r="Y24" s="240" t="n"/>
+      <c r="Z24" s="240" t="n"/>
+      <c r="AA24" s="240" t="n"/>
+      <c r="AB24" s="240" t="n"/>
+      <c r="AC24" s="240" t="n"/>
+      <c r="AD24" s="240" t="n"/>
+      <c r="AE24" s="240" t="n"/>
+      <c r="AF24" s="240" t="n"/>
+      <c r="AG24" s="241" t="n"/>
     </row>
     <row r="25" ht="14" customHeight="1">
       <c r="A25" s="110" t="n"/>
@@ -23231,7 +23551,15 @@
       <c r="V25" s="16" t="n"/>
       <c r="W25" s="16" t="n"/>
       <c r="X25" s="16" t="n"/>
-      <c r="Y25" s="14" t="n"/>
+      <c r="Y25" s="242" t="n"/>
+      <c r="Z25" s="242" t="n"/>
+      <c r="AA25" s="242" t="n"/>
+      <c r="AB25" s="242" t="n"/>
+      <c r="AC25" s="242" t="n"/>
+      <c r="AD25" s="242" t="n"/>
+      <c r="AE25" s="242" t="n"/>
+      <c r="AF25" s="242" t="n"/>
+      <c r="AG25" s="243" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="41">
@@ -23241,15 +23569,12 @@
     <mergeCell ref="A8:A10"/>
     <mergeCell ref="A6:AG6"/>
     <mergeCell ref="A17:A19"/>
-    <mergeCell ref="W3:Y3"/>
     <mergeCell ref="A20:A22"/>
-    <mergeCell ref="A5:Y5"/>
     <mergeCell ref="G3:L3"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="A11:A16"/>
     <mergeCell ref="S3:T3"/>
-    <mergeCell ref="S1:Y1"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="M2:N2"/>
     <mergeCell ref="S2:T2"/>
@@ -23258,10 +23583,12 @@
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="B20:B22"/>
     <mergeCell ref="Z7:AG7"/>
-    <mergeCell ref="W2:Y2"/>
+    <mergeCell ref="A5:AG5"/>
+    <mergeCell ref="W3:AG3"/>
     <mergeCell ref="U7:Y7"/>
     <mergeCell ref="Q1:R1"/>
     <mergeCell ref="U3:V3"/>
+    <mergeCell ref="S1:AG1"/>
     <mergeCell ref="B11:B13"/>
     <mergeCell ref="B8:B10"/>
     <mergeCell ref="M3:N3"/>
@@ -23275,6 +23602,7 @@
     <mergeCell ref="G2:L2"/>
     <mergeCell ref="E7:F7"/>
     <mergeCell ref="G1:H1"/>
+    <mergeCell ref="W2:AG2"/>
     <mergeCell ref="B14:B16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
BPF: step codes of Step Detail, User Process and Abnormality in sync with the F1 / F2 diagrams
- F1 M8 = XD01 check status and history (no abnormality), as on the diagram
- F2 steps as on the revised diagram: D0 AP POLE release, D1 at 27:30, D12 / D13 interfaces, D14 receive by GTOPAS, D15 H0253 update; Log Monitoring step removed (U11 -> D10); next steps D2 / D3 -> D6, D7 -> D8, D9, D10 -> D11, D12
- Abnormality steps: AB08 D6, AB09 D7 / H4, AB17 D2, AB18 D15 / D3
- Diagram F2: number badges D0, D12-D15 and AB18 on D15; tidy grid reader handles both attribute orders

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QL8Do8Pd2rXEDNa1ifG2RK
</commit_message>
<xml_diff>
--- a/deliverables/function_list_v2/bpf/Crossdock_BPF_Level2.xlsx
+++ b/deliverables/function_list_v2/bpf/Crossdock_BPF_Level2.xlsx
@@ -14978,6 +14978,346 @@
     </xdr:cxnSp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>28575</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>43760</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>276225</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>158060</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="501" name="no D0"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="781050" y="1326460"/>
+          <a:ext cx="247650" cy="114300"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="000000"/>
+        </a:solidFill>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="C00000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="overflow" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="1" dirty="0">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:rPr>
+            <a:t>D0</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>180975</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>219075</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="502" name="no D12"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="17516475" y="3044825"/>
+          <a:ext cx="247650" cy="114300"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="000000"/>
+        </a:solidFill>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="C00000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="overflow" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="1" dirty="0">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:rPr>
+            <a:t>D12</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>182470</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>688600</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>220570</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>802900</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="503" name="no D13"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="17517970" y="2161800"/>
+          <a:ext cx="247650" cy="114300"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="000000"/>
+        </a:solidFill>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="C00000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="overflow" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="1" dirty="0">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:rPr>
+            <a:t>D13</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>170516</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>211312</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>418166</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>97012</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="504" name="no D14"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="21335066" y="1265412"/>
+          <a:ext cx="247650" cy="114300"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="000000"/>
+        </a:solidFill>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="C00000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="overflow" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="1" dirty="0">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:rPr>
+            <a:t>D14</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>464860</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>504824</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>29</xdr:col>
+      <xdr:colOff>102910</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>619124</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="505" name="no D15"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="23458210" y="1978024"/>
+          <a:ext cx="247650" cy="114300"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="000000"/>
+        </a:solidFill>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="C00000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="overflow" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="650" b="1" dirty="0">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:rPr>
+            <a:t>D15</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>338546</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>504824</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>24221</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>619124</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="506" name="ab D15 AB18"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="24551096" y="1978024"/>
+          <a:ext cx="295275" cy="114300"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="C00000"/>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="overflow" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="600" b="1" dirty="0">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:rPr>
+            <a:t>AB18</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -24856,7 +25196,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J44"/>
+  <dimension ref="A1:J46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -25336,12 +25676,12 @@
       </c>
       <c r="E12" s="206" t="inlineStr">
         <is>
-          <t>XD01 · XD02</t>
+          <t>XD01</t>
         </is>
       </c>
       <c r="F12" s="206" t="inlineStr">
         <is>
-          <t>Check history of the candidate part</t>
+          <t>Check status and history of the parts</t>
         </is>
       </c>
       <c r="G12" s="206" t="inlineStr">
@@ -25362,7 +25702,7 @@
       </c>
       <c r="J12" s="206" t="inlineStr">
         <is>
-          <t>AB04</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -25636,7 +25976,7 @@
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="208" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>D0</t>
         </is>
       </c>
       <c r="B18" s="209" t="inlineStr">
@@ -25656,27 +25996,27 @@
       </c>
       <c r="E18" s="206" t="inlineStr">
         <is>
+          <t>existing</t>
+        </is>
+      </c>
+      <c r="F18" s="206" t="inlineStr">
+        <is>
+          <t>Release crossdock customer orders (multiples of pcs/case) from AP POLE System</t>
+        </is>
+      </c>
+      <c r="G18" s="206" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F18" s="206" t="inlineStr">
-        <is>
-          <t>Release crossdock customer orders (ORDER_STATUS 7, multiples of pcs/case)</t>
-        </is>
-      </c>
-      <c r="G18" s="206" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="H18" s="206" t="inlineStr">
         <is>
-          <t>TB_R_H0253_ORDER_CONTROL_PRE (DB Surrounding)</t>
+          <t>GTOPAS</t>
         </is>
       </c>
       <c r="I18" s="206" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>D1, D2</t>
         </is>
       </c>
       <c r="J18" s="206" t="inlineStr">
@@ -25729,153 +26069,205 @@
       </c>
       <c r="I19" s="206" t="inlineStr">
         <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="J19" s="206" t="inlineStr">
+        <is>
+          <t>AB17</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="24" customHeight="1">
+      <c r="A20" s="208" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
+      <c r="B20" s="209" t="inlineStr">
+        <is>
+          <t>F2</t>
+        </is>
+      </c>
+      <c r="C20" s="209" t="inlineStr">
+        <is>
+          <t>27:30 (D 03:30) · XD08</t>
+        </is>
+      </c>
+      <c r="D20" s="206" t="inlineStr">
+        <is>
+          <t>GTOPAS / DB Surrounding</t>
+        </is>
+      </c>
+      <c r="E20" s="206" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F20" s="206" t="inlineStr">
+        <is>
+          <t>Release crossdock customer orders (ORDER_STATUS 7, multiples of pcs/case)</t>
+        </is>
+      </c>
+      <c r="G20" s="206" t="inlineStr">
+        <is>
+          <t>TB_R_H0253_ORDER_CONTROL_PRE (Surrounding DPV)</t>
+        </is>
+      </c>
+      <c r="H20" s="206" t="inlineStr">
+        <is>
+          <t>TB_R_H0253_ORDER_CONTROL_PRE (DB Surrounding)</t>
+        </is>
+      </c>
+      <c r="I20" s="206" t="inlineStr">
+        <is>
           <t>D3</t>
         </is>
       </c>
-      <c r="J19" s="206" t="inlineStr">
-        <is>
-          <t>AB17</t>
+      <c r="J20" s="206" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="60" customHeight="1">
-      <c r="A20" s="210" t="inlineStr">
+    <row r="21" ht="60" customHeight="1">
+      <c r="A21" s="210" t="inlineStr">
         <is>
           <t>D3</t>
         </is>
       </c>
-      <c r="B20" s="211" t="inlineStr">
+      <c r="B21" s="211" t="inlineStr">
         <is>
           <t>F2</t>
         </is>
       </c>
-      <c r="C20" s="211" t="inlineStr">
+      <c r="C21" s="211" t="inlineStr">
         <is>
           <t>27:30 (D 03:30) · XD08</t>
         </is>
       </c>
-      <c r="D20" s="206" t="inlineStr">
+      <c r="D21" s="206" t="inlineStr">
         <is>
           <t>NSP Batch (System)</t>
         </is>
       </c>
-      <c r="E20" s="206" t="inlineStr">
+      <c r="E21" s="206" t="inlineStr">
         <is>
           <t>XD08</t>
         </is>
       </c>
-      <c r="F20" s="206" t="inlineStr">
+      <c r="F21" s="206" t="inlineStr">
         <is>
           <t>Upsert changed rows (delta INTF_UPDATE_DT); UPD_STATUS 6 / 2; serial split: each part stays linked to its ASN; release all drafts</t>
         </is>
       </c>
-      <c r="G20" s="206" t="inlineStr">
+      <c r="G21" s="206" t="inlineStr">
         <is>
           <t>TB_R_H0253_ORDER_CONTROL_PRE (DB Surrounding)</t>
         </is>
       </c>
-      <c r="H20" s="206" t="inlineStr">
+      <c r="H21" s="206" t="inlineStr">
         <is>
           <t>TB_R_H0253_ORDER_CONTROL_PRE (NSP)
 TB_R_INSTRUCTION (SERIAL_NO)
 Log</t>
         </is>
       </c>
-      <c r="I20" s="206" t="inlineStr">
+      <c r="I21" s="206" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="J21" s="206" t="inlineStr">
+        <is>
+          <t>AB07, AB18</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="15" customHeight="1">
+      <c r="A22" s="218" t="inlineStr">
         <is>
           <t>D5</t>
         </is>
       </c>
-      <c r="J20" s="206" t="inlineStr">
-        <is>
-          <t>AB07, AB18</t>
+      <c r="B22" s="219" t="inlineStr">
+        <is>
+          <t>F2</t>
+        </is>
+      </c>
+      <c r="C22" s="219" t="inlineStr">
+        <is>
+          <t>Daily · scheduler</t>
+        </is>
+      </c>
+      <c r="D22" s="206" t="inlineStr">
+        <is>
+          <t>Supplier</t>
+        </is>
+      </c>
+      <c r="E22" s="206" t="inlineStr">
+        <is>
+          <t>XD10</t>
+        </is>
+      </c>
+      <c r="F22" s="206" t="inlineStr">
+        <is>
+          <t>Choose Delivery Date + Rit, [Search]</t>
+        </is>
+      </c>
+      <c r="G22" s="206" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H22" s="206" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I22" s="206" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="J22" s="206" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1">
-      <c r="A21" s="218" t="inlineStr">
-        <is>
-          <t>D5</t>
-        </is>
-      </c>
-      <c r="B21" s="219" t="inlineStr">
+    <row r="23" ht="96" customHeight="1">
+      <c r="A23" s="210" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="B23" s="211" t="inlineStr">
         <is>
           <t>F2</t>
         </is>
       </c>
-      <c r="C21" s="219" t="inlineStr">
+      <c r="C23" s="211" t="inlineStr">
         <is>
           <t>Daily · scheduler</t>
         </is>
       </c>
-      <c r="D21" s="206" t="inlineStr">
-        <is>
-          <t>Supplier</t>
-        </is>
-      </c>
-      <c r="E21" s="206" t="inlineStr">
-        <is>
-          <t>XD10</t>
-        </is>
-      </c>
-      <c r="F21" s="206" t="inlineStr">
-        <is>
-          <t>Choose Delivery Date + Rit, [Search]</t>
-        </is>
-      </c>
-      <c r="G21" s="206" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H21" s="206" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I21" s="206" t="inlineStr">
-        <is>
-          <t>D6</t>
-        </is>
-      </c>
-      <c r="J21" s="206" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="96" customHeight="1">
-      <c r="A22" s="210" t="inlineStr">
-        <is>
-          <t>D6</t>
-        </is>
-      </c>
-      <c r="B22" s="211" t="inlineStr">
-        <is>
-          <t>F2</t>
-        </is>
-      </c>
-      <c r="C22" s="211" t="inlineStr">
-        <is>
-          <t>Daily · scheduler</t>
-        </is>
-      </c>
-      <c r="D22" s="206" t="inlineStr">
+      <c r="D23" s="206" t="inlineStr">
         <is>
           <t>NSP Batch (System)</t>
         </is>
       </c>
-      <c r="E22" s="206" t="inlineStr">
+      <c r="E23" s="206" t="inlineStr">
         <is>
           <t>XD09</t>
         </is>
       </c>
-      <c r="F22" s="206" t="inlineStr">
+      <c r="F23" s="206" t="inlineStr">
         <is>
           <t>Pre-map in H0253 order; supplier cases, blocks (ASN options), Ready / Not Ready</t>
         </is>
       </c>
-      <c r="G22" s="206" t="inlineStr">
+      <c r="G23" s="206" t="inlineStr">
         <is>
           <t>TB_R_H0253_ORDER_CONTROL_PRE (status 7, HOLD N, open qty)
 TB_R_INSTRUCTION
@@ -25884,213 +26276,213 @@
 TB_R_PRA_DAILY_ORDER_MAPPED</t>
         </is>
       </c>
-      <c r="H22" s="206" t="inlineStr">
+      <c r="H23" s="206" t="inlineStr">
         <is>
           <t>#TEMP_INSTRUCTION</t>
         </is>
       </c>
-      <c r="I22" s="206" t="inlineStr">
+      <c r="I23" s="206" t="inlineStr">
         <is>
           <t>D7</t>
         </is>
       </c>
-      <c r="J22" s="206" t="inlineStr">
+      <c r="J23" s="206" t="inlineStr">
         <is>
           <t>AB08</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="36" customHeight="1">
-      <c r="A23" s="218" t="inlineStr">
+    <row r="24" ht="36" customHeight="1">
+      <c r="A24" s="218" t="inlineStr">
         <is>
           <t>D7</t>
         </is>
       </c>
-      <c r="B23" s="219" t="inlineStr">
+      <c r="B24" s="219" t="inlineStr">
         <is>
           <t>F2</t>
         </is>
       </c>
-      <c r="C23" s="219" t="inlineStr">
+      <c r="C24" s="219" t="inlineStr">
         <is>
           <t>Daily · scheduler</t>
         </is>
       </c>
-      <c r="D23" s="206" t="inlineStr">
+      <c r="D24" s="206" t="inlineStr">
         <is>
           <t>Supplier</t>
         </is>
       </c>
-      <c r="E23" s="206" t="inlineStr">
+      <c r="E24" s="206" t="inlineStr">
         <is>
           <t>XD10</t>
         </is>
       </c>
-      <c r="F23" s="206" t="inlineStr">
+      <c r="F24" s="206" t="inlineStr">
         <is>
           <t>Tick cases: per part the oldest Customer Order Date first; from case 1 up to a cut (CUT_FLAG); [Create ASN]</t>
         </is>
       </c>
-      <c r="G23" s="206" t="inlineStr">
+      <c r="G24" s="206" t="inlineStr">
         <is>
           <t>#TEMP_INSTRUCTION</t>
         </is>
       </c>
-      <c r="H23" s="206" t="inlineStr">
+      <c r="H24" s="206" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I23" s="206" t="inlineStr">
+      <c r="I24" s="206" t="inlineStr">
+        <is>
+          <t>D8, D9</t>
+        </is>
+      </c>
+      <c r="J24" s="206" t="inlineStr">
+        <is>
+          <t>AB09, AB10, AB11</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="60" customHeight="1">
+      <c r="A25" s="210" t="inlineStr">
         <is>
           <t>D8</t>
         </is>
       </c>
-      <c r="J23" s="206" t="inlineStr">
-        <is>
-          <t>AB10, AB11</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="60" customHeight="1">
-      <c r="A24" s="210" t="inlineStr">
-        <is>
-          <t>D8</t>
-        </is>
-      </c>
-      <c r="B24" s="211" t="inlineStr">
+      <c r="B25" s="211" t="inlineStr">
         <is>
           <t>F2</t>
         </is>
       </c>
-      <c r="C24" s="211" t="inlineStr">
+      <c r="C25" s="211" t="inlineStr">
         <is>
           <t>Daily · scheduler</t>
         </is>
       </c>
-      <c r="D24" s="206" t="inlineStr">
+      <c r="D25" s="206" t="inlineStr">
         <is>
           <t>NSP Batch (System)</t>
         </is>
       </c>
-      <c r="E24" s="206" t="inlineStr">
+      <c r="E25" s="206" t="inlineStr">
         <is>
           <t>XD10</t>
         </is>
       </c>
-      <c r="F24" s="206" t="inlineStr">
+      <c r="F25" s="206" t="inlineStr">
         <is>
           <t>Lock + re-check; insert the ticked cases (XD09); real mapping; PO_MAPPED_FLAG Y when the whole line is in the ASN</t>
         </is>
       </c>
-      <c r="G24" s="206" t="inlineStr">
+      <c r="G25" s="206" t="inlineStr">
         <is>
           <t>#TEMP_INSTRUCTION
 TB_R_H0253_ORDER_CONTROL_PRE</t>
         </is>
       </c>
-      <c r="H24" s="206" t="inlineStr">
+      <c r="H25" s="206" t="inlineStr">
         <is>
           <t>TB_R_INSTRUCTION
 TB_R_H0253_ORDER_CONTROL_PRE (PO_MAPPED_FLAG Y)
 TB_R_PRA_DAILY_ORDER_MAPPED (MAPPED_QTY)</t>
         </is>
       </c>
-      <c r="I24" s="206" t="inlineStr">
+      <c r="I25" s="206" t="inlineStr">
         <is>
           <t>D9</t>
         </is>
       </c>
-      <c r="J24" s="206" t="inlineStr">
+      <c r="J25" s="206" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="24" customHeight="1">
-      <c r="A25" s="218" t="inlineStr">
+    <row r="26" ht="24" customHeight="1">
+      <c r="A26" s="218" t="inlineStr">
         <is>
           <t>D9</t>
         </is>
       </c>
-      <c r="B25" s="219" t="inlineStr">
+      <c r="B26" s="219" t="inlineStr">
         <is>
           <t>F2</t>
         </is>
       </c>
-      <c r="C25" s="219" t="inlineStr">
+      <c r="C26" s="219" t="inlineStr">
         <is>
           <t>Daily · scheduler</t>
         </is>
       </c>
-      <c r="D25" s="206" t="inlineStr">
+      <c r="D26" s="206" t="inlineStr">
         <is>
           <t>Supplier</t>
         </is>
       </c>
-      <c r="E25" s="206" t="inlineStr">
+      <c r="E26" s="206" t="inlineStr">
         <is>
           <t>XD10</t>
         </is>
       </c>
-      <c r="F25" s="206" t="inlineStr">
+      <c r="F26" s="206" t="inlineStr">
         <is>
           <t>Case List: check cases, [Submit ASN] → [Yes, submit]</t>
         </is>
       </c>
-      <c r="G25" s="206" t="inlineStr">
+      <c r="G26" s="206" t="inlineStr">
         <is>
           <t>TB_R_INSTRUCTION</t>
         </is>
       </c>
-      <c r="H25" s="206" t="inlineStr">
+      <c r="H26" s="206" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I25" s="206" t="inlineStr">
+      <c r="I26" s="206" t="inlineStr">
         <is>
           <t>D10</t>
         </is>
       </c>
-      <c r="J25" s="206" t="inlineStr">
+      <c r="J26" s="206" t="inlineStr">
         <is>
           <t>AB12</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="84" customHeight="1">
-      <c r="A26" s="210" t="inlineStr">
+    <row r="27" ht="84" customHeight="1">
+      <c r="A27" s="210" t="inlineStr">
         <is>
           <t>D10</t>
         </is>
       </c>
-      <c r="B26" s="211" t="inlineStr">
+      <c r="B27" s="211" t="inlineStr">
         <is>
           <t>F2</t>
         </is>
       </c>
-      <c r="C26" s="211" t="inlineStr">
+      <c r="C27" s="211" t="inlineStr">
         <is>
           <t>Daily · scheduler</t>
         </is>
       </c>
-      <c r="D26" s="206" t="inlineStr">
+      <c r="D27" s="206" t="inlineStr">
         <is>
           <t>NSP Batch (System)</t>
         </is>
       </c>
-      <c r="E26" s="206" t="inlineStr">
+      <c r="E27" s="206" t="inlineStr">
         <is>
           <t>XD10 (5.7)</t>
         </is>
       </c>
-      <c r="F26" s="206" t="inlineStr">
+      <c r="F27" s="206" t="inlineStr">
         <is>
           <t>Submit process (Submit ID): ASN No / Case No by existing sequence, ASN Created</t>
         </is>
       </c>
-      <c r="G26" s="206" t="inlineStr">
+      <c r="G27" s="206" t="inlineStr">
         <is>
           <t>TB_R_INSTRUCTION
 TB_R_PRA_DAILY_ORDER_MANIFEST
@@ -26098,7 +26490,7 @@
 TB_M_PART_MASTER (PART_NAME)</t>
         </is>
       </c>
-      <c r="H26" s="206" t="inlineStr">
+      <c r="H27" s="206" t="inlineStr">
         <is>
           <t>TB_R_DAILY_ORDER_MANIFEST
 TB_R_DAILY_ORDER_PART
@@ -26107,98 +26499,46 @@
 Log</t>
         </is>
       </c>
-      <c r="I26" s="206" t="inlineStr">
-        <is>
-          <t>D11, D12, D13</t>
-        </is>
-      </c>
-      <c r="J26" s="206" t="inlineStr">
+      <c r="I27" s="206" t="inlineStr">
+        <is>
+          <t>D11, D12</t>
+        </is>
+      </c>
+      <c r="J27" s="206" t="inlineStr">
         <is>
           <t>AB13</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="24" customHeight="1">
-      <c r="A27" s="208" t="inlineStr">
-        <is>
-          <t>D12</t>
-        </is>
-      </c>
-      <c r="B27" s="209" t="inlineStr">
-        <is>
-          <t>F2</t>
-        </is>
-      </c>
-      <c r="C27" s="209" t="inlineStr">
-        <is>
-          <t>Day D · after submit / receiving</t>
-        </is>
-      </c>
-      <c r="D27" s="206" t="inlineStr">
-        <is>
-          <t>GTOPAS / DB Surrounding</t>
-        </is>
-      </c>
-      <c r="E27" s="206" t="inlineStr">
-        <is>
-          <t>existing</t>
-        </is>
-      </c>
-      <c r="F27" s="206" t="inlineStr">
-        <is>
-          <t>Receive ASN</t>
-        </is>
-      </c>
-      <c r="G27" s="206" t="inlineStr">
-        <is>
-          <t>Existing ASN feedback</t>
-        </is>
-      </c>
-      <c r="H27" s="206" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I27" s="206" t="inlineStr">
-        <is>
-          <t>End</t>
-        </is>
-      </c>
-      <c r="J27" s="206" t="inlineStr">
-        <is>
-          <t>-</t>
         </is>
       </c>
     </row>
     <row r="28" ht="36" customHeight="1">
-      <c r="A28" s="218" t="inlineStr">
-        <is>
-          <t>D11</t>
-        </is>
-      </c>
-      <c r="B28" s="219" t="inlineStr">
+      <c r="A28" s="210" t="inlineStr">
+        <is>
+          <t>D12</t>
+        </is>
+      </c>
+      <c r="B28" s="211" t="inlineStr">
         <is>
           <t>F2</t>
         </is>
       </c>
-      <c r="C28" s="219" t="inlineStr">
-        <is>
-          <t>Day D · after submit / receiving</t>
+      <c r="C28" s="211" t="inlineStr">
+        <is>
+          <t>Day D · after submit</t>
         </is>
       </c>
       <c r="D28" s="206" t="inlineStr">
         <is>
-          <t>Supplier</t>
+          <t>NSP Batch (System)</t>
         </is>
       </c>
       <c r="E28" s="206" t="inlineStr">
         <is>
-          <t>XD15</t>
+          <t>existing</t>
         </is>
       </c>
       <c r="F28" s="206" t="inlineStr">
         <is>
-          <t>ASN Inquiry; download case label (1 label = 1 case of 1 destination)</t>
+          <t>Interface ASN data to Surrounding</t>
         </is>
       </c>
       <c r="G28" s="206" t="inlineStr">
@@ -26209,855 +26549,960 @@
       </c>
       <c r="H28" s="206" t="inlineStr">
         <is>
+          <t>ASN data (DB Surrounding)</t>
+        </is>
+      </c>
+      <c r="I28" s="206" t="inlineStr">
+        <is>
+          <t>D13</t>
+        </is>
+      </c>
+      <c r="J28" s="206" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I28" s="206" t="inlineStr">
+    </row>
+    <row r="29" ht="24" customHeight="1">
+      <c r="A29" s="208" t="inlineStr">
+        <is>
+          <t>D13</t>
+        </is>
+      </c>
+      <c r="B29" s="209" t="inlineStr">
+        <is>
+          <t>F2</t>
+        </is>
+      </c>
+      <c r="C29" s="209" t="inlineStr">
+        <is>
+          <t>Day D · after submit</t>
+        </is>
+      </c>
+      <c r="D29" s="206" t="inlineStr">
+        <is>
+          <t>GTOPAS / DB Surrounding</t>
+        </is>
+      </c>
+      <c r="E29" s="206" t="inlineStr">
+        <is>
+          <t>existing</t>
+        </is>
+      </c>
+      <c r="F29" s="206" t="inlineStr">
+        <is>
+          <t>Interface ASN data to GTOPAS</t>
+        </is>
+      </c>
+      <c r="G29" s="206" t="inlineStr">
+        <is>
+          <t>ASN data (DB Surrounding)</t>
+        </is>
+      </c>
+      <c r="H29" s="206" t="inlineStr">
+        <is>
+          <t>Receiving Data (GTOPAS)</t>
+        </is>
+      </c>
+      <c r="I29" s="206" t="inlineStr">
+        <is>
+          <t>D14</t>
+        </is>
+      </c>
+      <c r="J29" s="206" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="36" customHeight="1">
+      <c r="A30" s="218" t="inlineStr">
+        <is>
+          <t>D11</t>
+        </is>
+      </c>
+      <c r="B30" s="219" t="inlineStr">
+        <is>
+          <t>F2</t>
+        </is>
+      </c>
+      <c r="C30" s="219" t="inlineStr">
+        <is>
+          <t>Day D · after submit</t>
+        </is>
+      </c>
+      <c r="D30" s="206" t="inlineStr">
+        <is>
+          <t>Supplier</t>
+        </is>
+      </c>
+      <c r="E30" s="206" t="inlineStr">
+        <is>
+          <t>XD15</t>
+        </is>
+      </c>
+      <c r="F30" s="206" t="inlineStr">
+        <is>
+          <t>ASN Inquiry; download case label (1 label = 1 case of 1 destination)</t>
+        </is>
+      </c>
+      <c r="G30" s="206" t="inlineStr">
+        <is>
+          <t>TB_R_DAILY_ORDER_MANIFEST
+TB_R_DAILY_ORDER_PART</t>
+        </is>
+      </c>
+      <c r="H30" s="206" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I30" s="206" t="inlineStr">
         <is>
           <t>End</t>
         </is>
       </c>
-      <c r="J28" s="206" t="inlineStr">
+      <c r="J30" s="206" t="inlineStr">
         <is>
           <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="36" customHeight="1">
-      <c r="A29" s="208" t="inlineStr">
-        <is>
-          <t>D14</t>
-        </is>
-      </c>
-      <c r="B29" s="209" t="inlineStr">
-        <is>
-          <t>F2</t>
-        </is>
-      </c>
-      <c r="C29" s="209" t="inlineStr">
-        <is>
-          <t>Day D · after submit / receiving</t>
-        </is>
-      </c>
-      <c r="D29" s="206" t="inlineStr">
-        <is>
-          <t>GTOPAS / DB Surrounding</t>
-        </is>
-      </c>
-      <c r="E29" s="206" t="inlineStr">
-        <is>
-          <t>existing</t>
-        </is>
-      </c>
-      <c r="F29" s="206" t="inlineStr">
-        <is>
-          <t>Receive the ASN → ORDER_STATUS 6; a partial receipt splits the line (new SERIAL_NO); taken by the next XD08 run (D3)</t>
-        </is>
-      </c>
-      <c r="G29" s="206" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H29" s="206" t="inlineStr">
-        <is>
-          <t>TB_R_H0253_ORDER_CONTROL_PRE (DB Surrounding, INTF_UPDATE_DT)</t>
-        </is>
-      </c>
-      <c r="I29" s="206" t="inlineStr">
-        <is>
-          <t>End</t>
-        </is>
-      </c>
-      <c r="J29" s="206" t="inlineStr">
-        <is>
-          <t>AB18</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="24" customHeight="1">
-      <c r="A30" s="218" t="inlineStr">
-        <is>
-          <t>D13</t>
-        </is>
-      </c>
-      <c r="B30" s="219" t="inlineStr">
-        <is>
-          <t>F2</t>
-        </is>
-      </c>
-      <c r="C30" s="219" t="inlineStr">
-        <is>
-          <t>Day D · after submit / receiving</t>
-        </is>
-      </c>
-      <c r="D30" s="206" t="inlineStr">
-        <is>
-          <t>Supplier</t>
-        </is>
-      </c>
-      <c r="E30" s="206" t="inlineStr">
-        <is>
-          <t>Log Monitoring</t>
-        </is>
-      </c>
-      <c r="F30" s="206" t="inlineStr">
-        <is>
-          <t>Check the submit result per Submit ID</t>
-        </is>
-      </c>
-      <c r="G30" s="206" t="inlineStr">
-        <is>
-          <t>Log</t>
-        </is>
-      </c>
-      <c r="H30" s="206" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I30" s="206" t="inlineStr">
-        <is>
-          <t>End</t>
-        </is>
-      </c>
-      <c r="J30" s="206" t="inlineStr">
-        <is>
-          <t>AB13</t>
         </is>
       </c>
     </row>
     <row r="31" ht="24" customHeight="1">
-      <c r="A31" s="214" t="inlineStr">
+      <c r="A31" s="208" t="inlineStr">
+        <is>
+          <t>D14</t>
+        </is>
+      </c>
+      <c r="B31" s="209" t="inlineStr">
+        <is>
+          <t>F2</t>
+        </is>
+      </c>
+      <c r="C31" s="209" t="inlineStr">
+        <is>
+          <t>Day D+1 · after receive</t>
+        </is>
+      </c>
+      <c r="D31" s="206" t="inlineStr">
+        <is>
+          <t>GTOPAS / DB Surrounding</t>
+        </is>
+      </c>
+      <c r="E31" s="206" t="inlineStr">
+        <is>
+          <t>existing</t>
+        </is>
+      </c>
+      <c r="F31" s="206" t="inlineStr">
+        <is>
+          <t>Receive by GTOPAS</t>
+        </is>
+      </c>
+      <c r="G31" s="206" t="inlineStr">
+        <is>
+          <t>Receiving Data (GTOPAS)</t>
+        </is>
+      </c>
+      <c r="H31" s="206" t="inlineStr">
+        <is>
+          <t>TB_R_H0253_ORDER_CONTROL_PRE (Surrounding DPV)</t>
+        </is>
+      </c>
+      <c r="I31" s="206" t="inlineStr">
+        <is>
+          <t>D15</t>
+        </is>
+      </c>
+      <c r="J31" s="206" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="36" customHeight="1">
+      <c r="A32" s="208" t="inlineStr">
+        <is>
+          <t>D15</t>
+        </is>
+      </c>
+      <c r="B32" s="209" t="inlineStr">
+        <is>
+          <t>F2</t>
+        </is>
+      </c>
+      <c r="C32" s="209" t="inlineStr">
+        <is>
+          <t>Day D+1 · after receive</t>
+        </is>
+      </c>
+      <c r="D32" s="206" t="inlineStr">
+        <is>
+          <t>GTOPAS / DB Surrounding</t>
+        </is>
+      </c>
+      <c r="E32" s="206" t="inlineStr">
+        <is>
+          <t>existing</t>
+        </is>
+      </c>
+      <c r="F32" s="206" t="inlineStr">
+        <is>
+          <t>H0253 Update Data: ORDER_STATUS 6; a partial receipt splits the line (new SERIAL_NO); taken by the next XD08 run (D3)</t>
+        </is>
+      </c>
+      <c r="G32" s="206" t="inlineStr">
+        <is>
+          <t>TB_R_H0253_ORDER_CONTROL_PRE (Surrounding DPV)</t>
+        </is>
+      </c>
+      <c r="H32" s="206" t="inlineStr">
+        <is>
+          <t>TB_R_H0253_ORDER_CONTROL_PRE (DB Surrounding, INTF_UPDATE_DT)</t>
+        </is>
+      </c>
+      <c r="I32" s="206" t="inlineStr">
+        <is>
+          <t>End</t>
+        </is>
+      </c>
+      <c r="J32" s="206" t="inlineStr">
+        <is>
+          <t>AB18</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="24" customHeight="1">
+      <c r="A33" s="214" t="inlineStr">
         <is>
           <t>H1</t>
         </is>
       </c>
-      <c r="B31" s="215" t="inlineStr">
+      <c r="B33" s="215" t="inlineStr">
         <is>
           <t>F4</t>
         </is>
       </c>
-      <c r="C31" s="215" t="inlineStr">
+      <c r="C33" s="215" t="inlineStr">
         <is>
           <t>Day D · working hours (hold)</t>
         </is>
       </c>
-      <c r="D31" s="206" t="inlineStr">
+      <c r="D33" s="206" t="inlineStr">
         <is>
           <t>D/S Team</t>
         </is>
       </c>
-      <c r="E31" s="206" t="inlineStr">
+      <c r="E33" s="206" t="inlineStr">
         <is>
           <t>XD10</t>
         </is>
       </c>
-      <c r="F31" s="206" t="inlineStr">
+      <c r="F33" s="206" t="inlineStr">
         <is>
           <t>Monitor the destination detail of the delivery plan (View as D/S team)</t>
         </is>
       </c>
-      <c r="G31" s="206" t="inlineStr">
+      <c r="G33" s="206" t="inlineStr">
         <is>
           <t>TB_R_H0253_ORDER_CONTROL_PRE</t>
         </is>
       </c>
-      <c r="H31" s="206" t="inlineStr">
+      <c r="H33" s="206" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I31" s="206" t="inlineStr">
+      <c r="I33" s="206" t="inlineStr">
         <is>
           <t>H2</t>
         </is>
       </c>
-      <c r="J31" s="206" t="inlineStr">
+      <c r="J33" s="206" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="24" customHeight="1">
-      <c r="A32" s="214" t="inlineStr">
+    <row r="34" ht="24" customHeight="1">
+      <c r="A34" s="214" t="inlineStr">
         <is>
           <t>H2</t>
         </is>
       </c>
-      <c r="B32" s="215" t="inlineStr">
+      <c r="B34" s="215" t="inlineStr">
         <is>
           <t>F4</t>
         </is>
       </c>
-      <c r="C32" s="215" t="inlineStr">
+      <c r="C34" s="215" t="inlineStr">
         <is>
           <t>Day D · working hours (hold)</t>
         </is>
       </c>
-      <c r="D32" s="206" t="inlineStr">
+      <c r="D34" s="206" t="inlineStr">
         <is>
           <t>D/S Team</t>
         </is>
       </c>
-      <c r="E32" s="206" t="inlineStr">
+      <c r="E34" s="206" t="inlineStr">
         <is>
           <t>XD10</t>
         </is>
       </c>
-      <c r="F32" s="206" t="inlineStr">
+      <c r="F34" s="206" t="inlineStr">
         <is>
           <t>Hold a destination (all its order lines): HOLD_FLAG = Y</t>
         </is>
       </c>
-      <c r="G32" s="206" t="inlineStr">
+      <c r="G34" s="206" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H32" s="206" t="inlineStr">
+      <c r="H34" s="206" t="inlineStr">
         <is>
           <t>TB_R_H0253_ORDER_CONTROL_PRE (HOLD_FLAG Y)</t>
         </is>
       </c>
-      <c r="I32" s="206" t="inlineStr">
+      <c r="I34" s="206" t="inlineStr">
         <is>
           <t>H3</t>
         </is>
       </c>
-      <c r="J32" s="206" t="inlineStr">
+      <c r="J34" s="206" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="36" customHeight="1">
-      <c r="A33" s="210" t="inlineStr">
+    <row r="35" ht="36" customHeight="1">
+      <c r="A35" s="210" t="inlineStr">
         <is>
           <t>H3</t>
         </is>
       </c>
-      <c r="B33" s="211" t="inlineStr">
+      <c r="B35" s="211" t="inlineStr">
         <is>
           <t>F4</t>
         </is>
       </c>
-      <c r="C33" s="211" t="inlineStr">
+      <c r="C35" s="211" t="inlineStr">
         <is>
           <t>Day D · working hours (hold)</t>
         </is>
       </c>
-      <c r="D33" s="206" t="inlineStr">
+      <c r="D35" s="206" t="inlineStr">
         <is>
           <t>NSP Batch (System)</t>
         </is>
       </c>
-      <c r="E33" s="206" t="inlineStr">
+      <c r="E35" s="206" t="inlineStr">
         <is>
           <t>XD09</t>
         </is>
       </c>
-      <c r="F33" s="206" t="inlineStr">
+      <c r="F35" s="206" t="inlineStr">
         <is>
           <t>[Search]: lines with HOLD_FLAG Y are excluded from pre-mapping; the unit calculation excludes the held destination(s)</t>
         </is>
       </c>
-      <c r="G33" s="206" t="inlineStr">
+      <c r="G35" s="206" t="inlineStr">
         <is>
           <t>TB_R_H0253_ORDER_CONTROL_PRE (HOLD N)</t>
         </is>
       </c>
-      <c r="H33" s="206" t="inlineStr">
+      <c r="H35" s="206" t="inlineStr">
         <is>
           <t>#TEMP_INSTRUCTION</t>
         </is>
       </c>
-      <c r="I33" s="206" t="inlineStr">
+      <c r="I35" s="206" t="inlineStr">
         <is>
           <t>H4</t>
         </is>
       </c>
-      <c r="J33" s="206" t="inlineStr">
+      <c r="J35" s="206" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="48" customHeight="1">
-      <c r="A34" s="218" t="inlineStr">
+    <row r="36" ht="48" customHeight="1">
+      <c r="A36" s="218" t="inlineStr">
         <is>
           <t>H4</t>
         </is>
       </c>
-      <c r="B34" s="219" t="inlineStr">
+      <c r="B36" s="219" t="inlineStr">
         <is>
           <t>F4</t>
         </is>
       </c>
-      <c r="C34" s="219" t="inlineStr">
+      <c r="C36" s="219" t="inlineStr">
         <is>
           <t>Day D · working hours (hold)</t>
         </is>
       </c>
-      <c r="D34" s="206" t="inlineStr">
+      <c r="D36" s="206" t="inlineStr">
         <is>
           <t>Supplier</t>
         </is>
       </c>
-      <c r="E34" s="206" t="inlineStr">
+      <c r="E36" s="206" t="inlineStr">
         <is>
           <t>XD10</t>
         </is>
       </c>
-      <c r="F34" s="206" t="inlineStr">
+      <c r="F36" s="206" t="inlineStr">
         <is>
           <t>[Create ASN] re-checks the hold: a line held after the tick → whole create fails, list refreshed</t>
         </is>
       </c>
-      <c r="G34" s="206" t="inlineStr">
+      <c r="G36" s="206" t="inlineStr">
         <is>
           <t>#TEMP_INSTRUCTION
 TB_R_H0253_ORDER_CONTROL_PRE</t>
         </is>
       </c>
-      <c r="H34" s="206" t="inlineStr">
+      <c r="H36" s="206" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I34" s="206" t="inlineStr">
+      <c r="I36" s="206" t="inlineStr">
         <is>
           <t>End</t>
         </is>
       </c>
-      <c r="J34" s="206" t="inlineStr">
+      <c r="J36" s="206" t="inlineStr">
         <is>
           <t>AB09</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="24" customHeight="1">
-      <c r="A35" s="214" t="inlineStr">
-        <is>
-          <t>H5</t>
-        </is>
-      </c>
-      <c r="B35" s="215" t="inlineStr">
-        <is>
-          <t>F4</t>
-        </is>
-      </c>
-      <c r="C35" s="215" t="inlineStr">
-        <is>
-          <t>Later · working hours (release)</t>
-        </is>
-      </c>
-      <c r="D35" s="206" t="inlineStr">
-        <is>
-          <t>D/S Team</t>
-        </is>
-      </c>
-      <c r="E35" s="206" t="inlineStr">
-        <is>
-          <t>XD10</t>
-        </is>
-      </c>
-      <c r="F35" s="206" t="inlineStr">
-        <is>
-          <t>Release the destination: HOLD_FLAG = N</t>
-        </is>
-      </c>
-      <c r="G35" s="206" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H35" s="206" t="inlineStr">
-        <is>
-          <t>TB_R_H0253_ORDER_CONTROL_PRE (HOLD_FLAG N)</t>
-        </is>
-      </c>
-      <c r="I35" s="206" t="inlineStr">
-        <is>
-          <t>H6</t>
-        </is>
-      </c>
-      <c r="J35" s="206" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="36" customHeight="1">
-      <c r="A36" s="210" t="inlineStr">
-        <is>
-          <t>H6</t>
-        </is>
-      </c>
-      <c r="B36" s="211" t="inlineStr">
-        <is>
-          <t>F4</t>
-        </is>
-      </c>
-      <c r="C36" s="211" t="inlineStr">
-        <is>
-          <t>Later · working hours (release)</t>
-        </is>
-      </c>
-      <c r="D36" s="206" t="inlineStr">
-        <is>
-          <t>NSP Batch (System)</t>
-        </is>
-      </c>
-      <c r="E36" s="206" t="inlineStr">
-        <is>
-          <t>XD09</t>
-        </is>
-      </c>
-      <c r="F36" s="206" t="inlineStr">
-        <is>
-          <t>Next [Search]: released lines are automatically included in pre-mapping and unit calculation (unit qty increases by their qty)</t>
-        </is>
-      </c>
-      <c r="G36" s="206" t="inlineStr">
-        <is>
-          <t>TB_R_H0253_ORDER_CONTROL_PRE (HOLD N)</t>
-        </is>
-      </c>
-      <c r="H36" s="206" t="inlineStr">
-        <is>
-          <t>#TEMP_INSTRUCTION</t>
-        </is>
-      </c>
-      <c r="I36" s="206" t="inlineStr">
-        <is>
-          <t>End</t>
-        </is>
-      </c>
-      <c r="J36" s="206" t="inlineStr">
-        <is>
-          <t>-</t>
         </is>
       </c>
     </row>
     <row r="37" ht="24" customHeight="1">
-      <c r="A37" s="208" t="inlineStr">
+      <c r="A37" s="214" t="inlineStr">
+        <is>
+          <t>H5</t>
+        </is>
+      </c>
+      <c r="B37" s="215" t="inlineStr">
+        <is>
+          <t>F4</t>
+        </is>
+      </c>
+      <c r="C37" s="215" t="inlineStr">
+        <is>
+          <t>Later · working hours (release)</t>
+        </is>
+      </c>
+      <c r="D37" s="206" t="inlineStr">
+        <is>
+          <t>D/S Team</t>
+        </is>
+      </c>
+      <c r="E37" s="206" t="inlineStr">
+        <is>
+          <t>XD10</t>
+        </is>
+      </c>
+      <c r="F37" s="206" t="inlineStr">
+        <is>
+          <t>Release the destination: HOLD_FLAG = N</t>
+        </is>
+      </c>
+      <c r="G37" s="206" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H37" s="206" t="inlineStr">
+        <is>
+          <t>TB_R_H0253_ORDER_CONTROL_PRE (HOLD_FLAG N)</t>
+        </is>
+      </c>
+      <c r="I37" s="206" t="inlineStr">
+        <is>
+          <t>H6</t>
+        </is>
+      </c>
+      <c r="J37" s="206" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="36" customHeight="1">
+      <c r="A38" s="210" t="inlineStr">
+        <is>
+          <t>H6</t>
+        </is>
+      </c>
+      <c r="B38" s="211" t="inlineStr">
+        <is>
+          <t>F4</t>
+        </is>
+      </c>
+      <c r="C38" s="211" t="inlineStr">
+        <is>
+          <t>Later · working hours (release)</t>
+        </is>
+      </c>
+      <c r="D38" s="206" t="inlineStr">
+        <is>
+          <t>NSP Batch (System)</t>
+        </is>
+      </c>
+      <c r="E38" s="206" t="inlineStr">
+        <is>
+          <t>XD09</t>
+        </is>
+      </c>
+      <c r="F38" s="206" t="inlineStr">
+        <is>
+          <t>Next [Search]: released lines are automatically included in pre-mapping and unit calculation (unit qty increases by their qty)</t>
+        </is>
+      </c>
+      <c r="G38" s="206" t="inlineStr">
+        <is>
+          <t>TB_R_H0253_ORDER_CONTROL_PRE (HOLD N)</t>
+        </is>
+      </c>
+      <c r="H38" s="206" t="inlineStr">
+        <is>
+          <t>#TEMP_INSTRUCTION</t>
+        </is>
+      </c>
+      <c r="I38" s="206" t="inlineStr">
+        <is>
+          <t>End</t>
+        </is>
+      </c>
+      <c r="J38" s="206" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="24" customHeight="1">
+      <c r="A39" s="208" t="inlineStr">
         <is>
           <t>C1</t>
         </is>
       </c>
-      <c r="B37" s="209" t="inlineStr">
+      <c r="B39" s="209" t="inlineStr">
         <is>
           <t>F4</t>
         </is>
       </c>
-      <c r="C37" s="209" t="inlineStr">
+      <c r="C39" s="209" t="inlineStr">
         <is>
           <t>Any time · GTOPAS (cancel)</t>
         </is>
       </c>
-      <c r="D37" s="206" t="inlineStr">
+      <c r="D39" s="206" t="inlineStr">
         <is>
           <t>GTOPAS / DB Surrounding</t>
         </is>
       </c>
-      <c r="E37" s="206" t="inlineStr">
+      <c r="E39" s="206" t="inlineStr">
         <is>
           <t>SOP</t>
         </is>
       </c>
-      <c r="F37" s="206" t="inlineStr">
+      <c r="F39" s="206" t="inlineStr">
         <is>
           <t>Check the ASN feedback: only qty not yet in an ASN may be cancelled</t>
         </is>
       </c>
-      <c r="G37" s="206" t="inlineStr">
+      <c r="G39" s="206" t="inlineStr">
         <is>
           <t>Existing ASN feedback</t>
         </is>
       </c>
-      <c r="H37" s="206" t="inlineStr">
+      <c r="H39" s="206" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I37" s="206" t="inlineStr">
+      <c r="I39" s="206" t="inlineStr">
         <is>
           <t>C2</t>
         </is>
       </c>
-      <c r="J37" s="206" t="inlineStr">
+      <c r="J39" s="206" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="24" customHeight="1">
-      <c r="A38" s="208" t="inlineStr">
+    <row r="40" ht="24" customHeight="1">
+      <c r="A40" s="208" t="inlineStr">
         <is>
           <t>C2</t>
         </is>
       </c>
-      <c r="B38" s="209" t="inlineStr">
+      <c r="B40" s="209" t="inlineStr">
         <is>
           <t>F4</t>
         </is>
       </c>
-      <c r="C38" s="209" t="inlineStr">
+      <c r="C40" s="209" t="inlineStr">
         <is>
           <t>Any time · GTOPAS (cancel)</t>
         </is>
       </c>
-      <c r="D38" s="206" t="inlineStr">
+      <c r="D40" s="206" t="inlineStr">
         <is>
           <t>GTOPAS / DB Surrounding</t>
         </is>
       </c>
-      <c r="E38" s="206" t="inlineStr">
+      <c r="E40" s="206" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F38" s="206" t="inlineStr">
+      <c r="F40" s="206" t="inlineStr">
         <is>
           <t>Cancel (with or without HOLD_FLAG): ORDER_STATUS 2; partial cancel = new SERIAL_NO</t>
         </is>
       </c>
-      <c r="G38" s="206" t="inlineStr">
+      <c r="G40" s="206" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H38" s="206" t="inlineStr">
+      <c r="H40" s="206" t="inlineStr">
         <is>
           <t>TB_R_H0253_ORDER_CONTROL_PRE (DB Surrounding, INTF_UPDATE_DT)</t>
         </is>
       </c>
-      <c r="I38" s="206" t="inlineStr">
+      <c r="I40" s="206" t="inlineStr">
         <is>
           <t>C3</t>
         </is>
       </c>
-      <c r="J38" s="206" t="inlineStr">
+      <c r="J40" s="206" t="inlineStr">
         <is>
           <t>AB16</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="48" customHeight="1">
-      <c r="A39" s="210" t="inlineStr">
+    <row r="41" ht="48" customHeight="1">
+      <c r="A41" s="210" t="inlineStr">
         <is>
           <t>C3</t>
         </is>
       </c>
-      <c r="B39" s="211" t="inlineStr">
+      <c r="B41" s="211" t="inlineStr">
         <is>
           <t>F4</t>
         </is>
       </c>
-      <c r="C39" s="211" t="inlineStr">
+      <c r="C41" s="211" t="inlineStr">
         <is>
           <t>27:30 · XD08 (one H0253 batch)</t>
         </is>
       </c>
-      <c r="D39" s="206" t="inlineStr">
+      <c r="D41" s="206" t="inlineStr">
         <is>
           <t>NSP Batch (System)</t>
         </is>
       </c>
-      <c r="E39" s="206" t="inlineStr">
+      <c r="E41" s="206" t="inlineStr">
         <is>
           <t>XD08</t>
         </is>
       </c>
-      <c r="F39" s="206" t="inlineStr">
+      <c r="F41" s="206" t="inlineStr">
         <is>
           <t>Upsert the changed rows: UPD_STATUS 2 (cancel) / 6 (received); ORDER_STATUS keeps the first value</t>
         </is>
       </c>
-      <c r="G39" s="206" t="inlineStr">
+      <c r="G41" s="206" t="inlineStr">
         <is>
           <t>TB_R_H0253_ORDER_CONTROL_PRE (DB Surrounding)</t>
         </is>
       </c>
-      <c r="H39" s="206" t="inlineStr">
+      <c r="H41" s="206" t="inlineStr">
         <is>
           <t>TB_R_H0253_ORDER_CONTROL_PRE (NSP, UPD_STATUS)
 Log</t>
         </is>
       </c>
-      <c r="I39" s="206" t="inlineStr">
+      <c r="I41" s="206" t="inlineStr">
         <is>
           <t>C4</t>
         </is>
       </c>
-      <c r="J39" s="206" t="inlineStr">
+      <c r="J41" s="206" t="inlineStr">
         <is>
           <t>AB07</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="60" customHeight="1">
-      <c r="A40" s="210" t="inlineStr">
+    <row r="42" ht="60" customHeight="1">
+      <c r="A42" s="210" t="inlineStr">
         <is>
           <t>C4</t>
         </is>
       </c>
-      <c r="B40" s="211" t="inlineStr">
+      <c r="B42" s="211" t="inlineStr">
         <is>
           <t>F4</t>
         </is>
       </c>
-      <c r="C40" s="211" t="inlineStr">
+      <c r="C42" s="211" t="inlineStr">
         <is>
           <t>27:30 · XD08 (one H0253 batch)</t>
         </is>
       </c>
-      <c r="D40" s="206" t="inlineStr">
+      <c r="D42" s="206" t="inlineStr">
         <is>
           <t>NSP Batch (System)</t>
         </is>
       </c>
-      <c r="E40" s="206" t="inlineStr">
+      <c r="E42" s="206" t="inlineStr">
         <is>
           <t>XD08</t>
         </is>
       </c>
-      <c r="F40" s="206" t="inlineStr">
+      <c r="F42" s="206" t="inlineStr">
         <is>
           <t>Release all drafts (Create ASN not submitted); the cases come back in the delivery plan</t>
         </is>
       </c>
-      <c r="G40" s="206" t="inlineStr">
+      <c r="G42" s="206" t="inlineStr">
         <is>
           <t>TB_R_INSTRUCTION (ASN_NO NULL)</t>
         </is>
       </c>
-      <c r="H40" s="206" t="inlineStr">
+      <c r="H42" s="206" t="inlineStr">
         <is>
           <t>TB_R_INSTRUCTION (delete drafts)
 TB_R_PRA_DAILY_ORDER_MAPPED (MAPPED_QTY −)
 TB_R_H0253_ORDER_CONTROL_PRE (PO_MAPPED_FLAG N)</t>
         </is>
       </c>
-      <c r="I40" s="206" t="inlineStr">
+      <c r="I42" s="206" t="inlineStr">
         <is>
           <t>C5, C6</t>
         </is>
       </c>
-      <c r="J40" s="206" t="inlineStr">
+      <c r="J42" s="206" t="inlineStr">
         <is>
           <t>AB12</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="36" customHeight="1">
-      <c r="A41" s="210" t="inlineStr">
+    <row r="43" ht="36" customHeight="1">
+      <c r="A43" s="210" t="inlineStr">
         <is>
           <t>C5</t>
         </is>
       </c>
-      <c r="B41" s="211" t="inlineStr">
+      <c r="B43" s="211" t="inlineStr">
         <is>
           <t>F4</t>
         </is>
       </c>
-      <c r="C41" s="211" t="inlineStr">
+      <c r="C43" s="211" t="inlineStr">
         <is>
           <t>27:30 · XD08 (one H0253 batch)</t>
         </is>
       </c>
-      <c r="D41" s="206" t="inlineStr">
+      <c r="D43" s="206" t="inlineStr">
         <is>
           <t>NSP Batch (System)</t>
         </is>
       </c>
-      <c r="E41" s="206" t="inlineStr">
+      <c r="E43" s="206" t="inlineStr">
         <is>
           <t>XD08</t>
         </is>
       </c>
-      <c r="F41" s="206" t="inlineStr">
+      <c r="F43" s="206" t="inlineStr">
         <is>
           <t>Cancel of qty in a submitted ASN: LOG5, listed in Change Order Number (ASN not changed)</t>
         </is>
       </c>
-      <c r="G41" s="206" t="inlineStr">
+      <c r="G43" s="206" t="inlineStr">
         <is>
           <t>TB_R_H0253_ORDER_CONTROL_PRE (UPD_STATUS 2)
 TB_R_INSTRUCTION (ASN_NO)</t>
         </is>
       </c>
-      <c r="H41" s="206" t="inlineStr">
+      <c r="H43" s="206" t="inlineStr">
         <is>
           <t>Log</t>
         </is>
       </c>
-      <c r="I41" s="206" t="inlineStr">
+      <c r="I43" s="206" t="inlineStr">
         <is>
           <t>C7</t>
         </is>
       </c>
-      <c r="J41" s="206" t="inlineStr">
+      <c r="J43" s="206" t="inlineStr">
         <is>
           <t>AB16</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="24" customHeight="1">
-      <c r="A42" s="218" t="inlineStr">
+    <row r="44" ht="24" customHeight="1">
+      <c r="A44" s="218" t="inlineStr">
         <is>
           <t>C6</t>
         </is>
       </c>
-      <c r="B42" s="219" t="inlineStr">
+      <c r="B44" s="219" t="inlineStr">
         <is>
           <t>F4</t>
         </is>
       </c>
-      <c r="C42" s="219" t="inlineStr">
+      <c r="C44" s="219" t="inlineStr">
         <is>
           <t>Day D · working hours</t>
         </is>
       </c>
-      <c r="D42" s="206" t="inlineStr">
+      <c r="D44" s="206" t="inlineStr">
         <is>
           <t>Supplier</t>
         </is>
       </c>
-      <c r="E42" s="206" t="inlineStr">
+      <c r="E44" s="206" t="inlineStr">
         <is>
           <t>XD10</t>
         </is>
       </c>
-      <c r="F42" s="206" t="inlineStr">
+      <c r="F44" s="206" t="inlineStr">
         <is>
           <t>[Search] again and tick the cases again; [Submit ASN] of an old draft fails (MSG11)</t>
         </is>
       </c>
-      <c r="G42" s="206" t="inlineStr">
+      <c r="G44" s="206" t="inlineStr">
         <is>
           <t>#TEMP_INSTRUCTION</t>
         </is>
       </c>
-      <c r="H42" s="206" t="inlineStr">
+      <c r="H44" s="206" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I42" s="206" t="inlineStr">
+      <c r="I44" s="206" t="inlineStr">
         <is>
           <t>End</t>
         </is>
       </c>
-      <c r="J42" s="206" t="inlineStr">
+      <c r="J44" s="206" t="inlineStr">
         <is>
           <t>AB12</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="48" customHeight="1">
-      <c r="A43" s="214" t="inlineStr">
+    <row r="45" ht="48" customHeight="1">
+      <c r="A45" s="214" t="inlineStr">
         <is>
           <t>C7</t>
         </is>
       </c>
-      <c r="B43" s="215" t="inlineStr">
+      <c r="B45" s="215" t="inlineStr">
         <is>
           <t>F4</t>
         </is>
       </c>
-      <c r="C43" s="215" t="inlineStr">
+      <c r="C45" s="215" t="inlineStr">
         <is>
           <t>Day D · working hours</t>
         </is>
       </c>
-      <c r="D43" s="206" t="inlineStr">
+      <c r="D45" s="206" t="inlineStr">
         <is>
           <t>D/S Team</t>
         </is>
       </c>
-      <c r="E43" s="206" t="inlineStr">
+      <c r="E45" s="206" t="inlineStr">
         <is>
           <t>XD11</t>
         </is>
       </c>
-      <c r="F43" s="206" t="inlineStr">
+      <c r="F45" s="206" t="inlineStr">
         <is>
           <t>Change Order Number: cancelled qty and candidates (same part, UPD_STATUS 6, PO_MAPPED N, no ASN, oldest first)</t>
         </is>
       </c>
-      <c r="G43" s="206" t="inlineStr">
+      <c r="G45" s="206" t="inlineStr">
         <is>
           <t>TB_R_H0253_ORDER_CONTROL_PRE
 TB_R_INSTRUCTION</t>
         </is>
       </c>
-      <c r="H43" s="206" t="inlineStr">
+      <c r="H45" s="206" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I43" s="206" t="inlineStr">
+      <c r="I45" s="206" t="inlineStr">
         <is>
           <t>C8</t>
         </is>
       </c>
-      <c r="J43" s="206" t="inlineStr">
+      <c r="J45" s="206" t="inlineStr">
         <is>
           <t>AB16</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="60" customHeight="1">
-      <c r="A44" s="214" t="inlineStr">
+    <row r="46" ht="60" customHeight="1">
+      <c r="A46" s="214" t="inlineStr">
         <is>
           <t>C8</t>
         </is>
       </c>
-      <c r="B44" s="215" t="inlineStr">
+      <c r="B46" s="215" t="inlineStr">
         <is>
           <t>F4</t>
         </is>
       </c>
-      <c r="C44" s="215" t="inlineStr">
+      <c r="C46" s="215" t="inlineStr">
         <is>
           <t>Day D · working hours</t>
         </is>
       </c>
-      <c r="D44" s="206" t="inlineStr">
+      <c r="D46" s="206" t="inlineStr">
         <is>
           <t>D/S Team</t>
         </is>
       </c>
-      <c r="E44" s="206" t="inlineStr">
+      <c r="E46" s="206" t="inlineStr">
         <is>
           <t>XD11</t>
         </is>
       </c>
-      <c r="F44" s="206" t="inlineStr">
+      <c r="F46" s="206" t="inlineStr">
         <is>
           <t>Move the qty from the last case (row split when needed) to one or more lines; history</t>
         </is>
       </c>
-      <c r="G44" s="206" t="inlineStr">
+      <c r="G46" s="206" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H44" s="206" t="inlineStr">
+      <c r="H46" s="206" t="inlineStr">
         <is>
           <t>TB_R_INSTRUCTION (order key / split)
 TB_R_H0253_ORDER_CONTROL_PRE (PO_MAPPED_FLAG Y)
 TB_H_CROSSDOCK_ORDER_CHANGE</t>
         </is>
       </c>
-      <c r="I44" s="206" t="inlineStr">
+      <c r="I46" s="206" t="inlineStr">
         <is>
           <t>End</t>
         </is>
       </c>
-      <c r="J44" s="206" t="inlineStr">
+      <c r="J46" s="206" t="inlineStr">
         <is>
           <t>AB15</t>
         </is>
@@ -27688,7 +28133,7 @@
       </c>
       <c r="I18" s="231" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D10</t>
         </is>
       </c>
     </row>
@@ -28213,7 +28658,7 @@
       </c>
       <c r="C12" s="206" t="inlineStr">
         <is>
-          <t>D6 / D7</t>
+          <t>D6</t>
         </is>
       </c>
       <c r="D12" s="206" t="inlineStr">
@@ -28255,12 +28700,12 @@
       </c>
       <c r="B13" s="206" t="inlineStr">
         <is>
-          <t>F4</t>
+          <t>F2 / F4</t>
         </is>
       </c>
       <c r="C13" s="206" t="inlineStr">
         <is>
-          <t>H4</t>
+          <t>D7 / H4</t>
         </is>
       </c>
       <c r="D13" s="206" t="inlineStr">
@@ -28589,7 +29034,7 @@
       </c>
       <c r="C20" s="206" t="inlineStr">
         <is>
-          <t>D2 / D6</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D20" s="206" t="inlineStr">
@@ -28636,7 +29081,7 @@
       </c>
       <c r="C21" s="206" t="inlineStr">
         <is>
-          <t>D14 / D3</t>
+          <t>D15 / D3</t>
         </is>
       </c>
       <c r="D21" s="206" t="inlineStr">

</xml_diff>

<commit_message>
FB-100 / FB-101: BPF, Confirmation page and re-send wording follow the RPA / delete concept
- BPF: M11 'GTOPAS by RPA, AP POLE file by SFTP (Inactive: delete)' (also in the hand-edited F1
  shape), M12 / M13 texts and abnormality AB06 (RPA bot failure) updated; prototype data rebuilt.
- Confirmation page: A7, A8, A10, A11 show the decisions of 30-Oct.
- XD01 5.16 c. and XD07 4.3: 'replace is repeatable' replaced by the current behaviour
  (GTOPAS gets the differences, AP POLE the complete set) - apply_3110.py.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QL8Do8Pd2rXEDNa1ifG2RK
</commit_message>
<xml_diff>
--- a/deliverables/function_list_v2/bpf/Crossdock_BPF_Level2.xlsx
+++ b/deliverables/function_list_v2/bpf/Crossdock_BPF_Level2.xlsx
@@ -4422,7 +4422,7 @@
               <a:latin typeface="Arial"/>
               <a:cs typeface="Arial"/>
             </a:rPr>
-            <a:t>Send crossdock master (CROSSDOCK_FLAG Y / N): GTOPAS existing IF, AP POLE file by SFTP</a:t>
+            <a:t>Send crossdock master: GTOPAS by RPA, AP POLE file by SFTP (Inactive: delete)</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -25841,7 +25841,7 @@
       </c>
       <c r="F15" s="206" t="inlineStr">
         <is>
-          <t>Send crossdock master (CROSSDOCK_FLAG Y / N): GTOPAS existing IF, AP POLE file by SFTP</t>
+          <t>Send crossdock master: GTOPAS by RPA, AP POLE file by SFTP (Inactive: delete)</t>
         </is>
       </c>
       <c r="G15" s="206" t="inlineStr">
@@ -25869,7 +25869,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="24" customHeight="1">
+    <row r="16" ht="36" customHeight="1">
       <c r="A16" s="208" t="inlineStr">
         <is>
           <t>M12</t>
@@ -25897,17 +25897,17 @@
       </c>
       <c r="F16" s="206" t="inlineStr">
         <is>
-          <t>Modify part number and destination in Crossdock Master (Supply Menu)</t>
+          <t>RPA: register / delete part + destination in Crossdock Master (Supply &gt; Master); Inactive: delete all rows</t>
         </is>
       </c>
       <c r="G16" s="206" t="inlineStr">
         <is>
-          <t>Interface data from NSP</t>
+          <t>RPA input from NSP</t>
         </is>
       </c>
       <c r="H16" s="206" t="inlineStr">
         <is>
-          <t>GTOPAS master (not detailed)</t>
+          <t>GTOPAS Crossdock Master</t>
         </is>
       </c>
       <c r="I16" s="206" t="inlineStr">
@@ -25921,7 +25921,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="24" customHeight="1">
+    <row r="17" ht="36" customHeight="1">
       <c r="A17" s="216" t="inlineStr">
         <is>
           <t>M13</t>
@@ -25949,7 +25949,7 @@
       </c>
       <c r="F17" s="206" t="inlineStr">
         <is>
-          <t>TMMIN SFTP → TMA SFTP → receive IF by TMA AP POLE Crossdock Kanban Part Master</t>
+          <t>TMMIN SFTP → TMA SFTP → receive IF by TMA AP POLE Crossdock Kanban Part Master (Inactive: delete part)</t>
         </is>
       </c>
       <c r="G17" s="206" t="inlineStr">
@@ -28551,7 +28551,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="24" customHeight="1">
+    <row r="10" ht="36" customHeight="1">
       <c r="A10" s="205" t="inlineStr">
         <is>
           <t>AB06</t>
@@ -28574,7 +28574,7 @@
       </c>
       <c r="E10" s="206" t="inlineStr">
         <is>
-          <t>Interface file cannot be created, or GTOPAS / AP POLE SFTP not available after retry</t>
+          <t>Interface file / RPA input cannot be created, GTOPAS RPA bot fails, or AP POLE SFTP not available after retry</t>
         </is>
       </c>
       <c r="F10" s="206" t="inlineStr">
@@ -28584,7 +28584,7 @@
       </c>
       <c r="G10" s="206" t="inlineStr">
         <is>
-          <t>Keep the file in the outbound folder; parts stay Failed.</t>
+          <t>Keep the file (outbound folder / RPA input); parts stay Failed.</t>
         </is>
       </c>
       <c r="H10" s="206" t="inlineStr">

</xml_diff>